<commit_message>
Replace SuDS rill with swales/attenuation assumption (7% of site)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014iit8YdqqexD3WDZo9gb62
</commit_message>
<xml_diff>
--- a/model/ZON_Wivenhoe_Appraisal.xlsx
+++ b/model/ZON_Wivenhoe_Appraisal.xlsx
@@ -335,10 +335,10 @@
     <t xml:space="preserve">Припущення: петля Manual for Streets + гостьові місця</t>
   </si>
   <si>
-    <t xml:space="preserve">SuDS-струмок, ставок, відкритий простір</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Припущення; уточнює інженер з дренажу</t>
+    <t xml:space="preserve">SuDS (свейли, атенюація) та відкритий простір</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Без струмка. Припущення; уточнює інженер з дренажу після тестів інфільтрації</t>
   </si>
   <si>
     <t xml:space="preserve">BNG / ландшафтні буфери на ділянці</t>
@@ -1378,15 +1378,15 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">'Сценарій A'!$B$25</f>
-        <v>-908.300000000001</v>
+        <v>-480.950000000001</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">'Сценарій B'!$B$25</f>
-        <v>-1778.3</v>
+        <v>-1350.95</v>
       </c>
       <c r="D6" s="7" t="n">
         <f aca="false">C6-B6</f>
-        <v>-869.999999999998</v>
+        <v>-870</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -2821,7 +2821,7 @@
         <v>103</v>
       </c>
       <c r="B14" s="27" t="n">
-        <v>0.1</v>
+        <v>0.07</v>
       </c>
       <c r="C14" s="5" t="s">
         <v>101</v>
@@ -3832,7 +3832,7 @@
       </c>
       <c r="B20" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$14</f>
-        <v>1424.5</v>
+        <v>997.15</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -3871,7 +3871,7 @@
       </c>
       <c r="B23" s="33" t="n">
         <f aca="false">SUM($B$18:$B$22)</f>
-        <v>15153.3</v>
+        <v>14725.95</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -3897,7 +3897,7 @@
       </c>
       <c r="B25" s="33" t="n">
         <f aca="false">$B$24-$B$23</f>
-        <v>-908.300000000001</v>
+        <v>-480.950000000001</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -4723,7 +4723,7 @@
       </c>
       <c r="B20" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$14</f>
-        <v>1424.5</v>
+        <v>997.15</v>
       </c>
       <c r="C20" s="2"/>
       <c r="D20" s="2"/>
@@ -4762,7 +4762,7 @@
       </c>
       <c r="B23" s="33" t="n">
         <f aca="false">SUM($B$18:$B$22)</f>
-        <v>16023.3</v>
+        <v>15595.95</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -4788,7 +4788,7 @@
       </c>
       <c r="B25" s="33" t="n">
         <f aca="false">$B$24-$B$23</f>
-        <v>-1778.3</v>
+        <v>-1350.95</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>

</xml_diff>

<commit_message>
Add selector for which unit type is delivered as affordable housing
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014iit8YdqqexD3WDZo9gb62
</commit_message>
<xml_diff>
--- a/model/ZON_Wivenhoe_Appraisal.xlsx
+++ b/model/ZON_Wivenhoe_Appraisal.xlsx
@@ -24,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="336" uniqueCount="234">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="237">
   <si>
     <t xml:space="preserve">ZON Wivenhoe — порівняння сценаріїв</t>
   </si>
@@ -374,6 +374,15 @@
     <t xml:space="preserve">Припущення: мікс affordable rent + shared ownership</t>
   </si>
   <si>
+    <t xml:space="preserve">Який тип іде як доступне житло</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1/2/3</t>
+  </si>
+  <si>
+    <t xml:space="preserve">1 = Compact 61, 2 = Meadow 71, 3 = Country 140</t>
+  </si>
+  <si>
     <t xml:space="preserve">Вартість будівництва</t>
   </si>
   <si>
@@ -632,7 +641,7 @@
     <t xml:space="preserve">округлення вгору від усіх житлових юнітів</t>
   </si>
   <si>
-    <t xml:space="preserve">…з них покривається Meadow 71</t>
+    <t xml:space="preserve">…з них покривається обраним типом</t>
   </si>
   <si>
     <t xml:space="preserve">Перевірка покриття</t>
@@ -641,7 +650,7 @@
     <t xml:space="preserve">Знижка на доступне житло</t>
   </si>
   <si>
-    <t xml:space="preserve">усі доступні юніти рахуються за ціною Meadow</t>
+    <t xml:space="preserve">усі доступні юніти — за ціною обраного типу</t>
   </si>
   <si>
     <t xml:space="preserve">ZON Hub: кав'ярня (капіталізація)</t>
@@ -1664,23 +1673,23 @@
         <v>-0.1</v>
       </c>
       <c r="B23" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
         <v>-1191197.8125</v>
       </c>
       <c r="C23" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
         <v>-1535973.5625</v>
       </c>
       <c r="D23" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
         <v>-1880749.3125</v>
       </c>
       <c r="E23" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
         <v>-2225525.0625</v>
       </c>
       <c r="F23" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
         <v>-2570300.8125</v>
       </c>
     </row>
@@ -1689,23 +1698,23 @@
         <v>-0.05</v>
       </c>
       <c r="B24" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
         <v>-744494.25</v>
       </c>
       <c r="C24" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
         <v>-1089270</v>
       </c>
       <c r="D24" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
         <v>-1434045.75</v>
       </c>
       <c r="E24" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
         <v>-1778821.5</v>
       </c>
       <c r="F24" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
         <v>-2123597.25</v>
       </c>
     </row>
@@ -1714,23 +1723,23 @@
         <v>0</v>
       </c>
       <c r="B25" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
         <v>-297790.6875</v>
       </c>
       <c r="C25" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
         <v>-642566.4375</v>
       </c>
       <c r="D25" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
         <v>-987342.1875</v>
       </c>
       <c r="E25" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
         <v>-1332117.9375</v>
       </c>
       <c r="F25" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
         <v>-1676893.6875</v>
       </c>
     </row>
@@ -1739,23 +1748,23 @@
         <v>0.05</v>
       </c>
       <c r="B26" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
         <v>148912.875</v>
       </c>
       <c r="C26" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
         <v>-195862.875</v>
       </c>
       <c r="D26" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
         <v>-540638.625</v>
       </c>
       <c r="E26" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
         <v>-885414.375</v>
       </c>
       <c r="F26" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
         <v>-1230190.125</v>
       </c>
     </row>
@@ -1764,23 +1773,23 @@
         <v>0.1</v>
       </c>
       <c r="B27" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
         <v>595616.4375</v>
       </c>
       <c r="C27" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
         <v>250840.6875</v>
       </c>
       <c r="D27" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
         <v>-93935.0625</v>
       </c>
       <c r="E27" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
         <v>-438710.8125</v>
       </c>
       <c r="F27" s="10" t="n">
-        <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$33)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
+        <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
         <v>-783486.562500001</v>
       </c>
     </row>
@@ -1835,23 +1844,23 @@
         <v>-0.1</v>
       </c>
       <c r="B32" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
         <v>-1817134.465</v>
       </c>
       <c r="C32" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
         <v>-2229833.815</v>
       </c>
       <c r="D32" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
         <v>-2642533.165</v>
       </c>
       <c r="E32" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
         <v>-3055232.515</v>
       </c>
       <c r="F32" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
         <v>-3467931.865</v>
       </c>
     </row>
@@ -1860,23 +1869,23 @@
         <v>-0.05</v>
       </c>
       <c r="B33" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
         <v>-1318370.29</v>
       </c>
       <c r="C33" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
         <v>-1731069.64</v>
       </c>
       <c r="D33" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
         <v>-2143768.99</v>
       </c>
       <c r="E33" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
         <v>-2556468.34</v>
       </c>
       <c r="F33" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
         <v>-2969167.69</v>
       </c>
     </row>
@@ -1885,23 +1894,23 @@
         <v>0</v>
       </c>
       <c r="B34" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
         <v>-819606.114999999</v>
       </c>
       <c r="C34" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
         <v>-1232305.465</v>
       </c>
       <c r="D34" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
         <v>-1645004.815</v>
       </c>
       <c r="E34" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
         <v>-2057704.165</v>
       </c>
       <c r="F34" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
         <v>-2470403.515</v>
       </c>
     </row>
@@ -1910,23 +1919,23 @@
         <v>0.05</v>
       </c>
       <c r="B35" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
         <v>-320841.94</v>
       </c>
       <c r="C35" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
         <v>-733541.29</v>
       </c>
       <c r="D35" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
         <v>-1146240.64</v>
       </c>
       <c r="E35" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
         <v>-1558939.99</v>
       </c>
       <c r="F35" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
         <v>-1971639.34</v>
       </c>
     </row>
@@ -1935,23 +1944,23 @@
         <v>0.1</v>
       </c>
       <c r="B36" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
         <v>177922.235</v>
       </c>
       <c r="C36" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
         <v>-234777.114999999</v>
       </c>
       <c r="D36" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
         <v>-647476.465</v>
       </c>
       <c r="E36" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
         <v>-1060175.815</v>
       </c>
       <c r="F36" s="10" t="n">
-        <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$33)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
+        <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
         <v>-1472875.165</v>
       </c>
     </row>
@@ -2111,7 +2120,7 @@
         <v>37</v>
       </c>
       <c r="B14" s="13" t="n">
-        <f aca="false">$B$13*(1-Припущення!$B$33)-$B$12</f>
+        <f aca="false">$B$13*(1-Припущення!$B$34)-$B$12</f>
         <v>-6964.28571428574</v>
       </c>
       <c r="C14" s="24" t="s">
@@ -2209,7 +2218,7 @@
         <v>49</v>
       </c>
       <c r="B23" s="13" t="n">
-        <f aca="false">$B$21*($B$19*(1-Припущення!$B$33)-$B$20)</f>
+        <f aca="false">$B$21*($B$19*(1-Припущення!$B$34)-$B$20)</f>
         <v>141250</v>
       </c>
       <c r="C23" s="2"/>
@@ -2283,7 +2292,7 @@
         <v>57</v>
       </c>
       <c r="B31" s="13" t="n">
-        <f aca="false">$B$30*(1+Припущення!$B$41)*(1+Припущення!$B$35*(Припущення!$B$37+'Сценарій A'!$B$13)/12)</f>
+        <f aca="false">$B$30*(1+Припущення!$B$42)*(1+Припущення!$B$36*(Припущення!$B$38+'Сценарій A'!$B$13)/12)</f>
         <v>175112</v>
       </c>
       <c r="C31" s="2"/>
@@ -2494,7 +2503,7 @@
         <v>75</v>
       </c>
       <c r="B52" s="13" t="n">
-        <f aca="false">MAX(0,Припущення!$B$42*$B$50-$B$49)</f>
+        <f aca="false">MAX(0,Припущення!$B$43*$B$50-$B$49)</f>
         <v>2326055.61428572</v>
       </c>
       <c r="C52" s="2"/>
@@ -2519,7 +2528,7 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:K50"/>
+  <dimension ref="A1:K51"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
     <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="42"/>
@@ -2950,10 +2959,18 @@
       <c r="K20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="2"/>
-      <c r="B21" s="2"/>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
+      <c r="A21" s="5" t="s">
+        <v>116</v>
+      </c>
+      <c r="B21" s="28" t="n">
+        <v>2</v>
+      </c>
+      <c r="C21" s="5" t="s">
+        <v>117</v>
+      </c>
+      <c r="D21" s="5" t="s">
+        <v>118</v>
+      </c>
       <c r="E21" s="2"/>
       <c r="F21" s="2"/>
       <c r="G21" s="2"/>
@@ -2963,12 +2980,10 @@
       <c r="K21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="21" t="s">
-        <v>116</v>
-      </c>
-      <c r="B22" s="22"/>
-      <c r="C22" s="22"/>
-      <c r="D22" s="22"/>
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
       <c r="G22" s="2"/>
@@ -2978,18 +2993,12 @@
       <c r="K22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="5" t="s">
-        <v>117</v>
-      </c>
-      <c r="B23" s="23" t="n">
-        <v>2400</v>
-      </c>
-      <c r="C23" s="5" t="s">
-        <v>118</v>
-      </c>
-      <c r="D23" s="5" t="s">
+      <c r="A23" s="21" t="s">
         <v>119</v>
       </c>
+      <c r="B23" s="22"/>
+      <c r="C23" s="22"/>
+      <c r="D23" s="22"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
       <c r="G23" s="2"/>
@@ -3002,14 +3011,14 @@
       <c r="A24" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B24" s="26" t="n">
-        <v>3000</v>
+      <c r="B24" s="23" t="n">
+        <v>2400</v>
       </c>
       <c r="C24" s="5" t="s">
-        <v>118</v>
+        <v>121</v>
       </c>
       <c r="D24" s="5" t="s">
-        <v>121</v>
+        <v>122</v>
       </c>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
@@ -3021,13 +3030,13 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="5" t="s">
-        <v>122</v>
-      </c>
-      <c r="B25" s="27" t="n">
-        <v>0.15</v>
+        <v>123</v>
+      </c>
+      <c r="B25" s="26" t="n">
+        <v>3000</v>
       </c>
       <c r="C25" s="5" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="D25" s="5" t="s">
         <v>124</v>
@@ -3045,7 +3054,7 @@
         <v>125</v>
       </c>
       <c r="B26" s="27" t="n">
-        <v>0.05</v>
+        <v>0.15</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>126</v>
@@ -3066,13 +3075,13 @@
         <v>128</v>
       </c>
       <c r="B27" s="27" t="n">
-        <v>0.1</v>
+        <v>0.05</v>
       </c>
       <c r="C27" s="5" t="s">
-        <v>126</v>
+        <v>129</v>
       </c>
       <c r="D27" s="5" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E27" s="2"/>
       <c r="F27" s="2"/>
@@ -3084,16 +3093,16 @@
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A28" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B28" s="27" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="C28" s="5" t="s">
         <v>129</v>
       </c>
-      <c r="B28" s="26" t="n">
-        <v>15000</v>
-      </c>
-      <c r="C28" s="5" t="s">
+      <c r="D28" s="5" t="s">
         <v>130</v>
-      </c>
-      <c r="D28" s="5" t="s">
-        <v>131</v>
       </c>
       <c r="E28" s="2"/>
       <c r="F28" s="2"/>
@@ -3108,13 +3117,13 @@
         <v>132</v>
       </c>
       <c r="B29" s="26" t="n">
-        <v>160</v>
+        <v>15000</v>
       </c>
       <c r="C29" s="5" t="s">
-        <v>130</v>
+        <v>133</v>
       </c>
       <c r="D29" s="5" t="s">
-        <v>133</v>
+        <v>134</v>
       </c>
       <c r="E29" s="2"/>
       <c r="F29" s="2"/>
@@ -3126,16 +3135,16 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>134</v>
+        <v>135</v>
       </c>
       <c r="B30" s="26" t="n">
-        <v>50000</v>
+        <v>160</v>
       </c>
       <c r="C30" s="5" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D30" s="5" t="s">
-        <v>127</v>
+        <v>136</v>
       </c>
       <c r="E30" s="2"/>
       <c r="F30" s="2"/>
@@ -3146,10 +3155,18 @@
       <c r="K30" s="2"/>
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="2"/>
-      <c r="B31" s="2"/>
-      <c r="C31" s="2"/>
-      <c r="D31" s="2"/>
+      <c r="A31" s="5" t="s">
+        <v>137</v>
+      </c>
+      <c r="B31" s="26" t="n">
+        <v>50000</v>
+      </c>
+      <c r="C31" s="5" t="s">
+        <v>138</v>
+      </c>
+      <c r="D31" s="5" t="s">
+        <v>130</v>
+      </c>
       <c r="E31" s="2"/>
       <c r="F31" s="2"/>
       <c r="G31" s="2"/>
@@ -3159,12 +3176,10 @@
       <c r="K31" s="2"/>
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="21" t="s">
-        <v>136</v>
-      </c>
-      <c r="B32" s="22"/>
-      <c r="C32" s="22"/>
-      <c r="D32" s="22"/>
+      <c r="A32" s="2"/>
+      <c r="B32" s="2"/>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
       <c r="E32" s="2"/>
       <c r="F32" s="2"/>
       <c r="G32" s="2"/>
@@ -3174,18 +3189,12 @@
       <c r="K32" s="2"/>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>137</v>
-      </c>
-      <c r="B33" s="27" t="n">
-        <v>0.025</v>
-      </c>
-      <c r="C33" s="5" t="s">
-        <v>138</v>
-      </c>
-      <c r="D33" s="5" t="s">
-        <v>127</v>
-      </c>
+      <c r="A33" s="21" t="s">
+        <v>139</v>
+      </c>
+      <c r="B33" s="22"/>
+      <c r="C33" s="22"/>
+      <c r="D33" s="22"/>
       <c r="E33" s="2"/>
       <c r="F33" s="2"/>
       <c r="G33" s="2"/>
@@ -3196,16 +3205,16 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>139</v>
-      </c>
-      <c r="B34" s="26" t="n">
-        <v>1500</v>
+        <v>140</v>
+      </c>
+      <c r="B34" s="27" t="n">
+        <v>0.025</v>
       </c>
       <c r="C34" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D34" s="5" t="s">
         <v>130</v>
-      </c>
-      <c r="D34" s="5" t="s">
-        <v>127</v>
       </c>
       <c r="E34" s="2"/>
       <c r="F34" s="2"/>
@@ -3217,16 +3226,16 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B35" s="27" t="n">
-        <v>0.09</v>
+        <v>142</v>
+      </c>
+      <c r="B35" s="26" t="n">
+        <v>1500</v>
       </c>
       <c r="C35" s="5" t="s">
-        <v>141</v>
+        <v>133</v>
       </c>
       <c r="D35" s="5" t="s">
-        <v>127</v>
+        <v>130</v>
       </c>
       <c r="E35" s="2"/>
       <c r="F35" s="2"/>
@@ -3238,16 +3247,16 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>142</v>
+        <v>143</v>
       </c>
       <c r="B36" s="27" t="n">
-        <v>0.5</v>
+        <v>0.09</v>
       </c>
       <c r="C36" s="5" t="s">
-        <v>143</v>
+        <v>144</v>
       </c>
       <c r="D36" s="5" t="s">
-        <v>144</v>
+        <v>130</v>
       </c>
       <c r="E36" s="2"/>
       <c r="F36" s="2"/>
@@ -3261,14 +3270,14 @@
       <c r="A37" s="5" t="s">
         <v>145</v>
       </c>
-      <c r="B37" s="28" t="n">
-        <v>24</v>
+      <c r="B37" s="27" t="n">
+        <v>0.5</v>
       </c>
       <c r="C37" s="5" t="s">
         <v>146</v>
       </c>
       <c r="D37" s="5" t="s">
-        <v>127</v>
+        <v>147</v>
       </c>
       <c r="E37" s="2"/>
       <c r="F37" s="2"/>
@@ -3279,10 +3288,18 @@
       <c r="K37" s="2"/>
     </row>
     <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
+      <c r="A38" s="5" t="s">
+        <v>148</v>
+      </c>
+      <c r="B38" s="28" t="n">
+        <v>24</v>
+      </c>
+      <c r="C38" s="5" t="s">
+        <v>149</v>
+      </c>
+      <c r="D38" s="5" t="s">
+        <v>130</v>
+      </c>
       <c r="E38" s="2"/>
       <c r="F38" s="2"/>
       <c r="G38" s="2"/>
@@ -3292,12 +3309,10 @@
       <c r="K38" s="2"/>
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="21" t="s">
-        <v>147</v>
-      </c>
-      <c r="B39" s="22"/>
-      <c r="C39" s="22"/>
-      <c r="D39" s="22"/>
+      <c r="A39" s="2"/>
+      <c r="B39" s="2"/>
+      <c r="C39" s="2"/>
+      <c r="D39" s="2"/>
       <c r="E39" s="2"/>
       <c r="F39" s="2"/>
       <c r="G39" s="2"/>
@@ -3307,18 +3322,12 @@
       <c r="K39" s="2"/>
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="s">
-        <v>148</v>
-      </c>
-      <c r="B40" s="23" t="n">
-        <v>1500000</v>
-      </c>
-      <c r="C40" s="5" t="s">
-        <v>149</v>
-      </c>
-      <c r="D40" s="5" t="s">
+      <c r="A40" s="21" t="s">
         <v>150</v>
       </c>
+      <c r="B40" s="22"/>
+      <c r="C40" s="22"/>
+      <c r="D40" s="22"/>
       <c r="E40" s="2"/>
       <c r="F40" s="2"/>
       <c r="G40" s="2"/>
@@ -3331,8 +3340,8 @@
       <c r="A41" s="5" t="s">
         <v>151</v>
       </c>
-      <c r="B41" s="27" t="n">
-        <v>0.06</v>
+      <c r="B41" s="23" t="n">
+        <v>1500000</v>
       </c>
       <c r="C41" s="5" t="s">
         <v>152</v>
@@ -3353,13 +3362,13 @@
         <v>154</v>
       </c>
       <c r="B42" s="27" t="n">
-        <v>0.2</v>
+        <v>0.06</v>
       </c>
       <c r="C42" s="5" t="s">
-        <v>138</v>
+        <v>155</v>
       </c>
       <c r="D42" s="5" t="s">
-        <v>155</v>
+        <v>156</v>
       </c>
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
@@ -3370,10 +3379,18 @@
       <c r="K42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="2"/>
-      <c r="B43" s="2"/>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
+      <c r="A43" s="5" t="s">
+        <v>157</v>
+      </c>
+      <c r="B43" s="27" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C43" s="5" t="s">
+        <v>141</v>
+      </c>
+      <c r="D43" s="5" t="s">
+        <v>158</v>
+      </c>
       <c r="E43" s="2"/>
       <c r="F43" s="2"/>
       <c r="G43" s="2"/>
@@ -3383,12 +3400,10 @@
       <c r="K43" s="2"/>
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="21" t="s">
-        <v>156</v>
-      </c>
-      <c r="B44" s="22"/>
-      <c r="C44" s="22"/>
-      <c r="D44" s="22"/>
+      <c r="A44" s="2"/>
+      <c r="B44" s="2"/>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
       <c r="E44" s="2"/>
       <c r="F44" s="2"/>
       <c r="G44" s="2"/>
@@ -3398,18 +3413,12 @@
       <c r="K44" s="2"/>
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5" t="s">
-        <v>157</v>
-      </c>
-      <c r="B45" s="28" t="n">
-        <v>350</v>
-      </c>
-      <c r="C45" s="5" t="s">
-        <v>98</v>
-      </c>
-      <c r="D45" s="5" t="s">
-        <v>158</v>
-      </c>
+      <c r="A45" s="21" t="s">
+        <v>159</v>
+      </c>
+      <c r="B45" s="22"/>
+      <c r="C45" s="22"/>
+      <c r="D45" s="22"/>
       <c r="E45" s="2"/>
       <c r="F45" s="2"/>
       <c r="G45" s="2"/>
@@ -3420,16 +3429,16 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>159</v>
+        <v>160</v>
       </c>
       <c r="B46" s="28" t="n">
-        <v>175</v>
+        <v>350</v>
       </c>
       <c r="C46" s="5" t="s">
         <v>98</v>
       </c>
       <c r="D46" s="5" t="s">
-        <v>160</v>
+        <v>161</v>
       </c>
       <c r="E46" s="2"/>
       <c r="F46" s="2"/>
@@ -3441,13 +3450,13 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>161</v>
-      </c>
-      <c r="B47" s="26" t="n">
-        <v>150</v>
+        <v>162</v>
+      </c>
+      <c r="B47" s="28" t="n">
+        <v>175</v>
       </c>
       <c r="C47" s="5" t="s">
-        <v>162</v>
+        <v>98</v>
       </c>
       <c r="D47" s="5" t="s">
         <v>163</v>
@@ -3464,8 +3473,8 @@
       <c r="A48" s="5" t="s">
         <v>164</v>
       </c>
-      <c r="B48" s="27" t="n">
-        <v>0.075</v>
+      <c r="B48" s="26" t="n">
+        <v>150</v>
       </c>
       <c r="C48" s="5" t="s">
         <v>165</v>
@@ -3485,14 +3494,14 @@
       <c r="A49" s="5" t="s">
         <v>167</v>
       </c>
-      <c r="B49" s="28" t="n">
-        <v>4</v>
+      <c r="B49" s="27" t="n">
+        <v>0.075</v>
       </c>
       <c r="C49" s="5" t="s">
         <v>168</v>
       </c>
       <c r="D49" s="5" t="s">
-        <v>160</v>
+        <v>169</v>
       </c>
       <c r="E49" s="2"/>
       <c r="F49" s="2"/>
@@ -3504,16 +3513,16 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>169</v>
-      </c>
-      <c r="B50" s="26" t="n">
-        <v>220000</v>
+        <v>170</v>
+      </c>
+      <c r="B50" s="28" t="n">
+        <v>4</v>
       </c>
       <c r="C50" s="5" t="s">
-        <v>170</v>
+        <v>171</v>
       </c>
       <c r="D50" s="5" t="s">
-        <v>127</v>
+        <v>163</v>
       </c>
       <c r="E50" s="2"/>
       <c r="F50" s="2"/>
@@ -3522,6 +3531,27 @@
       <c r="I50" s="2"/>
       <c r="J50" s="2"/>
       <c r="K50" s="2"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="s">
+        <v>172</v>
+      </c>
+      <c r="B51" s="26" t="n">
+        <v>220000</v>
+      </c>
+      <c r="C51" s="5" t="s">
+        <v>173</v>
+      </c>
+      <c r="D51" s="5" t="s">
+        <v>130</v>
+      </c>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+      <c r="G51" s="2"/>
+      <c r="H51" s="2"/>
+      <c r="I51" s="2"/>
+      <c r="J51" s="2"/>
+      <c r="K51" s="2"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -3552,7 +3582,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>171</v>
+        <v>174</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -3562,7 +3592,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>172</v>
+        <v>175</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -3583,19 +3613,19 @@
         <v>78</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>86</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3675,7 +3705,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B8" s="33" t="n">
         <f aca="false">SUM(B5:B7)</f>
@@ -3705,7 +3735,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -3715,7 +3745,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B11" s="28" t="n">
         <v>0</v>
@@ -3727,13 +3757,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B12" s="25" t="n">
         <v>0.85</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -3741,13 +3771,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B13" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -3755,13 +3785,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B14" s="26" t="n">
         <v>100000</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -3769,14 +3799,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B15" s="7" t="n">
-        <f aca="false">B8+$B$11*Припущення!$B$49</f>
+        <f aca="false">B8+$B$11*Припущення!$B$50</f>
         <v>25</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
@@ -3792,7 +3822,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B17" s="22"/>
       <c r="C17" s="22"/>
@@ -3802,7 +3832,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B18" s="7" t="n">
         <f aca="false">F8</f>
@@ -3815,7 +3845,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B19" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$13</f>
@@ -3828,7 +3858,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B20" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$14</f>
@@ -3841,7 +3871,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$15</f>
@@ -3854,7 +3884,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">$B$11*Припущення!$B$16</f>
@@ -3867,7 +3897,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B23" s="33" t="n">
         <f aca="false">SUM($B$18:$B$22)</f>
@@ -3880,7 +3910,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B24" s="6" t="n">
         <f aca="false">Припущення!$B$12</f>
@@ -3893,7 +3923,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B25" s="33" t="n">
         <f aca="false">$B$24-$B$23</f>
@@ -3906,7 +3936,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B26" s="36" t="str">
         <f aca="false">IF($B$25&gt;=0,"Вміщується","НЕ ВМІЩУЄТЬСЯ")</f>
@@ -3940,7 +3970,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B29" s="22"/>
       <c r="C29" s="22"/>
@@ -3950,7 +3980,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B30" s="10" t="n">
         <f aca="false">E8</f>
@@ -3963,14 +3993,14 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B31" s="7" t="n">
         <f aca="false">ROUNDUP($B$15*Припущення!$B$19,0)</f>
         <v>8</v>
       </c>
       <c r="C31" s="24" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
@@ -3978,10 +4008,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B32" s="7" t="n">
-        <f aca="false">MIN($B$31,B6)</f>
+        <f aca="false">MIN($B$31,INDEX(B5:B7,Припущення!$B$21))</f>
         <v>8</v>
       </c>
       <c r="C32" s="2"/>
@@ -3991,10 +4021,10 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B33" s="37" t="str">
-        <f aca="false">IF($B$32&lt;$B$31,"Meadow замало — потрібні інші типи","OK")</f>
+        <f aca="false">IF($B$32&lt;$B$31,"Обраного типу замало — потрібні інші типи","OK")</f>
         <v>OK</v>
       </c>
       <c r="C33" s="2"/>
@@ -4004,14 +4034,14 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B34" s="10" t="n">
-        <f aca="false">-$B$31*D6*(1-Припущення!$B$20)</f>
+        <f aca="false">-$B$31*INDEX(D5:D7,Припущення!$B$21)*(1-Припущення!$B$20)</f>
         <v>-1056480</v>
       </c>
       <c r="C34" s="24" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
@@ -4019,10 +4049,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B35" s="10" t="n">
-        <f aca="false">$B$11*Припущення!$B$46*Припущення!$B$47/Припущення!$B$48</f>
+        <f aca="false">$B$11*Припущення!$B$47*Припущення!$B$48/Припущення!$B$49</f>
         <v>0</v>
       </c>
       <c r="C35" s="2"/>
@@ -4032,10 +4062,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B36" s="10" t="n">
-        <f aca="false">$B$11*Припущення!$B$49*Припущення!$B$50</f>
+        <f aca="false">$B$11*Припущення!$B$50*Припущення!$B$51</f>
         <v>0</v>
       </c>
       <c r="C36" s="2"/>
@@ -4045,7 +4075,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B37" s="13" t="n">
         <f aca="false">SUM($B$30,$B$34,$B$35,$B$36)</f>
@@ -4066,7 +4096,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="21" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B39" s="22"/>
       <c r="C39" s="22"/>
@@ -4076,10 +4106,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B40" s="10" t="n">
-        <f aca="false">C8*Припущення!$B$23</f>
+        <f aca="false">C8*Припущення!$B$24</f>
         <v>5214000</v>
       </c>
       <c r="C40" s="2"/>
@@ -4089,10 +4119,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B41" s="10" t="n">
-        <f aca="false">$B$11*Припущення!$B$45*Припущення!$B$24</f>
+        <f aca="false">$B$11*Припущення!$B$46*Припущення!$B$25</f>
         <v>0</v>
       </c>
       <c r="C41" s="2"/>
@@ -4102,10 +4132,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B42" s="10" t="n">
-        <f aca="false">($B$40+$B$41)*Припущення!$B$25</f>
+        <f aca="false">($B$40+$B$41)*Припущення!$B$26</f>
         <v>782100</v>
       </c>
       <c r="C42" s="2"/>
@@ -4115,10 +4145,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B43" s="10" t="n">
-        <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$26</f>
+        <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$27</f>
         <v>299805</v>
       </c>
       <c r="C43" s="2"/>
@@ -4128,10 +4158,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B44" s="10" t="n">
-        <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$27</f>
+        <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$28</f>
         <v>599610</v>
       </c>
       <c r="C44" s="2"/>
@@ -4141,10 +4171,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B45" s="10" t="n">
-        <f aca="false">$B$15*Припущення!$B$28</f>
+        <f aca="false">$B$15*Припущення!$B$29</f>
         <v>375000</v>
       </c>
       <c r="C45" s="2"/>
@@ -4154,10 +4184,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B46" s="10" t="n">
-        <f aca="false">$B$15*Припущення!$B$29</f>
+        <f aca="false">$B$15*Припущення!$B$30</f>
         <v>4000</v>
       </c>
       <c r="C46" s="2"/>
@@ -4167,10 +4197,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B47" s="9" t="n">
-        <f aca="false">Припущення!$B$30</f>
+        <f aca="false">Припущення!$B$31</f>
         <v>50000</v>
       </c>
       <c r="C47" s="2"/>
@@ -4180,10 +4210,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B48" s="10" t="n">
-        <f aca="false">$B$37*Припущення!$B$33</f>
+        <f aca="false">$B$37*Припущення!$B$34</f>
         <v>229078.75</v>
       </c>
       <c r="C48" s="2"/>
@@ -4193,10 +4223,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B49" s="10" t="n">
-        <f aca="false">$B$15*Припущення!$B$34</f>
+        <f aca="false">$B$15*Припущення!$B$35</f>
         <v>37500</v>
       </c>
       <c r="C49" s="2"/>
@@ -4206,10 +4236,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B50" s="9" t="n">
-        <f aca="false">Припущення!$B$40</f>
+        <f aca="false">Припущення!$B$41</f>
         <v>1500000</v>
       </c>
       <c r="C50" s="2"/>
@@ -4219,10 +4249,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B51" s="10" t="n">
-        <f aca="false">$B$50*Припущення!$B$41</f>
+        <f aca="false">$B$50*Припущення!$B$42</f>
         <v>90000</v>
       </c>
       <c r="C51" s="2"/>
@@ -4232,14 +4262,14 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B52" s="10" t="n">
-        <f aca="false">Припущення!$B$35*(Припущення!$B$36*SUM($B$40:$B$49)*Припущення!$B$37/12+($B$50+$B$51)*(Припущення!$B$37+$B$13)/12)</f>
+        <f aca="false">Припущення!$B$36*(Припущення!$B$37*SUM($B$40:$B$49)*Припущення!$B$38/12+($B$50+$B$51)*(Припущення!$B$38+$B$13)/12)</f>
         <v>969398.4375</v>
       </c>
       <c r="C52" s="24" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
@@ -4247,7 +4277,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B53" s="13" t="n">
         <f aca="false">SUM($B$40:$B$52)</f>
@@ -4268,7 +4298,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="21" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B55" s="22"/>
       <c r="C55" s="22"/>
@@ -4278,7 +4308,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B56" s="13" t="n">
         <f aca="false">$B$37-$B$53</f>
@@ -4304,7 +4334,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B58" s="17" t="n">
         <f aca="false">IF($B$53&lt;&gt;0,$B$56/$B$53,0)</f>
@@ -4317,10 +4347,10 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B59" s="36" t="str">
-        <f aca="false">IF($B$57&gt;=Припущення!$B$42,"Досягає цілі","НИЖЧЕ ЦІЛІ")</f>
+        <f aca="false">IF($B$57&gt;=Припущення!$B$43,"Досягає цілі","НИЖЧЕ ЦІЛІ")</f>
         <v>НИЖЧЕ ЦІЛІ</v>
       </c>
       <c r="C59" s="2"/>
@@ -4330,14 +4360,14 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B60" s="10" t="n">
-        <f aca="false">($B$37*(1-Припущення!$B$42)-($B$53-$B$50-$B$51-Припущення!$B$35*($B$50+$B$51)*(Припущення!$B$37+$B$13)/12))/(1+Припущення!$B$41+Припущення!$B$35*(1+Припущення!$B$41)*(Припущення!$B$37+$B$13)/12)</f>
+        <f aca="false">($B$37*(1-Припущення!$B$43)-($B$53-$B$50-$B$51-Припущення!$B$36*($B$50+$B$51)*(Припущення!$B$38+$B$13)/12))/(1+Припущення!$B$42+Припущення!$B$36*(1+Припущення!$B$42)*(Припущення!$B$38+$B$13)/12)</f>
         <v>-754534.847697474</v>
       </c>
       <c r="C60" s="24" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
@@ -4345,7 +4375,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B61" s="13" t="n">
         <f aca="false">$B$12*$B$56-(1-$B$12)*$B$14</f>
@@ -4366,7 +4396,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="21" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B63" s="22"/>
       <c r="C63" s="22"/>
@@ -4376,7 +4406,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B64" s="10" t="n">
         <f aca="false">SUM($B$40:$B$44)</f>
@@ -4389,7 +4419,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B65" s="10" t="n">
         <f aca="false">$B$53-$B$64-$B$48</f>
@@ -4402,14 +4432,14 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B66" s="17" t="n">
-        <f aca="false">($B$64+$B$65)/($B$37*(1-Припущення!$B$33-Припущення!$B$42))-1</f>
+        <f aca="false">($B$64+$B$65)/($B$37*(1-Припущення!$B$34-Припущення!$B$43))-1</f>
         <v>0.397098573124153</v>
       </c>
       <c r="C66" s="24" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
@@ -4443,7 +4473,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>232</v>
+        <v>235</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4453,7 +4483,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>233</v>
+        <v>236</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4474,19 +4504,19 @@
         <v>78</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>173</v>
+        <v>176</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>174</v>
+        <v>177</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>86</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>176</v>
+        <v>179</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4566,7 +4596,7 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>177</v>
+        <v>180</v>
       </c>
       <c r="B8" s="33" t="n">
         <f aca="false">SUM(B5:B7)</f>
@@ -4596,7 +4626,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>178</v>
+        <v>181</v>
       </c>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -4606,7 +4636,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>179</v>
+        <v>182</v>
       </c>
       <c r="B11" s="28" t="n">
         <v>1</v>
@@ -4618,13 +4648,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>180</v>
+        <v>183</v>
       </c>
       <c r="B12" s="25" t="n">
         <v>0.45</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>181</v>
+        <v>184</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -4632,13 +4662,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>182</v>
+        <v>185</v>
       </c>
       <c r="B13" s="28" t="n">
         <v>12</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>183</v>
+        <v>186</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -4646,13 +4676,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>184</v>
+        <v>187</v>
       </c>
       <c r="B14" s="26" t="n">
         <v>250000</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>185</v>
+        <v>188</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -4660,14 +4690,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>186</v>
+        <v>189</v>
       </c>
       <c r="B15" s="7" t="n">
-        <f aca="false">B8+$B$11*Припущення!$B$49</f>
+        <f aca="false">B8+$B$11*Припущення!$B$50</f>
         <v>29</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>187</v>
+        <v>190</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
@@ -4683,7 +4713,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>188</v>
+        <v>191</v>
       </c>
       <c r="B17" s="22"/>
       <c r="C17" s="22"/>
@@ -4693,7 +4723,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>189</v>
+        <v>192</v>
       </c>
       <c r="B18" s="7" t="n">
         <f aca="false">F8</f>
@@ -4706,7 +4736,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>190</v>
+        <v>193</v>
       </c>
       <c r="B19" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$13</f>
@@ -4719,7 +4749,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>191</v>
+        <v>194</v>
       </c>
       <c r="B20" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$14</f>
@@ -4732,7 +4762,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>192</v>
+        <v>195</v>
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$15</f>
@@ -4745,7 +4775,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>193</v>
+        <v>196</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">$B$11*Припущення!$B$16</f>
@@ -4758,7 +4788,7 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>194</v>
+        <v>197</v>
       </c>
       <c r="B23" s="33" t="n">
         <f aca="false">SUM($B$18:$B$22)</f>
@@ -4771,7 +4801,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>195</v>
+        <v>198</v>
       </c>
       <c r="B24" s="6" t="n">
         <f aca="false">Припущення!$B$12</f>
@@ -4784,7 +4814,7 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>196</v>
+        <v>199</v>
       </c>
       <c r="B25" s="33" t="n">
         <f aca="false">$B$24-$B$23</f>
@@ -4797,7 +4827,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>197</v>
+        <v>200</v>
       </c>
       <c r="B26" s="36" t="str">
         <f aca="false">IF($B$25&gt;=0,"Вміщується","НЕ ВМІЩУЄТЬСЯ")</f>
@@ -4831,7 +4861,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>198</v>
+        <v>201</v>
       </c>
       <c r="B29" s="22"/>
       <c r="C29" s="22"/>
@@ -4841,7 +4871,7 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>199</v>
+        <v>202</v>
       </c>
       <c r="B30" s="10" t="n">
         <f aca="false">E8</f>
@@ -4854,14 +4884,14 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>200</v>
+        <v>203</v>
       </c>
       <c r="B31" s="7" t="n">
         <f aca="false">ROUNDUP($B$15*Припущення!$B$19,0)</f>
         <v>9</v>
       </c>
       <c r="C31" s="24" t="s">
-        <v>201</v>
+        <v>204</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
@@ -4869,10 +4899,10 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>202</v>
+        <v>205</v>
       </c>
       <c r="B32" s="7" t="n">
-        <f aca="false">MIN($B$31,B6)</f>
+        <f aca="false">MIN($B$31,INDEX(B5:B7,Припущення!$B$21))</f>
         <v>8</v>
       </c>
       <c r="C32" s="2"/>
@@ -4882,11 +4912,11 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>203</v>
+        <v>206</v>
       </c>
       <c r="B33" s="37" t="str">
-        <f aca="false">IF($B$32&lt;$B$31,"Meadow замало — потрібні інші типи","OK")</f>
-        <v>Meadow замало — потрібні інші типи</v>
+        <f aca="false">IF($B$32&lt;$B$31,"Обраного типу замало — потрібні інші типи","OK")</f>
+        <v>Обраного типу замало — потрібні інші типи</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -4895,14 +4925,14 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>204</v>
+        <v>207</v>
       </c>
       <c r="B34" s="10" t="n">
-        <f aca="false">-$B$31*D6*(1-Припущення!$B$20)</f>
+        <f aca="false">-$B$31*INDEX(D5:D7,Припущення!$B$21)*(1-Припущення!$B$20)</f>
         <v>-1188540</v>
       </c>
       <c r="C34" s="24" t="s">
-        <v>205</v>
+        <v>208</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
@@ -4910,10 +4940,10 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>206</v>
+        <v>209</v>
       </c>
       <c r="B35" s="10" t="n">
-        <f aca="false">$B$11*Припущення!$B$46*Припущення!$B$47/Припущення!$B$48</f>
+        <f aca="false">$B$11*Припущення!$B$47*Припущення!$B$48/Припущення!$B$49</f>
         <v>350000</v>
       </c>
       <c r="C35" s="2"/>
@@ -4923,10 +4953,10 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>207</v>
+        <v>210</v>
       </c>
       <c r="B36" s="10" t="n">
-        <f aca="false">$B$11*Припущення!$B$49*Припущення!$B$50</f>
+        <f aca="false">$B$11*Припущення!$B$50*Припущення!$B$51</f>
         <v>880000</v>
       </c>
       <c r="C36" s="2"/>
@@ -4936,7 +4966,7 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>208</v>
+        <v>211</v>
       </c>
       <c r="B37" s="13" t="n">
         <f aca="false">SUM($B$30,$B$34,$B$35,$B$36)</f>
@@ -4957,7 +4987,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="21" t="s">
-        <v>209</v>
+        <v>212</v>
       </c>
       <c r="B39" s="22"/>
       <c r="C39" s="22"/>
@@ -4967,10 +4997,10 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>117</v>
+        <v>120</v>
       </c>
       <c r="B40" s="10" t="n">
-        <f aca="false">C8*Припущення!$B$23</f>
+        <f aca="false">C8*Припущення!$B$24</f>
         <v>5191200</v>
       </c>
       <c r="C40" s="2"/>
@@ -4980,10 +5010,10 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>210</v>
+        <v>213</v>
       </c>
       <c r="B41" s="10" t="n">
-        <f aca="false">$B$11*Припущення!$B$45*Припущення!$B$24</f>
+        <f aca="false">$B$11*Припущення!$B$46*Припущення!$B$25</f>
         <v>1050000</v>
       </c>
       <c r="C41" s="2"/>
@@ -4993,10 +5023,10 @@
     </row>
     <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A42" s="5" t="s">
-        <v>122</v>
+        <v>125</v>
       </c>
       <c r="B42" s="10" t="n">
-        <f aca="false">($B$40+$B$41)*Припущення!$B$25</f>
+        <f aca="false">($B$40+$B$41)*Припущення!$B$26</f>
         <v>936180</v>
       </c>
       <c r="C42" s="2"/>
@@ -5006,10 +5036,10 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>211</v>
+        <v>214</v>
       </c>
       <c r="B43" s="10" t="n">
-        <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$26</f>
+        <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$27</f>
         <v>358869</v>
       </c>
       <c r="C43" s="2"/>
@@ -5019,10 +5049,10 @@
     </row>
     <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A44" s="5" t="s">
-        <v>128</v>
+        <v>131</v>
       </c>
       <c r="B44" s="10" t="n">
-        <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$27</f>
+        <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$28</f>
         <v>717738</v>
       </c>
       <c r="C44" s="2"/>
@@ -5032,10 +5062,10 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>212</v>
+        <v>215</v>
       </c>
       <c r="B45" s="10" t="n">
-        <f aca="false">$B$15*Припущення!$B$28</f>
+        <f aca="false">$B$15*Припущення!$B$29</f>
         <v>435000</v>
       </c>
       <c r="C45" s="2"/>
@@ -5045,10 +5075,10 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>213</v>
+        <v>216</v>
       </c>
       <c r="B46" s="10" t="n">
-        <f aca="false">$B$15*Припущення!$B$29</f>
+        <f aca="false">$B$15*Припущення!$B$30</f>
         <v>4640</v>
       </c>
       <c r="C46" s="2"/>
@@ -5058,10 +5088,10 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>214</v>
+        <v>217</v>
       </c>
       <c r="B47" s="9" t="n">
-        <f aca="false">Припущення!$B$30</f>
+        <f aca="false">Припущення!$B$31</f>
         <v>50000</v>
       </c>
       <c r="C47" s="2"/>
@@ -5071,10 +5101,10 @@
     </row>
     <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A48" s="5" t="s">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="B48" s="10" t="n">
-        <f aca="false">$B$37*Припущення!$B$33</f>
+        <f aca="false">$B$37*Припущення!$B$34</f>
         <v>255776.5</v>
       </c>
       <c r="C48" s="2"/>
@@ -5084,10 +5114,10 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>215</v>
+        <v>218</v>
       </c>
       <c r="B49" s="10" t="n">
-        <f aca="false">$B$15*Припущення!$B$34</f>
+        <f aca="false">$B$15*Припущення!$B$35</f>
         <v>43500</v>
       </c>
       <c r="C49" s="2"/>
@@ -5097,10 +5127,10 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>216</v>
+        <v>219</v>
       </c>
       <c r="B50" s="9" t="n">
-        <f aca="false">Припущення!$B$40</f>
+        <f aca="false">Припущення!$B$41</f>
         <v>1500000</v>
       </c>
       <c r="C50" s="2"/>
@@ -5110,10 +5140,10 @@
     </row>
     <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A51" s="5" t="s">
-        <v>151</v>
+        <v>154</v>
       </c>
       <c r="B51" s="10" t="n">
-        <f aca="false">$B$50*Припущення!$B$41</f>
+        <f aca="false">$B$50*Припущення!$B$42</f>
         <v>90000</v>
       </c>
       <c r="C51" s="2"/>
@@ -5123,14 +5153,14 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>217</v>
+        <v>220</v>
       </c>
       <c r="B52" s="10" t="n">
-        <f aca="false">Припущення!$B$35*(Припущення!$B$36*SUM($B$40:$B$49)*Припущення!$B$37/12+($B$50+$B$51)*(Припущення!$B$37+$B$13)/12)</f>
+        <f aca="false">Припущення!$B$36*(Припущення!$B$37*SUM($B$40:$B$49)*Припущення!$B$38/12+($B$50+$B$51)*(Припущення!$B$38+$B$13)/12)</f>
         <v>1243161.315</v>
       </c>
       <c r="C52" s="24" t="s">
-        <v>218</v>
+        <v>221</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
@@ -5138,7 +5168,7 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>219</v>
+        <v>222</v>
       </c>
       <c r="B53" s="13" t="n">
         <f aca="false">SUM($B$40:$B$52)</f>
@@ -5159,7 +5189,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="21" t="s">
-        <v>220</v>
+        <v>223</v>
       </c>
       <c r="B55" s="22"/>
       <c r="C55" s="22"/>
@@ -5169,7 +5199,7 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="s">
-        <v>221</v>
+        <v>224</v>
       </c>
       <c r="B56" s="13" t="n">
         <f aca="false">$B$37-$B$53</f>
@@ -5195,7 +5225,7 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>222</v>
+        <v>225</v>
       </c>
       <c r="B58" s="17" t="n">
         <f aca="false">IF($B$53&lt;&gt;0,$B$56/$B$53,0)</f>
@@ -5208,10 +5238,10 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>223</v>
+        <v>226</v>
       </c>
       <c r="B59" s="36" t="str">
-        <f aca="false">IF($B$57&gt;=Припущення!$B$42,"Досягає цілі","НИЖЧЕ ЦІЛІ")</f>
+        <f aca="false">IF($B$57&gt;=Припущення!$B$43,"Досягає цілі","НИЖЧЕ ЦІЛІ")</f>
         <v>НИЖЧЕ ЦІЛІ</v>
       </c>
       <c r="C59" s="2"/>
@@ -5221,14 +5251,14 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>224</v>
+        <v>227</v>
       </c>
       <c r="B60" s="10" t="n">
-        <f aca="false">($B$37*(1-Припущення!$B$42)-($B$53-$B$50-$B$51-Припущення!$B$35*($B$50+$B$51)*(Припущення!$B$37+$B$13)/12))/(1+Припущення!$B$41+Припущення!$B$35*(1+Припущення!$B$41)*(Припущення!$B$37+$B$13)/12)</f>
+        <f aca="false">($B$37*(1-Припущення!$B$43)-($B$53-$B$50-$B$51-Припущення!$B$36*($B$50+$B$51)*(Припущення!$B$38+$B$13)/12))/(1+Припущення!$B$42+Припущення!$B$36*(1+Припущення!$B$42)*(Припущення!$B$38+$B$13)/12)</f>
         <v>-1241952.76704799</v>
       </c>
       <c r="C60" s="24" t="s">
-        <v>225</v>
+        <v>228</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
@@ -5236,7 +5266,7 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>226</v>
+        <v>229</v>
       </c>
       <c r="B61" s="13" t="n">
         <f aca="false">$B$12*$B$56-(1-$B$12)*$B$14</f>
@@ -5257,7 +5287,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="21" t="s">
-        <v>227</v>
+        <v>230</v>
       </c>
       <c r="B63" s="22"/>
       <c r="C63" s="22"/>
@@ -5267,7 +5297,7 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>228</v>
+        <v>231</v>
       </c>
       <c r="B64" s="10" t="n">
         <f aca="false">SUM($B$40:$B$44)</f>
@@ -5280,7 +5310,7 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>229</v>
+        <v>232</v>
       </c>
       <c r="B65" s="10" t="n">
         <f aca="false">$B$53-$B$64-$B$48</f>
@@ -5293,14 +5323,14 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>230</v>
+        <v>233</v>
       </c>
       <c r="B66" s="17" t="n">
-        <f aca="false">($B$64+$B$65)/($B$37*(1-Припущення!$B$33-Припущення!$B$42))-1</f>
+        <f aca="false">($B$64+$B$65)/($B$37*(1-Припущення!$B$34-Припущення!$B$43))-1</f>
         <v>0.465529515656405</v>
       </c>
       <c r="C66" s="24" t="s">
-        <v>231</v>
+        <v>234</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>

</xml_diff>

<commit_message>
Build up turnkey house cost from ZON shell price; adopt team sale prices and 10/8/7 mix
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014iit8YdqqexD3WDZo9gb62
</commit_message>
<xml_diff>
--- a/model/ZON_Wivenhoe_Appraisal.xlsx
+++ b/model/ZON_Wivenhoe_Appraisal.xlsx
@@ -11,8 +11,9 @@
     <sheet name="Порівняння" sheetId="1" state="visible" r:id="rId3"/>
     <sheet name="Покращений випадок" sheetId="2" state="visible" r:id="rId4"/>
     <sheet name="Припущення" sheetId="3" state="visible" r:id="rId5"/>
-    <sheet name="Сценарій A" sheetId="4" state="visible" r:id="rId6"/>
-    <sheet name="Сценарій B" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Собівартість будинку" sheetId="4" state="visible" r:id="rId6"/>
+    <sheet name="Сценарій A" sheetId="5" state="visible" r:id="rId7"/>
+    <sheet name="Сценарій B" sheetId="6" state="visible" r:id="rId8"/>
   </sheets>
   <calcPr iterateCount="100" refMode="A1" iterate="false" iterateDelta="0.0001"/>
   <extLst>
@@ -24,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="339" uniqueCount="237">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="274">
   <si>
     <t xml:space="preserve">ZON Wivenhoe — порівняння сценаріїв</t>
   </si>
@@ -296,22 +297,22 @@
     <t xml:space="preserve">Lake House Compact 61</t>
   </si>
   <si>
-    <t xml:space="preserve">GIA з брифу. NDSS 2b3p 1 пов. = 61 м² (не проходить як 2b4p = 70). Ціна — припущення.</t>
+    <t xml:space="preserve">GIA з брифу. NDSS 2b3p 1 пов. = 61 м². Ціна £340k — робоча ціна команди ZON, не підтверджена агентом.</t>
   </si>
   <si>
     <t xml:space="preserve">Meadow 71</t>
   </si>
   <si>
-    <t xml:space="preserve">GIA з брифу. NDSS 2b4p 1 пов. = 70 м². Юніт для доступного житла S106. Ціна — припущення.</t>
+    <t xml:space="preserve">GIA з брифу. NDSS 2b4p 1 пов. = 70 м². Ціна £390k — робоча ціна команди ZON, не підтверджена агентом.</t>
   </si>
   <si>
     <t xml:space="preserve">Country 140</t>
   </si>
   <si>
-    <t xml:space="preserve">GIA з брифу. NDSS 3b6p 1 пов. = 95 м². Ціна — припущення.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ціни £/м² — ринкове припущення (~£430–455/фут²) для нових бунгало в CO7. Треба підтвердити звітом агента (Savills / Fenn Wright / Beresfords).</t>
+    <t xml:space="preserve">GIA з брифу. NDSS 3b6p 1 пов. = 95 м². Ціна £550k — робоча ціна команди ZON, не підтверджена агентом.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ціни — робочі ціни команди ZON (£340k / £390k / £550k). Треба підтвердити звітом агента (Savills / Fenn Wright / Beresfords).</t>
   </si>
   <si>
     <t xml:space="preserve">Ділянка та планування</t>
@@ -386,283 +387,394 @@
     <t xml:space="preserve">Вартість будівництва</t>
   </si>
   <si>
+    <t xml:space="preserve">Будівництво бунгало (під ключ)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£/м² GIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Розрахунок з оболонки ZON £1 700/м² — аркуш «Собівартість будинку»</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Будівництво ZON Hub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Припущення: змішане використання, комерційне обладнання</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Зовнішні роботи та мережі</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% будівництва</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Припущення: дороги, SuDS, містки, мережі, підстанція</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Резерв на непередбачене</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% буд.+зовн.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Припущення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Проєктування та консультанти</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Внески S106 / інфраструктура</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£/юніт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Припущення; уточнити з угоди S106</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Essex Coast RAMS</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Приблизний тариф; перевірити поточну ставку</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BNG за межами ділянки (кредити)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£ разом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Продаж і фінансування</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Маркетинг і агенти</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% GDV</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Юридичні витрати на продаж</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ставка девелоперського кредиту</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% річних</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Середня вибірка кредиту</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% витрат</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Стандартне спрощення S-кривої</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Програма: будівництво + продаж</t>
+  </si>
+  <si>
+    <t xml:space="preserve">місяців</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Земля і ціль</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ціна землі</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ЗАГЛУШКА — замінити фактичною ціною / ціною опціону</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SDLT + юридичні на землю</t>
+  </si>
+  <si>
+    <t xml:space="preserve">% ціни землі</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Припущення (ставки для нежитлової нерухомості)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Цільова маржа девелопера</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Типовий орієнтир кредиторів 17–20%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZON Hub (лише сценарій B)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Hub GIA разом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Бриф: 175 + 175 м²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кав'ярня / коворкінг GIA</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Бриф</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Оренда кав'ярні</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£/м²/рік</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Припущення для невеликої локації</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дохідність при оцінці кав'ярні</t>
+  </si>
+  <si>
+    <t xml:space="preserve">%</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Припущення (вторинна роздрібна торгівля)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Бутік-апартаменти</t>
+  </si>
+  <si>
+    <t xml:space="preserve">шт.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вартість апартамента (продаж)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£/шт.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Собівартість будинку під ключ — від оболонки ZON £1 700/м²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Оболонка ZON (£1 700/м²) містить лише будинок і систему опалення. Усе, що потрібно, щоб будинок можна було продати під іпотеку, додано нижче. Ставки — припущення центрального сценарію; діапазони в примітках.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Стаття</t>
+  </si>
+  <si>
+    <t xml:space="preserve">База</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Compact 61</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Примітка / діапазон</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кількість у сценарії A</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Прямі витрати на будинок (за одиницю, £)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Оболонка ZON + опалення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Від команди ZON. Стіни, дах, вікна, опалення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фундаменти</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£120–220/м²; гвинтові палі — нижня межа</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доставка, кран, монтаж, герметизація</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£90–160/м²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Підлоги та фарбування</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£40–80/м²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сонячні панелі в дах (вимога Future Homes Standard)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">за будинок</t>
+  </si>
+  <si>
+    <t xml:space="preserve">3–5 кВт; батарея — опція ZON Ready</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вентиляція (dMEV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">MVHR — +£3–4k</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Кухня з технікою</t>
+  </si>
+  <si>
+    <t xml:space="preserve">середній клас</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Санвузли</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Country — 2 санвузли</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Гарантія 10 років, Building Control, SAP/EPC, тест повітря</t>
+  </si>
+  <si>
+    <t xml:space="preserve">без гарантії немає іпотеки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Роботи на ділянці: тераса, огорожа, доріжки, газон</t>
+  </si>
+  <si>
+    <t xml:space="preserve">живоплоти з граба — тут</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Разом прямі</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Майданчик і маржа підрядника</t>
+  </si>
+  <si>
+    <t xml:space="preserve">10–15%; менше, якщо ZON сам веде будівництво</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Будинок під ключ, £</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Під ключ, £/м²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Середнє під ключ для міксу сценарію A, £/м²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Не входить сюди (рахується в моделі окремо): дороги, мережі та підключення, SuDS — «Зовнішні роботи»; проєктування, резерв, S106, продаж, фінансування, земля.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сценарій A — 25 бунгало в межах outline consent</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Шлях: Reserved Matters. Без Hub. Відповідає ліміту 25 юнітів (за словами користувача).</t>
+  </si>
+  <si>
+    <t xml:space="preserve">К-сть</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GIA разом, м²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GDV ринковий, £</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ділянки, м²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Разом бунгало</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Параметри сценарію</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZON Hub включено (1 = так, 0 = ні)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ймовірність отримати дозвіл</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Експертна оцінка, не факт</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Додаткова затримка на планування</t>
+  </si>
+  <si>
+    <t xml:space="preserve">місяців; фінансування землі тим часом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Витрати, якщо в дозволі відмовлять</t>
+  </si>
+  <si>
+    <t xml:space="preserve">консультанти, звіти, апеляція</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Житлових юнітів разом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">бунгало + апартаменти Hub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Баланс території</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Приватні ділянки</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Дороги та паркування</t>
+  </si>
+  <si>
+    <t xml:space="preserve">SuDS / відкритий простір</t>
+  </si>
+  <si>
+    <t xml:space="preserve">BNG / буфери</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZON Hub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Потрібно разом, м²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Доступно, м²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Запас (+) / дефіцит (−), м²</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Перевірка</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Виручка (GDV)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Бунгало за ринковою ціною</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Юнітів доступного житла (вимога)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">округлення вгору від усіх житлових юнітів</t>
+  </si>
+  <si>
+    <t xml:space="preserve">…з них покривається обраним типом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Перевірка покриття</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Знижка на доступне житло</t>
+  </si>
+  <si>
+    <t xml:space="preserve">усі доступні юніти — за ціною обраного типу</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZON Hub: кав'ярня (капіталізація)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">ZON Hub: апартаменти</t>
+  </si>
+  <si>
+    <t xml:space="preserve">GDV разом</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Витрати (TDC)</t>
+  </si>
+  <si>
     <t xml:space="preserve">Будівництво бунгало</t>
-  </si>
-  <si>
-    <t xml:space="preserve">£/м² GIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Припущення, діапазон £2 100–2 800: високий клас, ASHP + PV + MVHR</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Будівництво ZON Hub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Припущення: змішане використання, комерційне обладнання</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Зовнішні роботи та мережі</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% будівництва</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Припущення: дороги, SuDS, містки, мережі, підстанція</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Резерв на непередбачене</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% буд.+зовн.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Припущення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Проєктування та консультанти</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Внески S106 / інфраструктура</t>
-  </si>
-  <si>
-    <t xml:space="preserve">£/юніт</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Припущення; уточнити з угоди S106</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Essex Coast RAMS</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Приблизний тариф; перевірити поточну ставку</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BNG за межами ділянки (кредити)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">£ разом</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Продаж і фінансування</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Маркетинг і агенти</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% GDV</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Юридичні витрати на продаж</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ставка девелоперського кредиту</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% річних</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Середня вибірка кредиту</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% витрат</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Стандартне спрощення S-кривої</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Програма: будівництво + продаж</t>
-  </si>
-  <si>
-    <t xml:space="preserve">місяців</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Земля і ціль</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ціна землі</t>
-  </si>
-  <si>
-    <t xml:space="preserve">£</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ЗАГЛУШКА — замінити фактичною ціною / ціною опціону</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SDLT + юридичні на землю</t>
-  </si>
-  <si>
-    <t xml:space="preserve">% ціни землі</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Припущення (ставки для нежитлової нерухомості)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Цільова маржа девелопера</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Типовий орієнтир кредиторів 17–20%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZON Hub (лише сценарій B)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Hub GIA разом</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Бриф: 175 + 175 м²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Кав'ярня / коворкінг GIA</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Бриф</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Оренда кав'ярні</t>
-  </si>
-  <si>
-    <t xml:space="preserve">£/м²/рік</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Припущення для невеликої локації</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Дохідність при оцінці кав'ярні</t>
-  </si>
-  <si>
-    <t xml:space="preserve">%</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Припущення (вторинна роздрібна торгівля)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Бутік-апартаменти</t>
-  </si>
-  <si>
-    <t xml:space="preserve">шт.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вартість апартамента (продаж)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">£/шт.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Сценарій A — 25 бунгало в межах outline consent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Шлях: Reserved Matters. Без Hub. Відповідає ліміту 25 юнітів (за словами користувача).</t>
-  </si>
-  <si>
-    <t xml:space="preserve">К-сть</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GIA разом, м²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GDV ринковий, £</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ділянки, м²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Разом бунгало</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Параметри сценарію</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZON Hub включено (1 = так, 0 = ні)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ймовірність отримати дозвіл</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Експертна оцінка, не факт</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Додаткова затримка на планування</t>
-  </si>
-  <si>
-    <t xml:space="preserve">місяців; фінансування землі тим часом</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Витрати, якщо в дозволі відмовлять</t>
-  </si>
-  <si>
-    <t xml:space="preserve">консультанти, звіти, апеляція</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Житлових юнітів разом</t>
-  </si>
-  <si>
-    <t xml:space="preserve">бунгало + апартаменти Hub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Баланс території</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Приватні ділянки</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Дороги та паркування</t>
-  </si>
-  <si>
-    <t xml:space="preserve">SuDS / відкритий простір</t>
-  </si>
-  <si>
-    <t xml:space="preserve">BNG / буфери</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZON Hub</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Потрібно разом, м²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Доступно, м²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Запас (+) / дефіцит (−), м²</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Перевірка</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Виручка (GDV)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Бунгало за ринковою ціною</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Юнітів доступного житла (вимога)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">округлення вгору від усіх житлових юнітів</t>
-  </si>
-  <si>
-    <t xml:space="preserve">…з них покривається обраним типом</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Перевірка покриття</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Знижка на доступне житло</t>
-  </si>
-  <si>
-    <t xml:space="preserve">усі доступні юніти — за ціною обраного типу</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZON Hub: кав'ярня (капіталізація)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">ZON Hub: апартаменти</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GDV разом</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Витрати (TDC)</t>
   </si>
   <si>
     <t xml:space="preserve">Будівництво Hub</t>
@@ -906,7 +1018,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="38">
+  <cellXfs count="41">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1031,6 +1143,22 @@
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="167" fontId="9" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="170" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
+    <xf numFmtId="167" fontId="10" fillId="4" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
     <xf numFmtId="164" fontId="9" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -1044,10 +1172,6 @@
       <protection locked="true" hidden="false"/>
     </xf>
     <xf numFmtId="170" fontId="10" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="167" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -1387,7 +1511,7 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">'Сценарій A'!$B$25</f>
-        <v>-480.950000000001</v>
+        <v>-450.950000000001</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">'Сценарій B'!$B$25</f>
@@ -1395,7 +1519,7 @@
       </c>
       <c r="D6" s="7" t="n">
         <f aca="false">C6-B6</f>
-        <v>-870</v>
+        <v>-900</v>
       </c>
       <c r="E6" s="2"/>
       <c r="F6" s="2"/>
@@ -1422,7 +1546,7 @@
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">'Сценарій A'!$B$27</f>
-        <v>412.4</v>
+        <v>411.2</v>
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">'Сценарій B'!$B$27</f>
@@ -1430,7 +1554,7 @@
       </c>
       <c r="D8" s="7" t="n">
         <f aca="false">C8-B8</f>
-        <v>-1.19999999999999</v>
+        <v>0</v>
       </c>
       <c r="E8" s="2"/>
       <c r="F8" s="2"/>
@@ -1460,15 +1584,15 @@
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">'Сценарій A'!$B$37</f>
-        <v>9163150</v>
+        <v>9282000</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">'Сценарій B'!$B$37</f>
-        <v>10231060</v>
+        <v>10376000</v>
       </c>
       <c r="D10" s="10" t="n">
         <f aca="false">C10-B10</f>
-        <v>1067910</v>
+        <v>1094000</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -1479,15 +1603,15 @@
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">'Сценарій A'!$B$53</f>
-        <v>10150492.1875</v>
+        <v>11315632.29016</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">'Сценарій B'!$B$53</f>
-        <v>11876064.815</v>
+        <v>12973875.89016</v>
       </c>
       <c r="D11" s="10" t="n">
         <f aca="false">C11-B11</f>
-        <v>1725572.6275</v>
+        <v>1658243.6</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -1498,15 +1622,15 @@
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">'Сценарій A'!$B$56</f>
-        <v>-987342.1875</v>
+        <v>-2033632.29016</v>
       </c>
       <c r="C12" s="12" t="n">
         <f aca="false">'Сценарій B'!$B$56</f>
-        <v>-1645004.815</v>
+        <v>-2597875.89016</v>
       </c>
       <c r="D12" s="13" t="n">
         <f aca="false">C12-B12</f>
-        <v>-657662.6275</v>
+        <v>-564243.6</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
@@ -1517,15 +1641,15 @@
       </c>
       <c r="B13" s="14" t="n">
         <f aca="false">'Сценарій A'!$B$57</f>
-        <v>-0.107751394171218</v>
+        <v>-0.219094192001724</v>
       </c>
       <c r="C13" s="14" t="n">
         <f aca="false">'Сценарій B'!$B$57</f>
-        <v>-0.160785374633713</v>
+        <v>-0.250373543770239</v>
       </c>
       <c r="D13" s="15" t="n">
         <f aca="false">C13-B13</f>
-        <v>-0.053033980462495</v>
+        <v>-0.0312793517685152</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
@@ -1552,15 +1676,15 @@
       </c>
       <c r="B15" s="9" t="n">
         <f aca="false">'Сценарій A'!$B$60</f>
-        <v>-754534.847697474</v>
+        <v>-1610035.40946594</v>
       </c>
       <c r="C15" s="9" t="n">
         <f aca="false">'Сценарій B'!$B$60</f>
-        <v>-1241952.76704799</v>
+        <v>-1971308.78781756</v>
       </c>
       <c r="D15" s="10" t="n">
         <f aca="false">C15-B15</f>
-        <v>-487417.919350513</v>
+        <v>-361273.378351619</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
@@ -1571,15 +1695,15 @@
       </c>
       <c r="B16" s="16" t="n">
         <f aca="false">'Сценарій A'!$B$66</f>
-        <v>0.397098573124153</v>
+        <v>0.540766699357063</v>
       </c>
       <c r="C16" s="16" t="n">
         <f aca="false">'Сценарій B'!$B$66</f>
-        <v>0.465529515656405</v>
+        <v>0.581127153251922</v>
       </c>
       <c r="D16" s="17" t="n">
         <f aca="false">C16-B16</f>
-        <v>0.0684309425322516</v>
+        <v>0.0403604538948583</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
@@ -1609,15 +1733,15 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">'Сценарій A'!$B$61</f>
-        <v>-854240.859375</v>
+        <v>-1743587.446636</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">'Сценарій B'!$B$61</f>
-        <v>-877752.16675</v>
+        <v>-1306544.150572</v>
       </c>
       <c r="D18" s="13" t="n">
         <f aca="false">C18-B18</f>
-        <v>-23511.3073749997</v>
+        <v>437043.296064</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
@@ -1674,23 +1798,23 @@
       </c>
       <c r="B23" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
-        <v>-1191197.8125</v>
+        <v>-2142479.32776</v>
       </c>
       <c r="C23" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
-        <v>-1535973.5625</v>
+        <v>-2540553.30896</v>
       </c>
       <c r="D23" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
-        <v>-1880749.3125</v>
+        <v>-2938627.29016</v>
       </c>
       <c r="E23" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
-        <v>-2225525.0625</v>
+        <v>-3336701.27136</v>
       </c>
       <c r="F23" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
-        <v>-2570300.8125</v>
+        <v>-3734775.25256</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1699,23 +1823,23 @@
       </c>
       <c r="B24" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
-        <v>-744494.25</v>
+        <v>-1689981.82776</v>
       </c>
       <c r="C24" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
-        <v>-1089270</v>
+        <v>-2088055.80896</v>
       </c>
       <c r="D24" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
-        <v>-1434045.75</v>
+        <v>-2486129.79016</v>
       </c>
       <c r="E24" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
-        <v>-1778821.5</v>
+        <v>-2884203.77136</v>
       </c>
       <c r="F24" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
-        <v>-2123597.25</v>
+        <v>-3282277.75256</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1724,23 +1848,23 @@
       </c>
       <c r="B25" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
-        <v>-297790.6875</v>
+        <v>-1237484.32776</v>
       </c>
       <c r="C25" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
-        <v>-642566.4375</v>
+        <v>-1635558.30896</v>
       </c>
       <c r="D25" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
-        <v>-987342.1875</v>
+        <v>-2033632.29016</v>
       </c>
       <c r="E25" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
-        <v>-1332117.9375</v>
+        <v>-2431706.27136</v>
       </c>
       <c r="F25" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
-        <v>-1676893.6875</v>
+        <v>-2829780.25256</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1749,23 +1873,23 @@
       </c>
       <c r="B26" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
-        <v>148912.875</v>
+        <v>-784986.827760001</v>
       </c>
       <c r="C26" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
-        <v>-195862.875</v>
+        <v>-1183060.80896</v>
       </c>
       <c r="D26" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
-        <v>-540638.625</v>
+        <v>-1581134.79016</v>
       </c>
       <c r="E26" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
-        <v>-885414.375</v>
+        <v>-1979208.77136</v>
       </c>
       <c r="F26" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
-        <v>-1230190.125</v>
+        <v>-2377282.75256</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1774,23 +1898,23 @@
       </c>
       <c r="B27" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
-        <v>595616.4375</v>
+        <v>-332489.327760001</v>
       </c>
       <c r="C27" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
-        <v>250840.6875</v>
+        <v>-730563.30896</v>
       </c>
       <c r="D27" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
-        <v>-93935.0625</v>
+        <v>-1128637.29016</v>
       </c>
       <c r="E27" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
-        <v>-438710.8125</v>
+        <v>-1526711.27136</v>
       </c>
       <c r="F27" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
-        <v>-783486.562500001</v>
+        <v>-1924785.25256</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1845,23 +1969,23 @@
       </c>
       <c r="B32" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
-        <v>-1817134.465</v>
+        <v>-2683782.92776</v>
       </c>
       <c r="C32" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
-        <v>-2229833.815</v>
+        <v>-3146659.40896</v>
       </c>
       <c r="D32" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
-        <v>-2642533.165</v>
+        <v>-3609535.89016</v>
       </c>
       <c r="E32" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
-        <v>-3055232.515</v>
+        <v>-4072412.37136</v>
       </c>
       <c r="F32" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
-        <v>-3467931.865</v>
+        <v>-4535288.85256</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1870,23 +1994,23 @@
       </c>
       <c r="B33" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
-        <v>-1318370.29</v>
+        <v>-2177952.92776</v>
       </c>
       <c r="C33" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
-        <v>-1731069.64</v>
+        <v>-2640829.40896</v>
       </c>
       <c r="D33" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
-        <v>-2143768.99</v>
+        <v>-3103705.89016</v>
       </c>
       <c r="E33" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
-        <v>-2556468.34</v>
+        <v>-3566582.37136</v>
       </c>
       <c r="F33" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
-        <v>-2969167.69</v>
+        <v>-4029458.85256</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1895,23 +2019,23 @@
       </c>
       <c r="B34" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
-        <v>-819606.114999999</v>
+        <v>-1672122.92776</v>
       </c>
       <c r="C34" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
-        <v>-1232305.465</v>
+        <v>-2134999.40896</v>
       </c>
       <c r="D34" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
-        <v>-1645004.815</v>
+        <v>-2597875.89016</v>
       </c>
       <c r="E34" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
-        <v>-2057704.165</v>
+        <v>-3060752.37136</v>
       </c>
       <c r="F34" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
-        <v>-2470403.515</v>
+        <v>-3523628.85256</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1920,23 +2044,23 @@
       </c>
       <c r="B35" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
-        <v>-320841.94</v>
+        <v>-1166292.92776</v>
       </c>
       <c r="C35" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
-        <v>-733541.29</v>
+        <v>-1629169.40896</v>
       </c>
       <c r="D35" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
-        <v>-1146240.64</v>
+        <v>-2092045.89016</v>
       </c>
       <c r="E35" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
-        <v>-1558939.99</v>
+        <v>-2554922.37136</v>
       </c>
       <c r="F35" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
-        <v>-1971639.34</v>
+        <v>-3017798.85256</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1945,23 +2069,23 @@
       </c>
       <c r="B36" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
-        <v>177922.235</v>
+        <v>-660462.92776</v>
       </c>
       <c r="C36" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
-        <v>-234777.114999999</v>
+        <v>-1123339.40896</v>
       </c>
       <c r="D36" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
-        <v>-647476.465</v>
+        <v>-1586215.89016</v>
       </c>
       <c r="E36" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
-        <v>-1060175.815</v>
+        <v>-2049092.37136</v>
       </c>
       <c r="F36" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
-        <v>-1472875.165</v>
+        <v>-2511968.85256</v>
       </c>
     </row>
   </sheetData>
@@ -2027,7 +2151,7 @@
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">'Сценарій A'!$B$37</f>
-        <v>9163150</v>
+        <v>9282000</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -2038,7 +2162,7 @@
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">'Сценарій A'!$B$56</f>
-        <v>-987342.1875</v>
+        <v>-2033632.29016</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -2049,7 +2173,7 @@
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">'Сценарій A'!$B$57</f>
-        <v>-0.107751394171218</v>
+        <v>-0.219094192001724</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -2256,7 +2380,7 @@
       </c>
       <c r="B27" s="13" t="n">
         <f aca="false">'Сценарій A'!$B$64*$B$26</f>
-        <v>275820.6</v>
+        <v>318459.18496</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -2330,7 +2454,7 @@
       </c>
       <c r="B35" s="13" t="n">
         <f aca="false">'Сценарій A'!$B$48*$B$34</f>
-        <v>57269.6875</v>
+        <v>58012.5</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -2460,7 +2584,7 @@
       </c>
       <c r="B48" s="13" t="n">
         <f aca="false">$B$14+$B$23+$B$27+$B$31+$B$35</f>
-        <v>642488.001785714</v>
+        <v>685869.399245714</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -2471,7 +2595,7 @@
       </c>
       <c r="B49" s="13" t="n">
         <f aca="false">$B$6+$B$48</f>
-        <v>-344854.185714286</v>
+        <v>-1347762.89091429</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
@@ -2482,7 +2606,7 @@
       </c>
       <c r="B50" s="10" t="n">
         <f aca="false">$B$5+$B$13+$B$22</f>
-        <v>9906007.14285714</v>
+        <v>10024857.1428571</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
@@ -2493,7 +2617,7 @@
       </c>
       <c r="B51" s="15" t="n">
         <f aca="false">IF($B$50&lt;&gt;0,$B$49/$B$50,0)</f>
-        <v>-0.0348126324502953</v>
+        <v>-0.134442104431841</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
@@ -2504,7 +2628,7 @@
       </c>
       <c r="B52" s="13" t="n">
         <f aca="false">MAX(0,Припущення!$B$43*$B$50-$B$49)</f>
-        <v>2326055.61428572</v>
+        <v>3352734.31948571</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
@@ -2640,11 +2764,12 @@
         <v>Так</v>
       </c>
       <c r="H5" s="23" t="n">
-        <v>4880</v>
+        <f aca="false">340000/B5</f>
+        <v>5528.45528455285</v>
       </c>
       <c r="I5" s="10" t="n">
         <f aca="false">B5*H5</f>
-        <v>300120</v>
+        <v>340000</v>
       </c>
       <c r="J5" s="28" t="n">
         <v>340</v>
@@ -2677,11 +2802,12 @@
         <v>Так</v>
       </c>
       <c r="H6" s="23" t="n">
-        <v>4650</v>
+        <f aca="false">390000/B6</f>
+        <v>5492.95774647887</v>
       </c>
       <c r="I6" s="10" t="n">
         <f aca="false">B6*H6</f>
-        <v>330150</v>
+        <v>390000</v>
       </c>
       <c r="J6" s="28" t="n">
         <v>370</v>
@@ -2714,11 +2840,12 @@
         <v>Так</v>
       </c>
       <c r="H7" s="23" t="n">
-        <v>4640</v>
+        <f aca="false">550000/B7</f>
+        <v>3928.57142857143</v>
       </c>
       <c r="I7" s="10" t="n">
         <f aca="false">B7*H7</f>
-        <v>649600</v>
+        <v>550000</v>
       </c>
       <c r="J7" s="28" t="n">
         <v>560</v>
@@ -2963,7 +3090,7 @@
         <v>116</v>
       </c>
       <c r="B21" s="28" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C21" s="5" t="s">
         <v>117</v>
@@ -3011,8 +3138,9 @@
       <c r="A24" s="5" t="s">
         <v>120</v>
       </c>
-      <c r="B24" s="23" t="n">
-        <v>2400</v>
+      <c r="B24" s="31" t="n">
+        <f aca="false">'Собівартість будинку'!$E$27</f>
+        <v>2783.18187702265</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>121</v>
@@ -3033,7 +3161,7 @@
         <v>123</v>
       </c>
       <c r="B25" s="26" t="n">
-        <v>3000</v>
+        <v>2800</v>
       </c>
       <c r="C25" s="5" t="s">
         <v>121</v>
@@ -3573,11 +3701,13 @@
   <sheetPr filterMode="false">
     <pageSetUpPr fitToPage="false"/>
   </sheetPr>
-  <dimension ref="A1:F66"/>
+  <dimension ref="A1:F28"/>
   <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
   <cols>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
-    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="18"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="56"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="2" min="2" style="0" width="14"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="5" min="3" style="0" width="16"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="6" style="0" width="46"/>
   </cols>
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3590,15 +3720,15 @@
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
     </row>
-    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A2" s="3" t="s">
+    <row r="2" customFormat="false" ht="45" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A2" s="20" t="s">
         <v>175</v>
       </c>
-      <c r="B2" s="3"/>
-      <c r="C2" s="3"/>
-      <c r="D2" s="3"/>
-      <c r="E2" s="3"/>
-      <c r="F2" s="3"/>
+      <c r="B2" s="20"/>
+      <c r="C2" s="20"/>
+      <c r="D2" s="20"/>
+      <c r="E2" s="20"/>
+      <c r="F2" s="20"/>
     </row>
     <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A3" s="2"/>
@@ -3608,846 +3738,433 @@
       <c r="E3" s="2"/>
       <c r="F3" s="2"/>
     </row>
-    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+    <row r="4" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A4" s="4" t="s">
-        <v>78</v>
+        <v>176</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>176</v>
+        <v>177</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>177</v>
+        <v>178</v>
       </c>
       <c r="D4" s="4" t="s">
-        <v>86</v>
+        <v>91</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>178</v>
+        <v>93</v>
       </c>
       <c r="F4" s="4" t="s">
         <v>179</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="str">
-        <f aca="false">Припущення!$A$5</f>
-        <v>Lake House Compact 61</v>
-      </c>
-      <c r="B5" s="28" t="n">
-        <v>9</v>
-      </c>
+      <c r="A5" s="2" t="s">
+        <v>79</v>
+      </c>
+      <c r="B5" s="2"/>
       <c r="C5" s="32" t="n">
-        <f aca="false">B5*Припущення!$B$5</f>
-        <v>553.5</v>
-      </c>
-      <c r="D5" s="9" t="n">
-        <f aca="false">Припущення!$I$5</f>
-        <v>300120</v>
-      </c>
-      <c r="E5" s="10" t="n">
-        <f aca="false">B5*D5</f>
-        <v>2701080</v>
-      </c>
-      <c r="F5" s="7" t="n">
-        <f aca="false">B5*Припущення!$J$5</f>
-        <v>3060</v>
-      </c>
+        <f aca="false">Припущення!$B$5</f>
+        <v>61.5</v>
+      </c>
+      <c r="D5" s="32" t="n">
+        <f aca="false">Припущення!$B$6</f>
+        <v>71</v>
+      </c>
+      <c r="E5" s="32" t="n">
+        <f aca="false">Припущення!$B$7</f>
+        <v>140</v>
+      </c>
+      <c r="F5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="str">
-        <f aca="false">Припущення!$A$6</f>
-        <v>Meadow 71</v>
-      </c>
-      <c r="B6" s="28" t="n">
-        <v>9</v>
-      </c>
-      <c r="C6" s="32" t="n">
-        <f aca="false">B6*Припущення!$B$6</f>
-        <v>639</v>
-      </c>
-      <c r="D6" s="9" t="n">
-        <f aca="false">Припущення!$I$6</f>
-        <v>330150</v>
-      </c>
-      <c r="E6" s="10" t="n">
-        <f aca="false">B6*D6</f>
-        <v>2971350</v>
-      </c>
-      <c r="F6" s="7" t="n">
-        <f aca="false">B6*Припущення!$J$6</f>
-        <v>3330</v>
-      </c>
+      <c r="A6" s="2" t="s">
+        <v>180</v>
+      </c>
+      <c r="B6" s="2"/>
+      <c r="C6" s="6" t="n">
+        <f aca="false">'Сценарій A'!$B$5</f>
+        <v>10</v>
+      </c>
+      <c r="D6" s="6" t="n">
+        <f aca="false">'Сценарій A'!$B$6</f>
+        <v>8</v>
+      </c>
+      <c r="E6" s="6" t="n">
+        <f aca="false">'Сценарій A'!$B$7</f>
+        <v>7</v>
+      </c>
+      <c r="F6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="31" t="str">
-        <f aca="false">Припущення!$A$7</f>
-        <v>Country 140</v>
-      </c>
-      <c r="B7" s="28" t="n">
-        <v>7</v>
-      </c>
-      <c r="C7" s="32" t="n">
-        <f aca="false">B7*Припущення!$B$7</f>
-        <v>980</v>
-      </c>
-      <c r="D7" s="9" t="n">
-        <f aca="false">Припущення!$I$7</f>
-        <v>649600</v>
-      </c>
-      <c r="E7" s="10" t="n">
-        <f aca="false">B7*D7</f>
-        <v>4547200</v>
-      </c>
-      <c r="F7" s="7" t="n">
-        <f aca="false">B7*Припущення!$J$7</f>
-        <v>3920</v>
-      </c>
+      <c r="A7" s="21" t="s">
+        <v>181</v>
+      </c>
+      <c r="B7" s="22"/>
+      <c r="C7" s="22"/>
+      <c r="D7" s="22"/>
+      <c r="E7" s="22"/>
+      <c r="F7" s="22"/>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A8" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="B8" s="33" t="n">
-        <f aca="false">SUM(B5:B7)</f>
-        <v>25</v>
-      </c>
-      <c r="C8" s="34" t="n">
-        <f aca="false">SUM(C5:C7)</f>
-        <v>2172.5</v>
-      </c>
-      <c r="D8" s="35"/>
-      <c r="E8" s="13" t="n">
-        <f aca="false">SUM(E5:E7)</f>
-        <v>10219630</v>
-      </c>
-      <c r="F8" s="33" t="n">
-        <f aca="false">SUM(F5:F7)</f>
-        <v>10310</v>
+      <c r="A8" s="5" t="s">
+        <v>182</v>
+      </c>
+      <c r="B8" s="26" t="n">
+        <v>1700</v>
+      </c>
+      <c r="C8" s="33" t="n">
+        <f aca="false">$B8*C$5</f>
+        <v>104550</v>
+      </c>
+      <c r="D8" s="33" t="n">
+        <f aca="false">$B8*D$5</f>
+        <v>120700</v>
+      </c>
+      <c r="E8" s="33" t="n">
+        <f aca="false">$B8*E$5</f>
+        <v>238000</v>
+      </c>
+      <c r="F8" s="24" t="s">
+        <v>183</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A9" s="2"/>
-      <c r="B9" s="2"/>
-      <c r="C9" s="2"/>
-      <c r="D9" s="2"/>
-      <c r="E9" s="2"/>
-      <c r="F9" s="2"/>
+      <c r="A9" s="5" t="s">
+        <v>184</v>
+      </c>
+      <c r="B9" s="26" t="n">
+        <v>160</v>
+      </c>
+      <c r="C9" s="33" t="n">
+        <f aca="false">$B9*C$5</f>
+        <v>9840</v>
+      </c>
+      <c r="D9" s="33" t="n">
+        <f aca="false">$B9*D$5</f>
+        <v>11360</v>
+      </c>
+      <c r="E9" s="33" t="n">
+        <f aca="false">$B9*E$5</f>
+        <v>22400</v>
+      </c>
+      <c r="F9" s="24" t="s">
+        <v>185</v>
+      </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A10" s="21" t="s">
-        <v>181</v>
-      </c>
-      <c r="B10" s="22"/>
-      <c r="C10" s="22"/>
-      <c r="D10" s="22"/>
-      <c r="E10" s="22"/>
-      <c r="F10" s="22"/>
+      <c r="A10" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="B10" s="26" t="n">
+        <v>120</v>
+      </c>
+      <c r="C10" s="33" t="n">
+        <f aca="false">$B10*C$5</f>
+        <v>7380</v>
+      </c>
+      <c r="D10" s="33" t="n">
+        <f aca="false">$B10*D$5</f>
+        <v>8520</v>
+      </c>
+      <c r="E10" s="33" t="n">
+        <f aca="false">$B10*E$5</f>
+        <v>16800</v>
+      </c>
+      <c r="F10" s="24" t="s">
+        <v>187</v>
+      </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>182</v>
-      </c>
-      <c r="B11" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C11" s="2"/>
-      <c r="D11" s="2"/>
-      <c r="E11" s="2"/>
-      <c r="F11" s="2"/>
+        <v>188</v>
+      </c>
+      <c r="B11" s="26" t="n">
+        <v>60</v>
+      </c>
+      <c r="C11" s="33" t="n">
+        <f aca="false">$B11*C$5</f>
+        <v>3690</v>
+      </c>
+      <c r="D11" s="33" t="n">
+        <f aca="false">$B11*D$5</f>
+        <v>4260</v>
+      </c>
+      <c r="E11" s="33" t="n">
+        <f aca="false">$B11*E$5</f>
+        <v>8400</v>
+      </c>
+      <c r="F11" s="24" t="s">
+        <v>189</v>
+      </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>183</v>
-      </c>
-      <c r="B12" s="25" t="n">
-        <v>0.85</v>
-      </c>
-      <c r="C12" s="24" t="s">
-        <v>184</v>
-      </c>
-      <c r="D12" s="2"/>
-      <c r="E12" s="2"/>
-      <c r="F12" s="2"/>
+        <v>190</v>
+      </c>
+      <c r="B12" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C12" s="26" t="n">
+        <v>6500</v>
+      </c>
+      <c r="D12" s="26" t="n">
+        <v>6500</v>
+      </c>
+      <c r="E12" s="26" t="n">
+        <v>8500</v>
+      </c>
+      <c r="F12" s="24" t="s">
+        <v>192</v>
+      </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>185</v>
-      </c>
-      <c r="B13" s="28" t="n">
-        <v>0</v>
-      </c>
-      <c r="C13" s="24" t="s">
-        <v>186</v>
-      </c>
-      <c r="D13" s="2"/>
-      <c r="E13" s="2"/>
-      <c r="F13" s="2"/>
+        <v>193</v>
+      </c>
+      <c r="B13" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C13" s="26" t="n">
+        <v>2000</v>
+      </c>
+      <c r="D13" s="26" t="n">
+        <v>2000</v>
+      </c>
+      <c r="E13" s="26" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F13" s="24" t="s">
+        <v>194</v>
+      </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>187</v>
-      </c>
-      <c r="B14" s="26" t="n">
-        <v>100000</v>
-      </c>
-      <c r="C14" s="24" t="s">
-        <v>188</v>
-      </c>
-      <c r="D14" s="2"/>
-      <c r="E14" s="2"/>
-      <c r="F14" s="2"/>
+        <v>195</v>
+      </c>
+      <c r="B14" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C14" s="26" t="n">
+        <v>9000</v>
+      </c>
+      <c r="D14" s="26" t="n">
+        <v>10000</v>
+      </c>
+      <c r="E14" s="26" t="n">
+        <v>15000</v>
+      </c>
+      <c r="F14" s="24" t="s">
+        <v>196</v>
+      </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>189</v>
-      </c>
-      <c r="B15" s="7" t="n">
-        <f aca="false">B8+$B$11*Припущення!$B$50</f>
-        <v>25</v>
-      </c>
-      <c r="C15" s="24" t="s">
-        <v>190</v>
-      </c>
-      <c r="D15" s="2"/>
-      <c r="E15" s="2"/>
-      <c r="F15" s="2"/>
+        <v>197</v>
+      </c>
+      <c r="B15" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C15" s="26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D15" s="26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E15" s="26" t="n">
+        <v>12000</v>
+      </c>
+      <c r="F15" s="24" t="s">
+        <v>198</v>
+      </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A16" s="2"/>
-      <c r="B16" s="2"/>
-      <c r="C16" s="2"/>
-      <c r="D16" s="2"/>
-      <c r="E16" s="2"/>
-      <c r="F16" s="2"/>
+      <c r="A16" s="5" t="s">
+        <v>199</v>
+      </c>
+      <c r="B16" s="5" t="s">
+        <v>191</v>
+      </c>
+      <c r="C16" s="26" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D16" s="26" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E16" s="26" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F16" s="24" t="s">
+        <v>200</v>
+      </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A17" s="21" t="s">
+      <c r="A17" s="5" t="s">
+        <v>201</v>
+      </c>
+      <c r="B17" s="5" t="s">
         <v>191</v>
       </c>
-      <c r="B17" s="22"/>
-      <c r="C17" s="22"/>
-      <c r="D17" s="22"/>
-      <c r="E17" s="22"/>
-      <c r="F17" s="22"/>
+      <c r="C17" s="26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D17" s="26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E17" s="26" t="n">
+        <v>9000</v>
+      </c>
+      <c r="F17" s="24" t="s">
+        <v>202</v>
+      </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="5" t="s">
-        <v>192</v>
-      </c>
-      <c r="B18" s="7" t="n">
-        <f aca="false">F8</f>
-        <v>10310</v>
-      </c>
-      <c r="C18" s="2"/>
-      <c r="D18" s="2"/>
-      <c r="E18" s="2"/>
+      <c r="A18" s="11" t="s">
+        <v>203</v>
+      </c>
+      <c r="B18" s="2"/>
+      <c r="C18" s="13" t="n">
+        <f aca="false">SUM(C8:C17)</f>
+        <v>158460</v>
+      </c>
+      <c r="D18" s="13" t="n">
+        <f aca="false">SUM(D8:D17)</f>
+        <v>178840</v>
+      </c>
+      <c r="E18" s="13" t="n">
+        <f aca="false">SUM(E8:E17)</f>
+        <v>337100</v>
+      </c>
       <c r="F18" s="2"/>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>193</v>
-      </c>
-      <c r="B19" s="6" t="n">
-        <f aca="false">Припущення!$B$12*Припущення!$B$13</f>
-        <v>2564.1</v>
-      </c>
-      <c r="C19" s="2"/>
-      <c r="D19" s="2"/>
-      <c r="E19" s="2"/>
-      <c r="F19" s="2"/>
+        <v>204</v>
+      </c>
+      <c r="B19" s="27" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C19" s="33" t="n">
+        <f aca="false">C18*$B19</f>
+        <v>19015.2</v>
+      </c>
+      <c r="D19" s="33" t="n">
+        <f aca="false">D18*$B19</f>
+        <v>21460.8</v>
+      </c>
+      <c r="E19" s="33" t="n">
+        <f aca="false">E18*$B19</f>
+        <v>40452</v>
+      </c>
+      <c r="F19" s="24" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A20" s="5" t="s">
-        <v>194</v>
-      </c>
-      <c r="B20" s="6" t="n">
-        <f aca="false">Припущення!$B$12*Припущення!$B$14</f>
-        <v>997.15</v>
-      </c>
-      <c r="C20" s="2"/>
-      <c r="D20" s="2"/>
-      <c r="E20" s="2"/>
+      <c r="A20" s="11" t="s">
+        <v>206</v>
+      </c>
+      <c r="B20" s="2"/>
+      <c r="C20" s="13" t="n">
+        <f aca="false">C18+C19</f>
+        <v>177475.2</v>
+      </c>
+      <c r="D20" s="13" t="n">
+        <f aca="false">D18+D19</f>
+        <v>200300.8</v>
+      </c>
+      <c r="E20" s="13" t="n">
+        <f aca="false">E18+E19</f>
+        <v>377552</v>
+      </c>
       <c r="F20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="5" t="s">
-        <v>195</v>
-      </c>
-      <c r="B21" s="6" t="n">
-        <f aca="false">Припущення!$B$12*Припущення!$B$15</f>
-        <v>854.7</v>
-      </c>
-      <c r="C21" s="2"/>
-      <c r="D21" s="2"/>
-      <c r="E21" s="2"/>
+      <c r="A21" s="11" t="s">
+        <v>207</v>
+      </c>
+      <c r="B21" s="2"/>
+      <c r="C21" s="13" t="n">
+        <f aca="false">IF(C5&gt;0,C20/C5,0)</f>
+        <v>2885.7756097561</v>
+      </c>
+      <c r="D21" s="13" t="n">
+        <f aca="false">IF(D5&gt;0,D20/D5,0)</f>
+        <v>2821.13802816901</v>
+      </c>
+      <c r="E21" s="13" t="n">
+        <f aca="false">IF(E5&gt;0,E20/E5,0)</f>
+        <v>2696.8</v>
+      </c>
       <c r="F21" s="2"/>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="5" t="s">
-        <v>196</v>
-      </c>
-      <c r="B22" s="7" t="n">
-        <f aca="false">$B$11*Припущення!$B$16</f>
-        <v>0</v>
-      </c>
+      <c r="A22" s="2"/>
+      <c r="B22" s="2"/>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
       <c r="E22" s="2"/>
       <c r="F22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="11" t="s">
-        <v>197</v>
-      </c>
-      <c r="B23" s="33" t="n">
-        <f aca="false">SUM($B$18:$B$22)</f>
-        <v>14725.95</v>
-      </c>
+      <c r="A23" s="2"/>
+      <c r="B23" s="2"/>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
       <c r="E23" s="2"/>
       <c r="F23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A24" s="5" t="s">
-        <v>198</v>
-      </c>
-      <c r="B24" s="6" t="n">
-        <f aca="false">Припущення!$B$12</f>
-        <v>14245</v>
-      </c>
+      <c r="A24" s="2"/>
+      <c r="B24" s="2"/>
       <c r="C24" s="2"/>
       <c r="D24" s="2"/>
       <c r="E24" s="2"/>
       <c r="F24" s="2"/>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A25" s="11" t="s">
-        <v>199</v>
-      </c>
-      <c r="B25" s="33" t="n">
-        <f aca="false">$B$24-$B$23</f>
-        <v>-480.950000000001</v>
-      </c>
+      <c r="A25" s="2"/>
+      <c r="B25" s="2"/>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
       <c r="E25" s="2"/>
       <c r="F25" s="2"/>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A26" s="11" t="s">
-        <v>200</v>
-      </c>
-      <c r="B26" s="36" t="str">
-        <f aca="false">IF($B$25&gt;=0,"Вміщується","НЕ ВМІЩУЄТЬСЯ")</f>
-        <v>НЕ ВМІЩУЄТЬСЯ</v>
-      </c>
+      <c r="A26" s="2"/>
+      <c r="B26" s="2"/>
       <c r="C26" s="2"/>
       <c r="D26" s="2"/>
       <c r="E26" s="2"/>
       <c r="F26" s="2"/>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A27" s="5" t="s">
-        <v>9</v>
-      </c>
-      <c r="B27" s="7" t="n">
-        <f aca="false">IF(B8&gt;0,F8/B8,0)</f>
-        <v>412.4</v>
-      </c>
+      <c r="A27" s="11" t="s">
+        <v>208</v>
+      </c>
+      <c r="B27" s="2"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
-      <c r="E27" s="2"/>
+      <c r="E27" s="34" t="n">
+        <f aca="false">SUMPRODUCT(C20:E20,C6:E6)/SUMPRODUCT(C5:E5,C6:E6)</f>
+        <v>2783.18187702265</v>
+      </c>
       <c r="F27" s="2"/>
     </row>
-    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A28" s="2"/>
-      <c r="B28" s="2"/>
-      <c r="C28" s="2"/>
-      <c r="D28" s="2"/>
-      <c r="E28" s="2"/>
-      <c r="F28" s="2"/>
-    </row>
-    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A29" s="21" t="s">
-        <v>201</v>
-      </c>
-      <c r="B29" s="22"/>
-      <c r="C29" s="22"/>
-      <c r="D29" s="22"/>
-      <c r="E29" s="22"/>
-      <c r="F29" s="22"/>
-    </row>
-    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A30" s="5" t="s">
-        <v>202</v>
-      </c>
-      <c r="B30" s="10" t="n">
-        <f aca="false">E8</f>
-        <v>10219630</v>
-      </c>
-      <c r="C30" s="2"/>
-      <c r="D30" s="2"/>
-      <c r="E30" s="2"/>
-      <c r="F30" s="2"/>
-    </row>
-    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A31" s="5" t="s">
-        <v>203</v>
-      </c>
-      <c r="B31" s="7" t="n">
-        <f aca="false">ROUNDUP($B$15*Припущення!$B$19,0)</f>
-        <v>8</v>
-      </c>
-      <c r="C31" s="24" t="s">
-        <v>204</v>
-      </c>
-      <c r="D31" s="2"/>
-      <c r="E31" s="2"/>
-      <c r="F31" s="2"/>
-    </row>
-    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A32" s="5" t="s">
-        <v>205</v>
-      </c>
-      <c r="B32" s="7" t="n">
-        <f aca="false">MIN($B$31,INDEX(B5:B7,Припущення!$B$21))</f>
-        <v>8</v>
-      </c>
-      <c r="C32" s="2"/>
-      <c r="D32" s="2"/>
-      <c r="E32" s="2"/>
-      <c r="F32" s="2"/>
-    </row>
-    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A33" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="B33" s="37" t="str">
-        <f aca="false">IF($B$32&lt;$B$31,"Обраного типу замало — потрібні інші типи","OK")</f>
-        <v>OK</v>
-      </c>
-      <c r="C33" s="2"/>
-      <c r="D33" s="2"/>
-      <c r="E33" s="2"/>
-      <c r="F33" s="2"/>
-    </row>
-    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A34" s="5" t="s">
-        <v>207</v>
-      </c>
-      <c r="B34" s="10" t="n">
-        <f aca="false">-$B$31*INDEX(D5:D7,Припущення!$B$21)*(1-Припущення!$B$20)</f>
-        <v>-1056480</v>
-      </c>
-      <c r="C34" s="24" t="s">
-        <v>208</v>
-      </c>
-      <c r="D34" s="2"/>
-      <c r="E34" s="2"/>
-      <c r="F34" s="2"/>
-    </row>
-    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A35" s="5" t="s">
+    <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A28" s="20" t="s">
         <v>209</v>
       </c>
-      <c r="B35" s="10" t="n">
-        <f aca="false">$B$11*Припущення!$B$47*Припущення!$B$48/Припущення!$B$49</f>
-        <v>0</v>
-      </c>
-      <c r="C35" s="2"/>
-      <c r="D35" s="2"/>
-      <c r="E35" s="2"/>
-      <c r="F35" s="2"/>
-    </row>
-    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="5" t="s">
-        <v>210</v>
-      </c>
-      <c r="B36" s="10" t="n">
-        <f aca="false">$B$11*Припущення!$B$50*Припущення!$B$51</f>
-        <v>0</v>
-      </c>
-      <c r="C36" s="2"/>
-      <c r="D36" s="2"/>
-      <c r="E36" s="2"/>
-      <c r="F36" s="2"/>
-    </row>
-    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A37" s="11" t="s">
-        <v>211</v>
-      </c>
-      <c r="B37" s="13" t="n">
-        <f aca="false">SUM($B$30,$B$34,$B$35,$B$36)</f>
-        <v>9163150</v>
-      </c>
-      <c r="C37" s="2"/>
-      <c r="D37" s="2"/>
-      <c r="E37" s="2"/>
-      <c r="F37" s="2"/>
-    </row>
-    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A38" s="2"/>
-      <c r="B38" s="2"/>
-      <c r="C38" s="2"/>
-      <c r="D38" s="2"/>
-      <c r="E38" s="2"/>
-      <c r="F38" s="2"/>
-    </row>
-    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A39" s="21" t="s">
-        <v>212</v>
-      </c>
-      <c r="B39" s="22"/>
-      <c r="C39" s="22"/>
-      <c r="D39" s="22"/>
-      <c r="E39" s="22"/>
-      <c r="F39" s="22"/>
-    </row>
-    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A40" s="5" t="s">
-        <v>120</v>
-      </c>
-      <c r="B40" s="10" t="n">
-        <f aca="false">C8*Припущення!$B$24</f>
-        <v>5214000</v>
-      </c>
-      <c r="C40" s="2"/>
-      <c r="D40" s="2"/>
-      <c r="E40" s="2"/>
-      <c r="F40" s="2"/>
-    </row>
-    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A41" s="5" t="s">
-        <v>213</v>
-      </c>
-      <c r="B41" s="10" t="n">
-        <f aca="false">$B$11*Припущення!$B$46*Припущення!$B$25</f>
-        <v>0</v>
-      </c>
-      <c r="C41" s="2"/>
-      <c r="D41" s="2"/>
-      <c r="E41" s="2"/>
-      <c r="F41" s="2"/>
-    </row>
-    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A42" s="5" t="s">
-        <v>125</v>
-      </c>
-      <c r="B42" s="10" t="n">
-        <f aca="false">($B$40+$B$41)*Припущення!$B$26</f>
-        <v>782100</v>
-      </c>
-      <c r="C42" s="2"/>
-      <c r="D42" s="2"/>
-      <c r="E42" s="2"/>
-      <c r="F42" s="2"/>
-    </row>
-    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A43" s="5" t="s">
-        <v>214</v>
-      </c>
-      <c r="B43" s="10" t="n">
-        <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$27</f>
-        <v>299805</v>
-      </c>
-      <c r="C43" s="2"/>
-      <c r="D43" s="2"/>
-      <c r="E43" s="2"/>
-      <c r="F43" s="2"/>
-    </row>
-    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A44" s="5" t="s">
-        <v>131</v>
-      </c>
-      <c r="B44" s="10" t="n">
-        <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$28</f>
-        <v>599610</v>
-      </c>
-      <c r="C44" s="2"/>
-      <c r="D44" s="2"/>
-      <c r="E44" s="2"/>
-      <c r="F44" s="2"/>
-    </row>
-    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A45" s="5" t="s">
-        <v>215</v>
-      </c>
-      <c r="B45" s="10" t="n">
-        <f aca="false">$B$15*Припущення!$B$29</f>
-        <v>375000</v>
-      </c>
-      <c r="C45" s="2"/>
-      <c r="D45" s="2"/>
-      <c r="E45" s="2"/>
-      <c r="F45" s="2"/>
-    </row>
-    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A46" s="5" t="s">
-        <v>216</v>
-      </c>
-      <c r="B46" s="10" t="n">
-        <f aca="false">$B$15*Припущення!$B$30</f>
-        <v>4000</v>
-      </c>
-      <c r="C46" s="2"/>
-      <c r="D46" s="2"/>
-      <c r="E46" s="2"/>
-      <c r="F46" s="2"/>
-    </row>
-    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A47" s="5" t="s">
-        <v>217</v>
-      </c>
-      <c r="B47" s="9" t="n">
-        <f aca="false">Припущення!$B$31</f>
-        <v>50000</v>
-      </c>
-      <c r="C47" s="2"/>
-      <c r="D47" s="2"/>
-      <c r="E47" s="2"/>
-      <c r="F47" s="2"/>
-    </row>
-    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A48" s="5" t="s">
-        <v>140</v>
-      </c>
-      <c r="B48" s="10" t="n">
-        <f aca="false">$B$37*Припущення!$B$34</f>
-        <v>229078.75</v>
-      </c>
-      <c r="C48" s="2"/>
-      <c r="D48" s="2"/>
-      <c r="E48" s="2"/>
-      <c r="F48" s="2"/>
-    </row>
-    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A49" s="5" t="s">
-        <v>218</v>
-      </c>
-      <c r="B49" s="10" t="n">
-        <f aca="false">$B$15*Припущення!$B$35</f>
-        <v>37500</v>
-      </c>
-      <c r="C49" s="2"/>
-      <c r="D49" s="2"/>
-      <c r="E49" s="2"/>
-      <c r="F49" s="2"/>
-    </row>
-    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A50" s="5" t="s">
-        <v>219</v>
-      </c>
-      <c r="B50" s="9" t="n">
-        <f aca="false">Припущення!$B$41</f>
-        <v>1500000</v>
-      </c>
-      <c r="C50" s="2"/>
-      <c r="D50" s="2"/>
-      <c r="E50" s="2"/>
-      <c r="F50" s="2"/>
-    </row>
-    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A51" s="5" t="s">
-        <v>154</v>
-      </c>
-      <c r="B51" s="10" t="n">
-        <f aca="false">$B$50*Припущення!$B$42</f>
-        <v>90000</v>
-      </c>
-      <c r="C51" s="2"/>
-      <c r="D51" s="2"/>
-      <c r="E51" s="2"/>
-      <c r="F51" s="2"/>
-    </row>
-    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A52" s="5" t="s">
-        <v>220</v>
-      </c>
-      <c r="B52" s="10" t="n">
-        <f aca="false">Припущення!$B$36*(Припущення!$B$37*SUM($B$40:$B$49)*Припущення!$B$38/12+($B$50+$B$51)*(Припущення!$B$38+$B$13)/12)</f>
-        <v>969398.4375</v>
-      </c>
-      <c r="C52" s="24" t="s">
-        <v>221</v>
-      </c>
-      <c r="D52" s="2"/>
-      <c r="E52" s="2"/>
-      <c r="F52" s="2"/>
-    </row>
-    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A53" s="11" t="s">
-        <v>222</v>
-      </c>
-      <c r="B53" s="13" t="n">
-        <f aca="false">SUM($B$40:$B$52)</f>
-        <v>10150492.1875</v>
-      </c>
-      <c r="C53" s="2"/>
-      <c r="D53" s="2"/>
-      <c r="E53" s="2"/>
-      <c r="F53" s="2"/>
-    </row>
-    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A54" s="2"/>
-      <c r="B54" s="2"/>
-      <c r="C54" s="2"/>
-      <c r="D54" s="2"/>
-      <c r="E54" s="2"/>
-      <c r="F54" s="2"/>
-    </row>
-    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A55" s="21" t="s">
-        <v>223</v>
-      </c>
-      <c r="B55" s="22"/>
-      <c r="C55" s="22"/>
-      <c r="D55" s="22"/>
-      <c r="E55" s="22"/>
-      <c r="F55" s="22"/>
-    </row>
-    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A56" s="11" t="s">
-        <v>224</v>
-      </c>
-      <c r="B56" s="13" t="n">
-        <f aca="false">$B$37-$B$53</f>
-        <v>-987342.1875</v>
-      </c>
-      <c r="C56" s="2"/>
-      <c r="D56" s="2"/>
-      <c r="E56" s="2"/>
-      <c r="F56" s="2"/>
-    </row>
-    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A57" s="11" t="s">
-        <v>14</v>
-      </c>
-      <c r="B57" s="15" t="n">
-        <f aca="false">IF($B$37&lt;&gt;0,$B$56/$B$37,0)</f>
-        <v>-0.107751394171218</v>
-      </c>
-      <c r="C57" s="2"/>
-      <c r="D57" s="2"/>
-      <c r="E57" s="2"/>
-      <c r="F57" s="2"/>
-    </row>
-    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A58" s="5" t="s">
-        <v>225</v>
-      </c>
-      <c r="B58" s="17" t="n">
-        <f aca="false">IF($B$53&lt;&gt;0,$B$56/$B$53,0)</f>
-        <v>-0.0972703755898536</v>
-      </c>
-      <c r="C58" s="2"/>
-      <c r="D58" s="2"/>
-      <c r="E58" s="2"/>
-      <c r="F58" s="2"/>
-    </row>
-    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A59" s="11" t="s">
-        <v>226</v>
-      </c>
-      <c r="B59" s="36" t="str">
-        <f aca="false">IF($B$57&gt;=Припущення!$B$43,"Досягає цілі","НИЖЧЕ ЦІЛІ")</f>
-        <v>НИЖЧЕ ЦІЛІ</v>
-      </c>
-      <c r="C59" s="2"/>
-      <c r="D59" s="2"/>
-      <c r="E59" s="2"/>
-      <c r="F59" s="2"/>
-    </row>
-    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A60" s="5" t="s">
-        <v>227</v>
-      </c>
-      <c r="B60" s="10" t="n">
-        <f aca="false">($B$37*(1-Припущення!$B$43)-($B$53-$B$50-$B$51-Припущення!$B$36*($B$50+$B$51)*(Припущення!$B$38+$B$13)/12))/(1+Припущення!$B$42+Припущення!$B$36*(1+Припущення!$B$42)*(Припущення!$B$38+$B$13)/12)</f>
-        <v>-754534.847697474</v>
-      </c>
-      <c r="C60" s="24" t="s">
-        <v>228</v>
-      </c>
-      <c r="D60" s="2"/>
-      <c r="E60" s="2"/>
-      <c r="F60" s="2"/>
-    </row>
-    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A61" s="11" t="s">
-        <v>229</v>
-      </c>
-      <c r="B61" s="13" t="n">
-        <f aca="false">$B$12*$B$56-(1-$B$12)*$B$14</f>
-        <v>-854240.859375</v>
-      </c>
-      <c r="C61" s="2"/>
-      <c r="D61" s="2"/>
-      <c r="E61" s="2"/>
-      <c r="F61" s="2"/>
-    </row>
-    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A62" s="2"/>
-      <c r="B62" s="2"/>
-      <c r="C62" s="2"/>
-      <c r="D62" s="2"/>
-      <c r="E62" s="2"/>
-      <c r="F62" s="2"/>
-    </row>
-    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A63" s="21" t="s">
-        <v>230</v>
-      </c>
-      <c r="B63" s="22"/>
-      <c r="C63" s="22"/>
-      <c r="D63" s="22"/>
-      <c r="E63" s="22"/>
-      <c r="F63" s="22"/>
-    </row>
-    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A64" s="5" t="s">
-        <v>231</v>
-      </c>
-      <c r="B64" s="10" t="n">
-        <f aca="false">SUM($B$40:$B$44)</f>
-        <v>6895515</v>
-      </c>
-      <c r="C64" s="2"/>
-      <c r="D64" s="2"/>
-      <c r="E64" s="2"/>
-      <c r="F64" s="2"/>
-    </row>
-    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A65" s="5" t="s">
-        <v>232</v>
-      </c>
-      <c r="B65" s="10" t="n">
-        <f aca="false">$B$53-$B$64-$B$48</f>
-        <v>3025898.4375</v>
-      </c>
-      <c r="C65" s="2"/>
-      <c r="D65" s="2"/>
-      <c r="E65" s="2"/>
-      <c r="F65" s="2"/>
-    </row>
-    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A66" s="5" t="s">
-        <v>233</v>
-      </c>
-      <c r="B66" s="17" t="n">
-        <f aca="false">($B$64+$B$65)/($B$37*(1-Припущення!$B$34-Припущення!$B$43))-1</f>
-        <v>0.397098573124153</v>
-      </c>
-      <c r="C66" s="24" t="s">
-        <v>234</v>
-      </c>
-      <c r="D66" s="2"/>
-      <c r="E66" s="2"/>
-      <c r="F66" s="2"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
+  <mergeCells count="2">
     <mergeCell ref="A2:F2"/>
+    <mergeCell ref="A28:F28"/>
   </mergeCells>
   <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
@@ -4473,7 +4190,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>235</v>
+        <v>210</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4483,7 +4200,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>236</v>
+        <v>211</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4504,40 +4221,40 @@
         <v>78</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>176</v>
+        <v>212</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>177</v>
+        <v>213</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>86</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>178</v>
+        <v>214</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>179</v>
+        <v>215</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A5" s="31" t="str">
+      <c r="A5" s="35" t="str">
         <f aca="false">Припущення!$A$5</f>
         <v>Lake House Compact 61</v>
       </c>
       <c r="B5" s="28" t="n">
         <v>10</v>
       </c>
-      <c r="C5" s="32" t="n">
+      <c r="C5" s="36" t="n">
         <f aca="false">B5*Припущення!$B$5</f>
         <v>615</v>
       </c>
       <c r="D5" s="9" t="n">
         <f aca="false">Припущення!$I$5</f>
-        <v>300120</v>
+        <v>340000</v>
       </c>
       <c r="E5" s="10" t="n">
         <f aca="false">B5*D5</f>
-        <v>3001200</v>
+        <v>3400000</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">B5*Припущення!$J$5</f>
@@ -4545,24 +4262,24 @@
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A6" s="31" t="str">
+      <c r="A6" s="35" t="str">
         <f aca="false">Припущення!$A$6</f>
         <v>Meadow 71</v>
       </c>
       <c r="B6" s="28" t="n">
         <v>8</v>
       </c>
-      <c r="C6" s="32" t="n">
+      <c r="C6" s="36" t="n">
         <f aca="false">B6*Припущення!$B$6</f>
         <v>568</v>
       </c>
       <c r="D6" s="9" t="n">
         <f aca="false">Припущення!$I$6</f>
-        <v>330150</v>
+        <v>390000</v>
       </c>
       <c r="E6" s="10" t="n">
         <f aca="false">B6*D6</f>
-        <v>2641200</v>
+        <v>3120000</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">B6*Припущення!$J$6</f>
@@ -4570,24 +4287,24 @@
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A7" s="31" t="str">
+      <c r="A7" s="35" t="str">
         <f aca="false">Припущення!$A$7</f>
         <v>Country 140</v>
       </c>
       <c r="B7" s="28" t="n">
         <v>7</v>
       </c>
-      <c r="C7" s="32" t="n">
+      <c r="C7" s="36" t="n">
         <f aca="false">B7*Припущення!$B$7</f>
         <v>980</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">Припущення!$I$7</f>
-        <v>649600</v>
+        <v>550000</v>
       </c>
       <c r="E7" s="10" t="n">
         <f aca="false">B7*D7</f>
-        <v>4547200</v>
+        <v>3850000</v>
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">B7*Припущення!$J$7</f>
@@ -4596,22 +4313,22 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>180</v>
-      </c>
-      <c r="B8" s="33" t="n">
+        <v>216</v>
+      </c>
+      <c r="B8" s="37" t="n">
         <f aca="false">SUM(B5:B7)</f>
         <v>25</v>
       </c>
-      <c r="C8" s="34" t="n">
+      <c r="C8" s="38" t="n">
         <f aca="false">SUM(C5:C7)</f>
         <v>2163</v>
       </c>
-      <c r="D8" s="35"/>
+      <c r="D8" s="33"/>
       <c r="E8" s="13" t="n">
         <f aca="false">SUM(E5:E7)</f>
-        <v>10189600</v>
-      </c>
-      <c r="F8" s="33" t="n">
+        <v>10370000</v>
+      </c>
+      <c r="F8" s="37" t="n">
         <f aca="false">SUM(F5:F7)</f>
         <v>10280</v>
       </c>
@@ -4626,7 +4343,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>181</v>
+        <v>217</v>
       </c>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -4636,10 +4353,10 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>182</v>
+        <v>218</v>
       </c>
       <c r="B11" s="28" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="C11" s="2"/>
       <c r="D11" s="2"/>
@@ -4648,13 +4365,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>183</v>
+        <v>219</v>
       </c>
       <c r="B12" s="25" t="n">
-        <v>0.45</v>
+        <v>0.85</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>184</v>
+        <v>220</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -4662,13 +4379,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>185</v>
+        <v>221</v>
       </c>
       <c r="B13" s="28" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>186</v>
+        <v>222</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -4676,13 +4393,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>187</v>
+        <v>223</v>
       </c>
       <c r="B14" s="26" t="n">
-        <v>250000</v>
+        <v>100000</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>188</v>
+        <v>224</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -4690,14 +4407,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>189</v>
+        <v>225</v>
       </c>
       <c r="B15" s="7" t="n">
         <f aca="false">B8+$B$11*Припущення!$B$50</f>
-        <v>29</v>
+        <v>25</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>190</v>
+        <v>226</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
@@ -4713,7 +4430,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>191</v>
+        <v>227</v>
       </c>
       <c r="B17" s="22"/>
       <c r="C17" s="22"/>
@@ -4723,7 +4440,7 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>192</v>
+        <v>228</v>
       </c>
       <c r="B18" s="7" t="n">
         <f aca="false">F8</f>
@@ -4736,7 +4453,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>193</v>
+        <v>229</v>
       </c>
       <c r="B19" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$13</f>
@@ -4749,7 +4466,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>194</v>
+        <v>230</v>
       </c>
       <c r="B20" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$14</f>
@@ -4762,7 +4479,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>195</v>
+        <v>231</v>
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$15</f>
@@ -4775,11 +4492,11 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>196</v>
+        <v>232</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">$B$11*Припущення!$B$16</f>
-        <v>900</v>
+        <v>0</v>
       </c>
       <c r="C22" s="2"/>
       <c r="D22" s="2"/>
@@ -4788,11 +4505,11 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>197</v>
-      </c>
-      <c r="B23" s="33" t="n">
+        <v>233</v>
+      </c>
+      <c r="B23" s="37" t="n">
         <f aca="false">SUM($B$18:$B$22)</f>
-        <v>15595.95</v>
+        <v>14695.95</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -4801,7 +4518,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>198</v>
+        <v>234</v>
       </c>
       <c r="B24" s="6" t="n">
         <f aca="false">Припущення!$B$12</f>
@@ -4814,11 +4531,11 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>199</v>
-      </c>
-      <c r="B25" s="33" t="n">
+        <v>235</v>
+      </c>
+      <c r="B25" s="37" t="n">
         <f aca="false">$B$24-$B$23</f>
-        <v>-1350.95</v>
+        <v>-450.950000000001</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -4827,9 +4544,9 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>200</v>
-      </c>
-      <c r="B26" s="36" t="str">
+        <v>236</v>
+      </c>
+      <c r="B26" s="39" t="str">
         <f aca="false">IF($B$25&gt;=0,"Вміщується","НЕ ВМІЩУЄТЬСЯ")</f>
         <v>НЕ ВМІЩУЄТЬСЯ</v>
       </c>
@@ -4861,7 +4578,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>201</v>
+        <v>237</v>
       </c>
       <c r="B29" s="22"/>
       <c r="C29" s="22"/>
@@ -4871,11 +4588,11 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>202</v>
+        <v>238</v>
       </c>
       <c r="B30" s="10" t="n">
         <f aca="false">E8</f>
-        <v>10189600</v>
+        <v>10370000</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -4884,14 +4601,14 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>203</v>
+        <v>239</v>
       </c>
       <c r="B31" s="7" t="n">
         <f aca="false">ROUNDUP($B$15*Припущення!$B$19,0)</f>
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="C31" s="24" t="s">
-        <v>204</v>
+        <v>240</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
@@ -4899,7 +4616,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>205</v>
+        <v>241</v>
       </c>
       <c r="B32" s="7" t="n">
         <f aca="false">MIN($B$31,INDEX(B5:B7,Припущення!$B$21))</f>
@@ -4912,11 +4629,11 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>206</v>
-      </c>
-      <c r="B33" s="37" t="str">
+        <v>242</v>
+      </c>
+      <c r="B33" s="40" t="str">
         <f aca="false">IF($B$32&lt;$B$31,"Обраного типу замало — потрібні інші типи","OK")</f>
-        <v>Обраного типу замало — потрібні інші типи</v>
+        <v>OK</v>
       </c>
       <c r="C33" s="2"/>
       <c r="D33" s="2"/>
@@ -4925,14 +4642,14 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>207</v>
+        <v>243</v>
       </c>
       <c r="B34" s="10" t="n">
         <f aca="false">-$B$31*INDEX(D5:D7,Припущення!$B$21)*(1-Припущення!$B$20)</f>
-        <v>-1188540</v>
+        <v>-1088000</v>
       </c>
       <c r="C34" s="24" t="s">
-        <v>208</v>
+        <v>244</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
@@ -4940,11 +4657,11 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>209</v>
+        <v>245</v>
       </c>
       <c r="B35" s="10" t="n">
         <f aca="false">$B$11*Припущення!$B$47*Припущення!$B$48/Припущення!$B$49</f>
-        <v>350000</v>
+        <v>0</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -4953,11 +4670,11 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>210</v>
+        <v>246</v>
       </c>
       <c r="B36" s="10" t="n">
         <f aca="false">$B$11*Припущення!$B$50*Припущення!$B$51</f>
-        <v>880000</v>
+        <v>0</v>
       </c>
       <c r="C36" s="2"/>
       <c r="D36" s="2"/>
@@ -4966,11 +4683,11 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>211</v>
+        <v>247</v>
       </c>
       <c r="B37" s="13" t="n">
         <f aca="false">SUM($B$30,$B$34,$B$35,$B$36)</f>
-        <v>10231060</v>
+        <v>9282000</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -4987,7 +4704,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="21" t="s">
-        <v>212</v>
+        <v>248</v>
       </c>
       <c r="B39" s="22"/>
       <c r="C39" s="22"/>
@@ -4997,11 +4714,11 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>120</v>
+        <v>249</v>
       </c>
       <c r="B40" s="10" t="n">
         <f aca="false">C8*Припущення!$B$24</f>
-        <v>5191200</v>
+        <v>6020022.4</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -5010,11 +4727,11 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>213</v>
+        <v>250</v>
       </c>
       <c r="B41" s="10" t="n">
         <f aca="false">$B$11*Припущення!$B$46*Припущення!$B$25</f>
-        <v>1050000</v>
+        <v>0</v>
       </c>
       <c r="C41" s="2"/>
       <c r="D41" s="2"/>
@@ -5027,7 +4744,7 @@
       </c>
       <c r="B42" s="10" t="n">
         <f aca="false">($B$40+$B$41)*Припущення!$B$26</f>
-        <v>936180</v>
+        <v>903003.36</v>
       </c>
       <c r="C42" s="2"/>
       <c r="D42" s="2"/>
@@ -5036,11 +4753,11 @@
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>214</v>
+        <v>251</v>
       </c>
       <c r="B43" s="10" t="n">
         <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$27</f>
-        <v>358869</v>
+        <v>346151.288</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -5053,7 +4770,7 @@
       </c>
       <c r="B44" s="10" t="n">
         <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$28</f>
-        <v>717738</v>
+        <v>692302.576</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
@@ -5062,11 +4779,11 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>215</v>
+        <v>252</v>
       </c>
       <c r="B45" s="10" t="n">
         <f aca="false">$B$15*Припущення!$B$29</f>
-        <v>435000</v>
+        <v>375000</v>
       </c>
       <c r="C45" s="2"/>
       <c r="D45" s="2"/>
@@ -5075,11 +4792,11 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>216</v>
+        <v>253</v>
       </c>
       <c r="B46" s="10" t="n">
         <f aca="false">$B$15*Припущення!$B$30</f>
-        <v>4640</v>
+        <v>4000</v>
       </c>
       <c r="C46" s="2"/>
       <c r="D46" s="2"/>
@@ -5088,7 +4805,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>217</v>
+        <v>254</v>
       </c>
       <c r="B47" s="9" t="n">
         <f aca="false">Припущення!$B$31</f>
@@ -5105,7 +4822,7 @@
       </c>
       <c r="B48" s="10" t="n">
         <f aca="false">$B$37*Припущення!$B$34</f>
-        <v>255776.5</v>
+        <v>232050</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -5114,11 +4831,11 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>218</v>
+        <v>255</v>
       </c>
       <c r="B49" s="10" t="n">
         <f aca="false">$B$15*Припущення!$B$35</f>
-        <v>43500</v>
+        <v>37500</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
@@ -5127,7 +4844,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>219</v>
+        <v>256</v>
       </c>
       <c r="B50" s="9" t="n">
         <f aca="false">Припущення!$B$41</f>
@@ -5153,14 +4870,14 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>220</v>
+        <v>257</v>
       </c>
       <c r="B52" s="10" t="n">
         <f aca="false">Припущення!$B$36*(Припущення!$B$37*SUM($B$40:$B$49)*Припущення!$B$38/12+($B$50+$B$51)*(Припущення!$B$38+$B$13)/12)</f>
-        <v>1243161.315</v>
+        <v>1065602.66616</v>
       </c>
       <c r="C52" s="24" t="s">
-        <v>221</v>
+        <v>258</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
@@ -5168,11 +4885,11 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>222</v>
+        <v>259</v>
       </c>
       <c r="B53" s="13" t="n">
         <f aca="false">SUM($B$40:$B$52)</f>
-        <v>11876064.815</v>
+        <v>11315632.29016</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
@@ -5189,7 +4906,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="21" t="s">
-        <v>223</v>
+        <v>260</v>
       </c>
       <c r="B55" s="22"/>
       <c r="C55" s="22"/>
@@ -5199,11 +4916,11 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="s">
-        <v>224</v>
+        <v>261</v>
       </c>
       <c r="B56" s="13" t="n">
         <f aca="false">$B$37-$B$53</f>
-        <v>-1645004.815</v>
+        <v>-2033632.29016</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
@@ -5216,7 +4933,7 @@
       </c>
       <c r="B57" s="15" t="n">
         <f aca="false">IF($B$37&lt;&gt;0,$B$56/$B$37,0)</f>
-        <v>-0.160785374633713</v>
+        <v>-0.219094192001724</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
@@ -5225,11 +4942,11 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>225</v>
+        <v>262</v>
       </c>
       <c r="B58" s="17" t="n">
         <f aca="false">IF($B$53&lt;&gt;0,$B$56/$B$53,0)</f>
-        <v>-0.138514300875344</v>
+        <v>-0.179718838330266</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
@@ -5238,9 +4955,9 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>226</v>
-      </c>
-      <c r="B59" s="36" t="str">
+        <v>263</v>
+      </c>
+      <c r="B59" s="39" t="str">
         <f aca="false">IF($B$57&gt;=Припущення!$B$43,"Досягає цілі","НИЖЧЕ ЦІЛІ")</f>
         <v>НИЖЧЕ ЦІЛІ</v>
       </c>
@@ -5251,14 +4968,14 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>227</v>
+        <v>264</v>
       </c>
       <c r="B60" s="10" t="n">
         <f aca="false">($B$37*(1-Припущення!$B$43)-($B$53-$B$50-$B$51-Припущення!$B$36*($B$50+$B$51)*(Припущення!$B$38+$B$13)/12))/(1+Припущення!$B$42+Припущення!$B$36*(1+Припущення!$B$42)*(Припущення!$B$38+$B$13)/12)</f>
-        <v>-1241952.76704799</v>
+        <v>-1610035.40946594</v>
       </c>
       <c r="C60" s="24" t="s">
-        <v>228</v>
+        <v>265</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
@@ -5266,11 +4983,11 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>229</v>
+        <v>266</v>
       </c>
       <c r="B61" s="13" t="n">
         <f aca="false">$B$12*$B$56-(1-$B$12)*$B$14</f>
-        <v>-877752.16675</v>
+        <v>-1743587.446636</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
@@ -5287,7 +5004,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="21" t="s">
-        <v>230</v>
+        <v>267</v>
       </c>
       <c r="B63" s="22"/>
       <c r="C63" s="22"/>
@@ -5297,11 +5014,11 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>231</v>
+        <v>268</v>
       </c>
       <c r="B64" s="10" t="n">
         <f aca="false">SUM($B$40:$B$44)</f>
-        <v>8253987</v>
+        <v>7961479.624</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
@@ -5310,11 +5027,11 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>232</v>
+        <v>269</v>
       </c>
       <c r="B65" s="10" t="n">
         <f aca="false">$B$53-$B$64-$B$48</f>
-        <v>3366301.315</v>
+        <v>3122102.66616</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
@@ -5323,14 +5040,905 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>233</v>
+        <v>270</v>
       </c>
       <c r="B66" s="17" t="n">
         <f aca="false">($B$64+$B$65)/($B$37*(1-Припущення!$B$34-Припущення!$B$43))-1</f>
-        <v>0.465529515656405</v>
+        <v>0.540766699357063</v>
       </c>
       <c r="C66" s="24" t="s">
+        <v>271</v>
+      </c>
+      <c r="D66" s="2"/>
+      <c r="E66" s="2"/>
+      <c r="F66" s="2"/>
+    </row>
+  </sheetData>
+  <mergeCells count="1">
+    <mergeCell ref="A2:F2"/>
+  </mergeCells>
+  <printOptions headings="false" gridLines="false" gridLinesSet="true" horizontalCentered="false" verticalCentered="false"/>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.511811023622047" footer="0.511811023622047"/>
+  <pageSetup paperSize="9" scale="100" fitToWidth="1" fitToHeight="1" pageOrder="downThenOver" orientation="portrait" blackAndWhite="false" draft="false" cellComments="none" horizontalDpi="300" verticalDpi="300" copies="1"/>
+  <headerFooter differentFirst="false" differentOddEven="false">
+    <oddHeader/>
+    <oddFooter/>
+  </headerFooter>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+  <sheetPr filterMode="false">
+    <pageSetUpPr fitToPage="false"/>
+  </sheetPr>
+  <dimension ref="A1:F66"/>
+  <sheetFormatPr defaultColWidth="8.6796875" defaultRowHeight="15" zeroHeight="false" outlineLevelRow="0" outlineLevelCol="0"/>
+  <cols>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="1" min="1" style="0" width="46"/>
+    <col collapsed="false" customWidth="true" hidden="false" outlineLevel="0" max="6" min="2" style="0" width="18"/>
+  </cols>
+  <sheetData>
+    <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A1" s="1" t="s">
+        <v>272</v>
+      </c>
+      <c r="B1" s="2"/>
+      <c r="C1" s="2"/>
+      <c r="D1" s="2"/>
+      <c r="E1" s="2"/>
+      <c r="F1" s="2"/>
+    </row>
+    <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A2" s="3" t="s">
+        <v>273</v>
+      </c>
+      <c r="B2" s="3"/>
+      <c r="C2" s="3"/>
+      <c r="D2" s="3"/>
+      <c r="E2" s="3"/>
+      <c r="F2" s="3"/>
+    </row>
+    <row r="3" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A3" s="2"/>
+      <c r="B3" s="2"/>
+      <c r="C3" s="2"/>
+      <c r="D3" s="2"/>
+      <c r="E3" s="2"/>
+      <c r="F3" s="2"/>
+    </row>
+    <row r="4" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
+      <c r="A4" s="4" t="s">
+        <v>78</v>
+      </c>
+      <c r="B4" s="4" t="s">
+        <v>212</v>
+      </c>
+      <c r="C4" s="4" t="s">
+        <v>213</v>
+      </c>
+      <c r="D4" s="4" t="s">
+        <v>86</v>
+      </c>
+      <c r="E4" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="F4" s="4" t="s">
+        <v>215</v>
+      </c>
+    </row>
+    <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A5" s="35" t="str">
+        <f aca="false">Припущення!$A$5</f>
+        <v>Lake House Compact 61</v>
+      </c>
+      <c r="B5" s="28" t="n">
+        <v>10</v>
+      </c>
+      <c r="C5" s="36" t="n">
+        <f aca="false">B5*Припущення!$B$5</f>
+        <v>615</v>
+      </c>
+      <c r="D5" s="9" t="n">
+        <f aca="false">Припущення!$I$5</f>
+        <v>340000</v>
+      </c>
+      <c r="E5" s="10" t="n">
+        <f aca="false">B5*D5</f>
+        <v>3400000</v>
+      </c>
+      <c r="F5" s="7" t="n">
+        <f aca="false">B5*Припущення!$J$5</f>
+        <v>3400</v>
+      </c>
+    </row>
+    <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A6" s="35" t="str">
+        <f aca="false">Припущення!$A$6</f>
+        <v>Meadow 71</v>
+      </c>
+      <c r="B6" s="28" t="n">
+        <v>8</v>
+      </c>
+      <c r="C6" s="36" t="n">
+        <f aca="false">B6*Припущення!$B$6</f>
+        <v>568</v>
+      </c>
+      <c r="D6" s="9" t="n">
+        <f aca="false">Припущення!$I$6</f>
+        <v>390000</v>
+      </c>
+      <c r="E6" s="10" t="n">
+        <f aca="false">B6*D6</f>
+        <v>3120000</v>
+      </c>
+      <c r="F6" s="7" t="n">
+        <f aca="false">B6*Припущення!$J$6</f>
+        <v>2960</v>
+      </c>
+    </row>
+    <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A7" s="35" t="str">
+        <f aca="false">Припущення!$A$7</f>
+        <v>Country 140</v>
+      </c>
+      <c r="B7" s="28" t="n">
+        <v>7</v>
+      </c>
+      <c r="C7" s="36" t="n">
+        <f aca="false">B7*Припущення!$B$7</f>
+        <v>980</v>
+      </c>
+      <c r="D7" s="9" t="n">
+        <f aca="false">Припущення!$I$7</f>
+        <v>550000</v>
+      </c>
+      <c r="E7" s="10" t="n">
+        <f aca="false">B7*D7</f>
+        <v>3850000</v>
+      </c>
+      <c r="F7" s="7" t="n">
+        <f aca="false">B7*Припущення!$J$7</f>
+        <v>3920</v>
+      </c>
+    </row>
+    <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A8" s="11" t="s">
+        <v>216</v>
+      </c>
+      <c r="B8" s="37" t="n">
+        <f aca="false">SUM(B5:B7)</f>
+        <v>25</v>
+      </c>
+      <c r="C8" s="38" t="n">
+        <f aca="false">SUM(C5:C7)</f>
+        <v>2163</v>
+      </c>
+      <c r="D8" s="33"/>
+      <c r="E8" s="13" t="n">
+        <f aca="false">SUM(E5:E7)</f>
+        <v>10370000</v>
+      </c>
+      <c r="F8" s="37" t="n">
+        <f aca="false">SUM(F5:F7)</f>
+        <v>10280</v>
+      </c>
+    </row>
+    <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A9" s="2"/>
+      <c r="B9" s="2"/>
+      <c r="C9" s="2"/>
+      <c r="D9" s="2"/>
+      <c r="E9" s="2"/>
+      <c r="F9" s="2"/>
+    </row>
+    <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A10" s="21" t="s">
+        <v>217</v>
+      </c>
+      <c r="B10" s="22"/>
+      <c r="C10" s="22"/>
+      <c r="D10" s="22"/>
+      <c r="E10" s="22"/>
+      <c r="F10" s="22"/>
+    </row>
+    <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A11" s="5" t="s">
+        <v>218</v>
+      </c>
+      <c r="B11" s="28" t="n">
+        <v>1</v>
+      </c>
+      <c r="C11" s="2"/>
+      <c r="D11" s="2"/>
+      <c r="E11" s="2"/>
+      <c r="F11" s="2"/>
+    </row>
+    <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A12" s="5" t="s">
+        <v>219</v>
+      </c>
+      <c r="B12" s="25" t="n">
+        <v>0.45</v>
+      </c>
+      <c r="C12" s="24" t="s">
+        <v>220</v>
+      </c>
+      <c r="D12" s="2"/>
+      <c r="E12" s="2"/>
+      <c r="F12" s="2"/>
+    </row>
+    <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A13" s="5" t="s">
+        <v>221</v>
+      </c>
+      <c r="B13" s="28" t="n">
+        <v>12</v>
+      </c>
+      <c r="C13" s="24" t="s">
+        <v>222</v>
+      </c>
+      <c r="D13" s="2"/>
+      <c r="E13" s="2"/>
+      <c r="F13" s="2"/>
+    </row>
+    <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A14" s="5" t="s">
+        <v>223</v>
+      </c>
+      <c r="B14" s="26" t="n">
+        <v>250000</v>
+      </c>
+      <c r="C14" s="24" t="s">
+        <v>224</v>
+      </c>
+      <c r="D14" s="2"/>
+      <c r="E14" s="2"/>
+      <c r="F14" s="2"/>
+    </row>
+    <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A15" s="5" t="s">
+        <v>225</v>
+      </c>
+      <c r="B15" s="7" t="n">
+        <f aca="false">B8+$B$11*Припущення!$B$50</f>
+        <v>29</v>
+      </c>
+      <c r="C15" s="24" t="s">
+        <v>226</v>
+      </c>
+      <c r="D15" s="2"/>
+      <c r="E15" s="2"/>
+      <c r="F15" s="2"/>
+    </row>
+    <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A16" s="2"/>
+      <c r="B16" s="2"/>
+      <c r="C16" s="2"/>
+      <c r="D16" s="2"/>
+      <c r="E16" s="2"/>
+      <c r="F16" s="2"/>
+    </row>
+    <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A17" s="21" t="s">
+        <v>227</v>
+      </c>
+      <c r="B17" s="22"/>
+      <c r="C17" s="22"/>
+      <c r="D17" s="22"/>
+      <c r="E17" s="22"/>
+      <c r="F17" s="22"/>
+    </row>
+    <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A18" s="5" t="s">
+        <v>228</v>
+      </c>
+      <c r="B18" s="7" t="n">
+        <f aca="false">F8</f>
+        <v>10280</v>
+      </c>
+      <c r="C18" s="2"/>
+      <c r="D18" s="2"/>
+      <c r="E18" s="2"/>
+      <c r="F18" s="2"/>
+    </row>
+    <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A19" s="5" t="s">
+        <v>229</v>
+      </c>
+      <c r="B19" s="6" t="n">
+        <f aca="false">Припущення!$B$12*Припущення!$B$13</f>
+        <v>2564.1</v>
+      </c>
+      <c r="C19" s="2"/>
+      <c r="D19" s="2"/>
+      <c r="E19" s="2"/>
+      <c r="F19" s="2"/>
+    </row>
+    <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A20" s="5" t="s">
+        <v>230</v>
+      </c>
+      <c r="B20" s="6" t="n">
+        <f aca="false">Припущення!$B$12*Припущення!$B$14</f>
+        <v>997.15</v>
+      </c>
+      <c r="C20" s="2"/>
+      <c r="D20" s="2"/>
+      <c r="E20" s="2"/>
+      <c r="F20" s="2"/>
+    </row>
+    <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A21" s="5" t="s">
+        <v>231</v>
+      </c>
+      <c r="B21" s="6" t="n">
+        <f aca="false">Припущення!$B$12*Припущення!$B$15</f>
+        <v>854.7</v>
+      </c>
+      <c r="C21" s="2"/>
+      <c r="D21" s="2"/>
+      <c r="E21" s="2"/>
+      <c r="F21" s="2"/>
+    </row>
+    <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A22" s="5" t="s">
+        <v>232</v>
+      </c>
+      <c r="B22" s="7" t="n">
+        <f aca="false">$B$11*Припущення!$B$16</f>
+        <v>900</v>
+      </c>
+      <c r="C22" s="2"/>
+      <c r="D22" s="2"/>
+      <c r="E22" s="2"/>
+      <c r="F22" s="2"/>
+    </row>
+    <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A23" s="11" t="s">
+        <v>233</v>
+      </c>
+      <c r="B23" s="37" t="n">
+        <f aca="false">SUM($B$18:$B$22)</f>
+        <v>15595.95</v>
+      </c>
+      <c r="C23" s="2"/>
+      <c r="D23" s="2"/>
+      <c r="E23" s="2"/>
+      <c r="F23" s="2"/>
+    </row>
+    <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A24" s="5" t="s">
         <v>234</v>
+      </c>
+      <c r="B24" s="6" t="n">
+        <f aca="false">Припущення!$B$12</f>
+        <v>14245</v>
+      </c>
+      <c r="C24" s="2"/>
+      <c r="D24" s="2"/>
+      <c r="E24" s="2"/>
+      <c r="F24" s="2"/>
+    </row>
+    <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A25" s="11" t="s">
+        <v>235</v>
+      </c>
+      <c r="B25" s="37" t="n">
+        <f aca="false">$B$24-$B$23</f>
+        <v>-1350.95</v>
+      </c>
+      <c r="C25" s="2"/>
+      <c r="D25" s="2"/>
+      <c r="E25" s="2"/>
+      <c r="F25" s="2"/>
+    </row>
+    <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A26" s="11" t="s">
+        <v>236</v>
+      </c>
+      <c r="B26" s="39" t="str">
+        <f aca="false">IF($B$25&gt;=0,"Вміщується","НЕ ВМІЩУЄТЬСЯ")</f>
+        <v>НЕ ВМІЩУЄТЬСЯ</v>
+      </c>
+      <c r="C26" s="2"/>
+      <c r="D26" s="2"/>
+      <c r="E26" s="2"/>
+      <c r="F26" s="2"/>
+    </row>
+    <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A27" s="5" t="s">
+        <v>9</v>
+      </c>
+      <c r="B27" s="7" t="n">
+        <f aca="false">IF(B8&gt;0,F8/B8,0)</f>
+        <v>411.2</v>
+      </c>
+      <c r="C27" s="2"/>
+      <c r="D27" s="2"/>
+      <c r="E27" s="2"/>
+      <c r="F27" s="2"/>
+    </row>
+    <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A28" s="2"/>
+      <c r="B28" s="2"/>
+      <c r="C28" s="2"/>
+      <c r="D28" s="2"/>
+      <c r="E28" s="2"/>
+      <c r="F28" s="2"/>
+    </row>
+    <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A29" s="21" t="s">
+        <v>237</v>
+      </c>
+      <c r="B29" s="22"/>
+      <c r="C29" s="22"/>
+      <c r="D29" s="22"/>
+      <c r="E29" s="22"/>
+      <c r="F29" s="22"/>
+    </row>
+    <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A30" s="5" t="s">
+        <v>238</v>
+      </c>
+      <c r="B30" s="10" t="n">
+        <f aca="false">E8</f>
+        <v>10370000</v>
+      </c>
+      <c r="C30" s="2"/>
+      <c r="D30" s="2"/>
+      <c r="E30" s="2"/>
+      <c r="F30" s="2"/>
+    </row>
+    <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A31" s="5" t="s">
+        <v>239</v>
+      </c>
+      <c r="B31" s="7" t="n">
+        <f aca="false">ROUNDUP($B$15*Припущення!$B$19,0)</f>
+        <v>9</v>
+      </c>
+      <c r="C31" s="24" t="s">
+        <v>240</v>
+      </c>
+      <c r="D31" s="2"/>
+      <c r="E31" s="2"/>
+      <c r="F31" s="2"/>
+    </row>
+    <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A32" s="5" t="s">
+        <v>241</v>
+      </c>
+      <c r="B32" s="7" t="n">
+        <f aca="false">MIN($B$31,INDEX(B5:B7,Припущення!$B$21))</f>
+        <v>9</v>
+      </c>
+      <c r="C32" s="2"/>
+      <c r="D32" s="2"/>
+      <c r="E32" s="2"/>
+      <c r="F32" s="2"/>
+    </row>
+    <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A33" s="5" t="s">
+        <v>242</v>
+      </c>
+      <c r="B33" s="40" t="str">
+        <f aca="false">IF($B$32&lt;$B$31,"Обраного типу замало — потрібні інші типи","OK")</f>
+        <v>OK</v>
+      </c>
+      <c r="C33" s="2"/>
+      <c r="D33" s="2"/>
+      <c r="E33" s="2"/>
+      <c r="F33" s="2"/>
+    </row>
+    <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A34" s="5" t="s">
+        <v>243</v>
+      </c>
+      <c r="B34" s="10" t="n">
+        <f aca="false">-$B$31*INDEX(D5:D7,Припущення!$B$21)*(1-Припущення!$B$20)</f>
+        <v>-1224000</v>
+      </c>
+      <c r="C34" s="24" t="s">
+        <v>244</v>
+      </c>
+      <c r="D34" s="2"/>
+      <c r="E34" s="2"/>
+      <c r="F34" s="2"/>
+    </row>
+    <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A35" s="5" t="s">
+        <v>245</v>
+      </c>
+      <c r="B35" s="10" t="n">
+        <f aca="false">$B$11*Припущення!$B$47*Припущення!$B$48/Припущення!$B$49</f>
+        <v>350000</v>
+      </c>
+      <c r="C35" s="2"/>
+      <c r="D35" s="2"/>
+      <c r="E35" s="2"/>
+      <c r="F35" s="2"/>
+    </row>
+    <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A36" s="5" t="s">
+        <v>246</v>
+      </c>
+      <c r="B36" s="10" t="n">
+        <f aca="false">$B$11*Припущення!$B$50*Припущення!$B$51</f>
+        <v>880000</v>
+      </c>
+      <c r="C36" s="2"/>
+      <c r="D36" s="2"/>
+      <c r="E36" s="2"/>
+      <c r="F36" s="2"/>
+    </row>
+    <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A37" s="11" t="s">
+        <v>247</v>
+      </c>
+      <c r="B37" s="13" t="n">
+        <f aca="false">SUM($B$30,$B$34,$B$35,$B$36)</f>
+        <v>10376000</v>
+      </c>
+      <c r="C37" s="2"/>
+      <c r="D37" s="2"/>
+      <c r="E37" s="2"/>
+      <c r="F37" s="2"/>
+    </row>
+    <row r="38" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A38" s="2"/>
+      <c r="B38" s="2"/>
+      <c r="C38" s="2"/>
+      <c r="D38" s="2"/>
+      <c r="E38" s="2"/>
+      <c r="F38" s="2"/>
+    </row>
+    <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A39" s="21" t="s">
+        <v>248</v>
+      </c>
+      <c r="B39" s="22"/>
+      <c r="C39" s="22"/>
+      <c r="D39" s="22"/>
+      <c r="E39" s="22"/>
+      <c r="F39" s="22"/>
+    </row>
+    <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A40" s="5" t="s">
+        <v>249</v>
+      </c>
+      <c r="B40" s="10" t="n">
+        <f aca="false">C8*Припущення!$B$24</f>
+        <v>6020022.4</v>
+      </c>
+      <c r="C40" s="2"/>
+      <c r="D40" s="2"/>
+      <c r="E40" s="2"/>
+      <c r="F40" s="2"/>
+    </row>
+    <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A41" s="5" t="s">
+        <v>250</v>
+      </c>
+      <c r="B41" s="10" t="n">
+        <f aca="false">$B$11*Припущення!$B$46*Припущення!$B$25</f>
+        <v>980000</v>
+      </c>
+      <c r="C41" s="2"/>
+      <c r="D41" s="2"/>
+      <c r="E41" s="2"/>
+      <c r="F41" s="2"/>
+    </row>
+    <row r="42" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A42" s="5" t="s">
+        <v>125</v>
+      </c>
+      <c r="B42" s="10" t="n">
+        <f aca="false">($B$40+$B$41)*Припущення!$B$26</f>
+        <v>1050003.36</v>
+      </c>
+      <c r="C42" s="2"/>
+      <c r="D42" s="2"/>
+      <c r="E42" s="2"/>
+      <c r="F42" s="2"/>
+    </row>
+    <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A43" s="5" t="s">
+        <v>251</v>
+      </c>
+      <c r="B43" s="10" t="n">
+        <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$27</f>
+        <v>402501.288</v>
+      </c>
+      <c r="C43" s="2"/>
+      <c r="D43" s="2"/>
+      <c r="E43" s="2"/>
+      <c r="F43" s="2"/>
+    </row>
+    <row r="44" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A44" s="5" t="s">
+        <v>131</v>
+      </c>
+      <c r="B44" s="10" t="n">
+        <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$28</f>
+        <v>805002.576</v>
+      </c>
+      <c r="C44" s="2"/>
+      <c r="D44" s="2"/>
+      <c r="E44" s="2"/>
+      <c r="F44" s="2"/>
+    </row>
+    <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A45" s="5" t="s">
+        <v>252</v>
+      </c>
+      <c r="B45" s="10" t="n">
+        <f aca="false">$B$15*Припущення!$B$29</f>
+        <v>435000</v>
+      </c>
+      <c r="C45" s="2"/>
+      <c r="D45" s="2"/>
+      <c r="E45" s="2"/>
+      <c r="F45" s="2"/>
+    </row>
+    <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A46" s="5" t="s">
+        <v>253</v>
+      </c>
+      <c r="B46" s="10" t="n">
+        <f aca="false">$B$15*Припущення!$B$30</f>
+        <v>4640</v>
+      </c>
+      <c r="C46" s="2"/>
+      <c r="D46" s="2"/>
+      <c r="E46" s="2"/>
+      <c r="F46" s="2"/>
+    </row>
+    <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A47" s="5" t="s">
+        <v>254</v>
+      </c>
+      <c r="B47" s="9" t="n">
+        <f aca="false">Припущення!$B$31</f>
+        <v>50000</v>
+      </c>
+      <c r="C47" s="2"/>
+      <c r="D47" s="2"/>
+      <c r="E47" s="2"/>
+      <c r="F47" s="2"/>
+    </row>
+    <row r="48" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A48" s="5" t="s">
+        <v>140</v>
+      </c>
+      <c r="B48" s="10" t="n">
+        <f aca="false">$B$37*Припущення!$B$34</f>
+        <v>259400</v>
+      </c>
+      <c r="C48" s="2"/>
+      <c r="D48" s="2"/>
+      <c r="E48" s="2"/>
+      <c r="F48" s="2"/>
+    </row>
+    <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A49" s="5" t="s">
+        <v>255</v>
+      </c>
+      <c r="B49" s="10" t="n">
+        <f aca="false">$B$15*Припущення!$B$35</f>
+        <v>43500</v>
+      </c>
+      <c r="C49" s="2"/>
+      <c r="D49" s="2"/>
+      <c r="E49" s="2"/>
+      <c r="F49" s="2"/>
+    </row>
+    <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A50" s="5" t="s">
+        <v>256</v>
+      </c>
+      <c r="B50" s="9" t="n">
+        <f aca="false">Припущення!$B$41</f>
+        <v>1500000</v>
+      </c>
+      <c r="C50" s="2"/>
+      <c r="D50" s="2"/>
+      <c r="E50" s="2"/>
+      <c r="F50" s="2"/>
+    </row>
+    <row r="51" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A51" s="5" t="s">
+        <v>154</v>
+      </c>
+      <c r="B51" s="10" t="n">
+        <f aca="false">$B$50*Припущення!$B$42</f>
+        <v>90000</v>
+      </c>
+      <c r="C51" s="2"/>
+      <c r="D51" s="2"/>
+      <c r="E51" s="2"/>
+      <c r="F51" s="2"/>
+    </row>
+    <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A52" s="5" t="s">
+        <v>257</v>
+      </c>
+      <c r="B52" s="10" t="n">
+        <f aca="false">Припущення!$B$36*(Припущення!$B$37*SUM($B$40:$B$49)*Припущення!$B$38/12+($B$50+$B$51)*(Припущення!$B$38+$B$13)/12)</f>
+        <v>1333806.26616</v>
+      </c>
+      <c r="C52" s="24" t="s">
+        <v>258</v>
+      </c>
+      <c r="D52" s="2"/>
+      <c r="E52" s="2"/>
+      <c r="F52" s="2"/>
+    </row>
+    <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A53" s="11" t="s">
+        <v>259</v>
+      </c>
+      <c r="B53" s="13" t="n">
+        <f aca="false">SUM($B$40:$B$52)</f>
+        <v>12973875.89016</v>
+      </c>
+      <c r="C53" s="2"/>
+      <c r="D53" s="2"/>
+      <c r="E53" s="2"/>
+      <c r="F53" s="2"/>
+    </row>
+    <row r="54" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A54" s="2"/>
+      <c r="B54" s="2"/>
+      <c r="C54" s="2"/>
+      <c r="D54" s="2"/>
+      <c r="E54" s="2"/>
+      <c r="F54" s="2"/>
+    </row>
+    <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A55" s="21" t="s">
+        <v>260</v>
+      </c>
+      <c r="B55" s="22"/>
+      <c r="C55" s="22"/>
+      <c r="D55" s="22"/>
+      <c r="E55" s="22"/>
+      <c r="F55" s="22"/>
+    </row>
+    <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A56" s="11" t="s">
+        <v>261</v>
+      </c>
+      <c r="B56" s="13" t="n">
+        <f aca="false">$B$37-$B$53</f>
+        <v>-2597875.89016</v>
+      </c>
+      <c r="C56" s="2"/>
+      <c r="D56" s="2"/>
+      <c r="E56" s="2"/>
+      <c r="F56" s="2"/>
+    </row>
+    <row r="57" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A57" s="11" t="s">
+        <v>14</v>
+      </c>
+      <c r="B57" s="15" t="n">
+        <f aca="false">IF($B$37&lt;&gt;0,$B$56/$B$37,0)</f>
+        <v>-0.250373543770239</v>
+      </c>
+      <c r="C57" s="2"/>
+      <c r="D57" s="2"/>
+      <c r="E57" s="2"/>
+      <c r="F57" s="2"/>
+    </row>
+    <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A58" s="5" t="s">
+        <v>262</v>
+      </c>
+      <c r="B58" s="17" t="n">
+        <f aca="false">IF($B$53&lt;&gt;0,$B$56/$B$53,0)</f>
+        <v>-0.200238996592402</v>
+      </c>
+      <c r="C58" s="2"/>
+      <c r="D58" s="2"/>
+      <c r="E58" s="2"/>
+      <c r="F58" s="2"/>
+    </row>
+    <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A59" s="11" t="s">
+        <v>263</v>
+      </c>
+      <c r="B59" s="39" t="str">
+        <f aca="false">IF($B$57&gt;=Припущення!$B$43,"Досягає цілі","НИЖЧЕ ЦІЛІ")</f>
+        <v>НИЖЧЕ ЦІЛІ</v>
+      </c>
+      <c r="C59" s="2"/>
+      <c r="D59" s="2"/>
+      <c r="E59" s="2"/>
+      <c r="F59" s="2"/>
+    </row>
+    <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A60" s="5" t="s">
+        <v>264</v>
+      </c>
+      <c r="B60" s="10" t="n">
+        <f aca="false">($B$37*(1-Припущення!$B$43)-($B$53-$B$50-$B$51-Припущення!$B$36*($B$50+$B$51)*(Припущення!$B$38+$B$13)/12))/(1+Припущення!$B$42+Припущення!$B$36*(1+Припущення!$B$42)*(Припущення!$B$38+$B$13)/12)</f>
+        <v>-1971308.78781756</v>
+      </c>
+      <c r="C60" s="24" t="s">
+        <v>265</v>
+      </c>
+      <c r="D60" s="2"/>
+      <c r="E60" s="2"/>
+      <c r="F60" s="2"/>
+    </row>
+    <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A61" s="11" t="s">
+        <v>266</v>
+      </c>
+      <c r="B61" s="13" t="n">
+        <f aca="false">$B$12*$B$56-(1-$B$12)*$B$14</f>
+        <v>-1306544.150572</v>
+      </c>
+      <c r="C61" s="2"/>
+      <c r="D61" s="2"/>
+      <c r="E61" s="2"/>
+      <c r="F61" s="2"/>
+    </row>
+    <row r="62" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A62" s="2"/>
+      <c r="B62" s="2"/>
+      <c r="C62" s="2"/>
+      <c r="D62" s="2"/>
+      <c r="E62" s="2"/>
+      <c r="F62" s="2"/>
+    </row>
+    <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A63" s="21" t="s">
+        <v>267</v>
+      </c>
+      <c r="B63" s="22"/>
+      <c r="C63" s="22"/>
+      <c r="D63" s="22"/>
+      <c r="E63" s="22"/>
+      <c r="F63" s="22"/>
+    </row>
+    <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A64" s="5" t="s">
+        <v>268</v>
+      </c>
+      <c r="B64" s="10" t="n">
+        <f aca="false">SUM($B$40:$B$44)</f>
+        <v>9257529.624</v>
+      </c>
+      <c r="C64" s="2"/>
+      <c r="D64" s="2"/>
+      <c r="E64" s="2"/>
+      <c r="F64" s="2"/>
+    </row>
+    <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A65" s="5" t="s">
+        <v>269</v>
+      </c>
+      <c r="B65" s="10" t="n">
+        <f aca="false">$B$53-$B$64-$B$48</f>
+        <v>3456946.26616</v>
+      </c>
+      <c r="C65" s="2"/>
+      <c r="D65" s="2"/>
+      <c r="E65" s="2"/>
+      <c r="F65" s="2"/>
+    </row>
+    <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
+      <c r="A66" s="5" t="s">
+        <v>270</v>
+      </c>
+      <c r="B66" s="17" t="n">
+        <f aca="false">($B$64+$B$65)/($B$37*(1-Припущення!$B$34-Припущення!$B$43))-1</f>
+        <v>0.581127153251922</v>
+      </c>
+      <c r="C66" s="24" t="s">
+        <v>271</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>

</xml_diff>

<commit_message>
Switch to catalogue types Lake 92 / Metropolis 128 / Halcyon 170; externals per house
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_014iit8YdqqexD3WDZo9gb62
</commit_message>
<xml_diff>
--- a/model/ZON_Wivenhoe_Appraisal.xlsx
+++ b/model/ZON_Wivenhoe_Appraisal.xlsx
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="383" uniqueCount="274">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="392" uniqueCount="280">
   <si>
     <t xml:space="preserve">ZON Wivenhoe — порівняння сценаріїв</t>
   </si>
@@ -294,25 +294,25 @@
     <t xml:space="preserve">Джерело / примітка</t>
   </si>
   <si>
-    <t xml:space="preserve">Lake House Compact 61</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GIA з брифу. NDSS 2b3p 1 пов. = 61 м². Ціна £340k — робоча ціна команди ZON, не підтверджена агентом.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Meadow 71</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GIA з брифу. NDSS 2b4p 1 пов. = 70 м². Ціна £390k — робоча ціна команди ZON, не підтверджена агентом.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Country 140</t>
-  </si>
-  <si>
-    <t xml:space="preserve">GIA з брифу. NDSS 3b6p 1 пов. = 95 м². Ціна £550k — робоча ціна команди ZON, не підтверджена агентом.</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Ціни — робочі ціни команди ZON (£340k / £390k / £550k). Треба підтвердити звітом агента (Savills / Fenn Wright / Beresfords).</t>
+    <t xml:space="preserve">Lake House Standard 92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Каталог ZON: 1 пов., 14 × 8 м, 2 спальні + кабінет, 2 санвузли. NDSS 2b4p = 70 м². Ціна £410k — оцінка Claude, підтверджує агент.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Metropolis 128</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Каталог ZON: 2 пов., 9,8 × 7,9 м, 3 спальні + кабінет. NDSS 3b6p 2 пов. = 102 м². УВАГА: не бунгало. Ціна £460k — оцінка Claude.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Halcyon Estate 170</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Каталог ZON 317 м² = 170 житлові + гараж 36 + тераси ~105. 18,6 × 16,6 м. NDSS 4b8p 1 пов. = 117 м². Ціна £700k — оцінка Claude.</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Ціни — оцінка Claude для нових будинків у CO7 (£410k / £460k / £700k). Треба підтвердити звітом агента (Savills / Fenn Wright / Beresfords).</t>
   </si>
   <si>
     <t xml:space="preserve">Ділянка та планування</t>
@@ -381,7 +381,7 @@
     <t xml:space="preserve">1/2/3</t>
   </si>
   <si>
-    <t xml:space="preserve">1 = Compact 61, 2 = Meadow 71, 3 = Country 140</t>
+    <t xml:space="preserve">1 = Lake 92, 2 = Metropolis 128, 3 = Halcyon 170</t>
   </si>
   <si>
     <t xml:space="preserve">Вартість будівництва</t>
@@ -405,10 +405,10 @@
     <t xml:space="preserve">Зовнішні роботи та мережі</t>
   </si>
   <si>
-    <t xml:space="preserve">% будівництва</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Припущення: дороги, SuDS, містки, мережі, підстанція</t>
+    <t xml:space="preserve">£/будинок</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Припущення: дороги, дренаж SuDS, мережі й підключення, підстанція (~£0,9 млн на 25)</t>
   </si>
   <si>
     <t xml:space="preserve">Резерв на непередбачене</t>
@@ -561,7 +561,10 @@
     <t xml:space="preserve">База</t>
   </si>
   <si>
-    <t xml:space="preserve">Compact 61</t>
+    <t xml:space="preserve">Lake 92</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Halcyon 170</t>
   </si>
   <si>
     <t xml:space="preserve">Примітка / діапазон</t>
@@ -576,13 +579,16 @@
     <t xml:space="preserve">Оболонка ZON + опалення</t>
   </si>
   <si>
-    <t xml:space="preserve">Від команди ZON. Стіни, дах, вікна, опалення</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Фундаменти</t>
-  </si>
-  <si>
-    <t xml:space="preserve">£120–220/м²; гвинтові палі — нижня межа</t>
+    <t xml:space="preserve">Від команди ZON, на житлову площу. Стіни, дах, вікна, опалення</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Фундаменти (на пляму забудови)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">за будинок</t>
+  </si>
+  <si>
+    <t xml:space="preserve">£160/м² плями: 112 / 77 / 309 м²</t>
   </si>
   <si>
     <t xml:space="preserve">Доставка, кран, монтаж, герметизація</t>
@@ -600,16 +606,13 @@
     <t xml:space="preserve">Сонячні панелі в дах (вимога Future Homes Standard)</t>
   </si>
   <si>
-    <t xml:space="preserve">за будинок</t>
-  </si>
-  <si>
-    <t xml:space="preserve">3–5 кВт; батарея — опція ZON Ready</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Вентиляція (dMEV)</t>
-  </si>
-  <si>
-    <t xml:space="preserve">MVHR — +£3–4k</t>
+    <t xml:space="preserve">3–6 кВт; батарея — опція ZON Ready</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Вентиляція</t>
+  </si>
+  <si>
+    <t xml:space="preserve">dMEV; для Halcyon — MVHR</t>
   </si>
   <si>
     <t xml:space="preserve">Кухня з технікою</t>
@@ -621,7 +624,19 @@
     <t xml:space="preserve">Санвузли</t>
   </si>
   <si>
-    <t xml:space="preserve">Country — 2 санвузли</t>
+    <t xml:space="preserve">2 / 3 / 2 санвузли</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Сходи</t>
+  </si>
+  <si>
+    <t xml:space="preserve">лише Metropolis (2 поверхи)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Гараж на 2 авто і криті тераси</t>
+  </si>
+  <si>
+    <t xml:space="preserve">36 м² × £900 + ~105 м² × £300</t>
   </si>
   <si>
     <t xml:space="preserve">Гарантія 10 років, Building Control, SAP/EPC, тест повітря</t>
@@ -657,10 +672,10 @@
     <t xml:space="preserve">Не входить сюди (рахується в моделі окремо): дороги, мережі та підключення, SuDS — «Зовнішні роботи»; проєктування, резерв, S106, продаж, фінансування, земля.</t>
   </si>
   <si>
-    <t xml:space="preserve">Сценарій A — 25 бунгало в межах outline consent</t>
-  </si>
-  <si>
-    <t xml:space="preserve">Шлях: Reserved Matters. Без Hub. Відповідає ліміту 25 юнітів (за словами користувача).</t>
+    <t xml:space="preserve">Сценарій A — 25 будинків: Lake 92, Metropolis 128, Halcyon 170</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Шлях: Reserved Matters, якщо рада прийме Metropolis (2 пов.) у дозволі на бунгало. Без Hub.</t>
   </si>
   <si>
     <t xml:space="preserve">К-сть</t>
@@ -778,6 +793,9 @@
   </si>
   <si>
     <t xml:space="preserve">Будівництво Hub</t>
+  </si>
+  <si>
+    <t xml:space="preserve">на будинок; Hub = ще один</t>
   </si>
   <si>
     <t xml:space="preserve">Резерв</t>
@@ -1511,11 +1529,11 @@
       </c>
       <c r="B6" s="6" t="n">
         <f aca="false">'Сценарій A'!$B$25</f>
-        <v>-450.950000000001</v>
+        <v>-220.950000000001</v>
       </c>
       <c r="C6" s="6" t="n">
         <f aca="false">'Сценарій B'!$B$25</f>
-        <v>-1350.95</v>
+        <v>-1120.95</v>
       </c>
       <c r="D6" s="7" t="n">
         <f aca="false">C6-B6</f>
@@ -1546,11 +1564,11 @@
       </c>
       <c r="B8" s="6" t="n">
         <f aca="false">'Сценарій A'!$B$27</f>
-        <v>411.2</v>
+        <v>402</v>
       </c>
       <c r="C8" s="6" t="n">
         <f aca="false">'Сценарій B'!$B$27</f>
-        <v>411.2</v>
+        <v>402</v>
       </c>
       <c r="D8" s="7" t="n">
         <f aca="false">C8-B8</f>
@@ -1584,15 +1602,15 @@
       </c>
       <c r="B10" s="9" t="n">
         <f aca="false">'Сценарій A'!$B$37</f>
-        <v>9282000</v>
+        <v>10158000</v>
       </c>
       <c r="C10" s="9" t="n">
         <f aca="false">'Сценарій B'!$B$37</f>
-        <v>10376000</v>
+        <v>11224000</v>
       </c>
       <c r="D10" s="10" t="n">
         <f aca="false">C10-B10</f>
-        <v>1094000</v>
+        <v>1066000</v>
       </c>
       <c r="E10" s="2"/>
       <c r="F10" s="2"/>
@@ -1603,15 +1621,15 @@
       </c>
       <c r="B11" s="9" t="n">
         <f aca="false">'Сценарій A'!$B$53</f>
-        <v>11315632.29016</v>
+        <v>13707715.5696</v>
       </c>
       <c r="C11" s="9" t="n">
         <f aca="false">'Сценарій B'!$B$53</f>
-        <v>12973875.89016</v>
+        <v>15224804.1696</v>
       </c>
       <c r="D11" s="10" t="n">
         <f aca="false">C11-B11</f>
-        <v>1658243.6</v>
+        <v>1517088.6</v>
       </c>
       <c r="E11" s="2"/>
       <c r="F11" s="2"/>
@@ -1622,15 +1640,15 @@
       </c>
       <c r="B12" s="12" t="n">
         <f aca="false">'Сценарій A'!$B$56</f>
-        <v>-2033632.29016</v>
+        <v>-3549715.5696</v>
       </c>
       <c r="C12" s="12" t="n">
         <f aca="false">'Сценарій B'!$B$56</f>
-        <v>-2597875.89016</v>
+        <v>-4000804.1696</v>
       </c>
       <c r="D12" s="13" t="n">
         <f aca="false">C12-B12</f>
-        <v>-564243.6</v>
+        <v>-451088.6</v>
       </c>
       <c r="E12" s="2"/>
       <c r="F12" s="2"/>
@@ -1641,15 +1659,15 @@
       </c>
       <c r="B13" s="14" t="n">
         <f aca="false">'Сценарій A'!$B$57</f>
-        <v>-0.219094192001724</v>
+        <v>-0.349450243118724</v>
       </c>
       <c r="C13" s="14" t="n">
         <f aca="false">'Сценарій B'!$B$57</f>
-        <v>-0.250373543770239</v>
+        <v>-0.356450834782609</v>
       </c>
       <c r="D13" s="15" t="n">
         <f aca="false">C13-B13</f>
-        <v>-0.0312793517685152</v>
+        <v>-0.0070005916638845</v>
       </c>
       <c r="E13" s="2"/>
       <c r="F13" s="2"/>
@@ -1676,15 +1694,15 @@
       </c>
       <c r="B15" s="9" t="n">
         <f aca="false">'Сценарій A'!$B$60</f>
-        <v>-1610035.40946594</v>
+        <v>-2962196.64982411</v>
       </c>
       <c r="C15" s="9" t="n">
         <f aca="false">'Сценарій B'!$B$60</f>
-        <v>-1971308.78781756</v>
+        <v>-3139432.60258505</v>
       </c>
       <c r="D15" s="10" t="n">
         <f aca="false">C15-B15</f>
-        <v>-361273.378351619</v>
+        <v>-177235.952760941</v>
       </c>
       <c r="E15" s="2"/>
       <c r="F15" s="2"/>
@@ -1695,15 +1713,15 @@
       </c>
       <c r="B16" s="16" t="n">
         <f aca="false">'Сценарій A'!$B$66</f>
-        <v>0.540766699357063</v>
+        <v>0.708968055637063</v>
       </c>
       <c r="C16" s="16" t="n">
         <f aca="false">'Сценарій B'!$B$66</f>
-        <v>0.581127153251922</v>
+        <v>0.71800107713885</v>
       </c>
       <c r="D16" s="17" t="n">
         <f aca="false">C16-B16</f>
-        <v>0.0403604538948583</v>
+        <v>0.00903302150178664</v>
       </c>
       <c r="E16" s="2"/>
       <c r="F16" s="2"/>
@@ -1733,15 +1751,15 @@
       </c>
       <c r="B18" s="12" t="n">
         <f aca="false">'Сценарій A'!$B$61</f>
-        <v>-1743587.446636</v>
+        <v>-3032258.23416</v>
       </c>
       <c r="C18" s="12" t="n">
         <f aca="false">'Сценарій B'!$B$61</f>
-        <v>-1306544.150572</v>
+        <v>-1937861.87632</v>
       </c>
       <c r="D18" s="13" t="n">
         <f aca="false">C18-B18</f>
-        <v>437043.296064</v>
+        <v>1094396.35784</v>
       </c>
       <c r="E18" s="2"/>
       <c r="F18" s="2"/>
@@ -1798,23 +1816,23 @@
       </c>
       <c r="B23" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
-        <v>-2142479.32776</v>
+        <v>-3526705.4256</v>
       </c>
       <c r="C23" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
-        <v>-2540553.30896</v>
+        <v>-4033412.9976</v>
       </c>
       <c r="D23" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
-        <v>-2938627.29016</v>
+        <v>-4540120.5696</v>
       </c>
       <c r="E23" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
-        <v>-3336701.27136</v>
+        <v>-5046828.1416</v>
       </c>
       <c r="F23" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A23)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
-        <v>-3734775.25256</v>
+        <v>-5553535.7136</v>
       </c>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1823,23 +1841,23 @@
       </c>
       <c r="B24" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
-        <v>-1689981.82776</v>
+        <v>-3031502.9256</v>
       </c>
       <c r="C24" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
-        <v>-2088055.80896</v>
+        <v>-3538210.4976</v>
       </c>
       <c r="D24" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
-        <v>-2486129.79016</v>
+        <v>-4044918.0696</v>
       </c>
       <c r="E24" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
-        <v>-2884203.77136</v>
+        <v>-4551625.6416</v>
       </c>
       <c r="F24" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A24)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
-        <v>-3282277.75256</v>
+        <v>-5058333.2136</v>
       </c>
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1848,23 +1866,23 @@
       </c>
       <c r="B25" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
-        <v>-1237484.32776</v>
+        <v>-2536300.4256</v>
       </c>
       <c r="C25" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
-        <v>-1635558.30896</v>
+        <v>-3043007.9976</v>
       </c>
       <c r="D25" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
-        <v>-2033632.29016</v>
+        <v>-3549715.5696</v>
       </c>
       <c r="E25" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
-        <v>-2431706.27136</v>
+        <v>-4056423.1416</v>
       </c>
       <c r="F25" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A25)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
-        <v>-2829780.25256</v>
+        <v>-4563130.7136</v>
       </c>
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1873,23 +1891,23 @@
       </c>
       <c r="B26" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
-        <v>-784986.827760001</v>
+        <v>-2041097.9256</v>
       </c>
       <c r="C26" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
-        <v>-1183060.80896</v>
+        <v>-2547805.4976</v>
       </c>
       <c r="D26" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
-        <v>-1581134.79016</v>
+        <v>-3054513.0696</v>
       </c>
       <c r="E26" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
-        <v>-1979208.77136</v>
+        <v>-3561220.6416</v>
       </c>
       <c r="F26" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A26)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
-        <v>-2377282.75256</v>
+        <v>-4067928.2136</v>
       </c>
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1898,23 +1916,23 @@
       </c>
       <c r="B27" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+B$22)-'Сценарій A'!$B$65</f>
-        <v>-332489.327760001</v>
+        <v>-1545895.4256</v>
       </c>
       <c r="C27" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+C$22)-'Сценарій A'!$B$65</f>
-        <v>-730563.30896</v>
+        <v>-2052602.9976</v>
       </c>
       <c r="D27" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+D$22)-'Сценарій A'!$B$65</f>
-        <v>-1128637.29016</v>
+        <v>-2559310.5696</v>
       </c>
       <c r="E27" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+E$22)-'Сценарій A'!$B$65</f>
-        <v>-1526711.27136</v>
+        <v>-3066018.1416</v>
       </c>
       <c r="F27" s="10" t="n">
         <f aca="false">'Сценарій A'!$B$37*(1+$A27)*(1-Припущення!$B$34)-'Сценарій A'!$B$64*(1+F$22)-'Сценарій A'!$B$65</f>
-        <v>-1924785.25256</v>
+        <v>-3572725.7136</v>
       </c>
     </row>
     <row r="28" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1969,23 +1987,23 @@
       </c>
       <c r="B32" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
-        <v>-2683782.92776</v>
+        <v>-3965004.0256</v>
       </c>
       <c r="C32" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
-        <v>-3146659.40896</v>
+        <v>-4530074.0976</v>
       </c>
       <c r="D32" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
-        <v>-3609535.89016</v>
+        <v>-5095144.1696</v>
       </c>
       <c r="E32" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
-        <v>-4072412.37136</v>
+        <v>-5660214.2416</v>
       </c>
       <c r="F32" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A32)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
-        <v>-4535288.85256</v>
+        <v>-6225284.3136</v>
       </c>
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -1994,23 +2012,23 @@
       </c>
       <c r="B33" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
-        <v>-2177952.92776</v>
+        <v>-3417834.0256</v>
       </c>
       <c r="C33" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
-        <v>-2640829.40896</v>
+        <v>-3982904.0976</v>
       </c>
       <c r="D33" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
-        <v>-3103705.89016</v>
+        <v>-4547974.1696</v>
       </c>
       <c r="E33" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
-        <v>-3566582.37136</v>
+        <v>-5113044.2416</v>
       </c>
       <c r="F33" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A33)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
-        <v>-4029458.85256</v>
+        <v>-5678114.3136</v>
       </c>
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2019,23 +2037,23 @@
       </c>
       <c r="B34" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
-        <v>-1672122.92776</v>
+        <v>-2870664.0256</v>
       </c>
       <c r="C34" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
-        <v>-2134999.40896</v>
+        <v>-3435734.0976</v>
       </c>
       <c r="D34" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
-        <v>-2597875.89016</v>
+        <v>-4000804.1696</v>
       </c>
       <c r="E34" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
-        <v>-3060752.37136</v>
+        <v>-4565874.2416</v>
       </c>
       <c r="F34" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A34)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
-        <v>-3523628.85256</v>
+        <v>-5130944.3136</v>
       </c>
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2044,23 +2062,23 @@
       </c>
       <c r="B35" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
-        <v>-1166292.92776</v>
+        <v>-2323494.0256</v>
       </c>
       <c r="C35" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
-        <v>-1629169.40896</v>
+        <v>-2888564.0976</v>
       </c>
       <c r="D35" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
-        <v>-2092045.89016</v>
+        <v>-3453634.1696</v>
       </c>
       <c r="E35" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
-        <v>-2554922.37136</v>
+        <v>-4018704.2416</v>
       </c>
       <c r="F35" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A35)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
-        <v>-3017798.85256</v>
+        <v>-4583774.3136</v>
       </c>
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -2069,23 +2087,23 @@
       </c>
       <c r="B36" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+B$31)-'Сценарій B'!$B$65</f>
-        <v>-660462.92776</v>
+        <v>-1776324.0256</v>
       </c>
       <c r="C36" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+C$31)-'Сценарій B'!$B$65</f>
-        <v>-1123339.40896</v>
+        <v>-2341394.0976</v>
       </c>
       <c r="D36" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+D$31)-'Сценарій B'!$B$65</f>
-        <v>-1586215.89016</v>
+        <v>-2906464.1696</v>
       </c>
       <c r="E36" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+E$31)-'Сценарій B'!$B$65</f>
-        <v>-2049092.37136</v>
+        <v>-3471534.2416</v>
       </c>
       <c r="F36" s="10" t="n">
         <f aca="false">'Сценарій B'!$B$37*(1+$A36)*(1-Припущення!$B$34)-'Сценарій B'!$B$64*(1+F$31)-'Сценарій B'!$B$65</f>
-        <v>-2511968.85256</v>
+        <v>-4036604.3136</v>
       </c>
     </row>
   </sheetData>
@@ -2151,7 +2169,7 @@
       </c>
       <c r="B5" s="9" t="n">
         <f aca="false">'Сценарій A'!$B$37</f>
-        <v>9282000</v>
+        <v>10158000</v>
       </c>
       <c r="C5" s="2"/>
       <c r="D5" s="2"/>
@@ -2162,7 +2180,7 @@
       </c>
       <c r="B6" s="9" t="n">
         <f aca="false">'Сценарій A'!$B$56</f>
-        <v>-2033632.29016</v>
+        <v>-3549715.5696</v>
       </c>
       <c r="C6" s="2"/>
       <c r="D6" s="2"/>
@@ -2173,7 +2191,7 @@
       </c>
       <c r="B7" s="16" t="n">
         <f aca="false">'Сценарій A'!$B$57</f>
-        <v>-0.219094192001724</v>
+        <v>-0.349450243118724</v>
       </c>
       <c r="C7" s="2"/>
       <c r="D7" s="2"/>
@@ -2380,7 +2398,7 @@
       </c>
       <c r="B27" s="13" t="n">
         <f aca="false">'Сценарій A'!$B$64*$B$26</f>
-        <v>318459.18496</v>
+        <v>405366.0576</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -2454,7 +2472,7 @@
       </c>
       <c r="B35" s="13" t="n">
         <f aca="false">'Сценарій A'!$B$48*$B$34</f>
-        <v>58012.5</v>
+        <v>63487.5</v>
       </c>
       <c r="C35" s="2"/>
       <c r="D35" s="2"/>
@@ -2584,7 +2602,7 @@
       </c>
       <c r="B48" s="13" t="n">
         <f aca="false">$B$14+$B$23+$B$27+$B$31+$B$35</f>
-        <v>685869.399245714</v>
+        <v>778251.271885714</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -2595,7 +2613,7 @@
       </c>
       <c r="B49" s="13" t="n">
         <f aca="false">$B$6+$B$48</f>
-        <v>-1347762.89091429</v>
+        <v>-2771464.29771428</v>
       </c>
       <c r="C49" s="2"/>
       <c r="D49" s="2"/>
@@ -2606,7 +2624,7 @@
       </c>
       <c r="B50" s="10" t="n">
         <f aca="false">$B$5+$B$13+$B$22</f>
-        <v>10024857.1428571</v>
+        <v>10900857.1428571</v>
       </c>
       <c r="C50" s="2"/>
       <c r="D50" s="2"/>
@@ -2617,7 +2635,7 @@
       </c>
       <c r="B51" s="15" t="n">
         <f aca="false">IF($B$50&lt;&gt;0,$B$49/$B$50,0)</f>
-        <v>-0.134442104431841</v>
+        <v>-0.254242786727125</v>
       </c>
       <c r="C51" s="2"/>
       <c r="D51" s="2"/>
@@ -2628,7 +2646,7 @@
       </c>
       <c r="B52" s="13" t="n">
         <f aca="false">MAX(0,Припущення!$B$43*$B$50-$B$49)</f>
-        <v>3352734.31948571</v>
+        <v>4951635.72628571</v>
       </c>
       <c r="C52" s="2"/>
       <c r="D52" s="2"/>
@@ -2745,34 +2763,34 @@
         <v>89</v>
       </c>
       <c r="B5" s="29" t="n">
-        <v>61.5</v>
+        <v>92</v>
       </c>
       <c r="C5" s="30" t="n">
         <v>2</v>
       </c>
       <c r="D5" s="30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="E5" s="30" t="n">
         <v>1</v>
       </c>
       <c r="F5" s="30" t="n">
-        <v>61</v>
+        <v>70</v>
       </c>
       <c r="G5" s="5" t="str">
         <f aca="false">IF(B5&gt;=F5,"Так","НІ")</f>
         <v>Так</v>
       </c>
       <c r="H5" s="23" t="n">
-        <f aca="false">340000/B5</f>
-        <v>5528.45528455285</v>
+        <f aca="false">410000/B5</f>
+        <v>4456.52173913044</v>
       </c>
       <c r="I5" s="10" t="n">
         <f aca="false">B5*H5</f>
-        <v>340000</v>
+        <v>410000</v>
       </c>
       <c r="J5" s="28" t="n">
-        <v>340</v>
+        <v>350</v>
       </c>
       <c r="K5" s="5" t="s">
         <v>90</v>
@@ -2783,34 +2801,34 @@
         <v>91</v>
       </c>
       <c r="B6" s="29" t="n">
-        <v>71</v>
+        <v>128</v>
       </c>
       <c r="C6" s="30" t="n">
+        <v>3</v>
+      </c>
+      <c r="D6" s="30" t="n">
+        <v>6</v>
+      </c>
+      <c r="E6" s="30" t="n">
         <v>2</v>
       </c>
-      <c r="D6" s="30" t="n">
-        <v>4</v>
-      </c>
-      <c r="E6" s="30" t="n">
-        <v>1</v>
-      </c>
       <c r="F6" s="30" t="n">
-        <v>70</v>
+        <v>102</v>
       </c>
       <c r="G6" s="5" t="str">
         <f aca="false">IF(B6&gt;=F6,"Так","НІ")</f>
         <v>Так</v>
       </c>
       <c r="H6" s="23" t="n">
-        <f aca="false">390000/B6</f>
-        <v>5492.95774647887</v>
+        <f aca="false">460000/B6</f>
+        <v>3593.75</v>
       </c>
       <c r="I6" s="10" t="n">
         <f aca="false">B6*H6</f>
-        <v>390000</v>
+        <v>460000</v>
       </c>
       <c r="J6" s="28" t="n">
-        <v>370</v>
+        <v>300</v>
       </c>
       <c r="K6" s="5" t="s">
         <v>92</v>
@@ -2821,34 +2839,34 @@
         <v>93</v>
       </c>
       <c r="B7" s="29" t="n">
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="C7" s="30" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="D7" s="30" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="E7" s="30" t="n">
         <v>1</v>
       </c>
       <c r="F7" s="30" t="n">
-        <v>95</v>
+        <v>117</v>
       </c>
       <c r="G7" s="5" t="str">
         <f aca="false">IF(B7&gt;=F7,"Так","НІ")</f>
         <v>Так</v>
       </c>
       <c r="H7" s="23" t="n">
-        <f aca="false">550000/B7</f>
-        <v>3928.57142857143</v>
+        <f aca="false">700000/B7</f>
+        <v>4117.64705882353</v>
       </c>
       <c r="I7" s="10" t="n">
         <f aca="false">B7*H7</f>
-        <v>550000</v>
+        <v>700000</v>
       </c>
       <c r="J7" s="28" t="n">
-        <v>560</v>
+        <v>900</v>
       </c>
       <c r="K7" s="5" t="s">
         <v>94</v>
@@ -3140,7 +3158,7 @@
       </c>
       <c r="B24" s="31" t="n">
         <f aca="false">'Собівартість будинку'!$E$27</f>
-        <v>2783.18187702265</v>
+        <v>2848.99698492462</v>
       </c>
       <c r="C24" s="5" t="s">
         <v>121</v>
@@ -3181,8 +3199,8 @@
       <c r="A26" s="5" t="s">
         <v>125</v>
       </c>
-      <c r="B26" s="27" t="n">
-        <v>0.15</v>
+      <c r="B26" s="26" t="n">
+        <v>35000</v>
       </c>
       <c r="C26" s="5" t="s">
         <v>126</v>
@@ -3752,10 +3770,10 @@
         <v>91</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>93</v>
+        <v>179</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>179</v>
+        <v>180</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -3765,40 +3783,40 @@
       <c r="B5" s="2"/>
       <c r="C5" s="32" t="n">
         <f aca="false">Припущення!$B$5</f>
-        <v>61.5</v>
+        <v>92</v>
       </c>
       <c r="D5" s="32" t="n">
         <f aca="false">Припущення!$B$6</f>
-        <v>71</v>
+        <v>128</v>
       </c>
       <c r="E5" s="32" t="n">
         <f aca="false">Припущення!$B$7</f>
-        <v>140</v>
+        <v>170</v>
       </c>
       <c r="F5" s="2"/>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="2" t="s">
-        <v>180</v>
+        <v>181</v>
       </c>
       <c r="B6" s="2"/>
       <c r="C6" s="6" t="n">
         <f aca="false">'Сценарій A'!$B$5</f>
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="D6" s="6" t="n">
         <f aca="false">'Сценарій A'!$B$6</f>
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="E6" s="6" t="n">
         <f aca="false">'Сценарій A'!$B$7</f>
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="F6" s="2"/>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="21" t="s">
-        <v>181</v>
+        <v>182</v>
       </c>
       <c r="B7" s="22"/>
       <c r="C7" s="22"/>
@@ -3808,102 +3826,99 @@
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="5" t="s">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="B8" s="26" t="n">
         <v>1700</v>
       </c>
       <c r="C8" s="33" t="n">
         <f aca="false">$B8*C$5</f>
-        <v>104550</v>
+        <v>156400</v>
       </c>
       <c r="D8" s="33" t="n">
         <f aca="false">$B8*D$5</f>
-        <v>120700</v>
+        <v>217600</v>
       </c>
       <c r="E8" s="33" t="n">
         <f aca="false">$B8*E$5</f>
-        <v>238000</v>
+        <v>289000</v>
       </c>
       <c r="F8" s="24" t="s">
-        <v>183</v>
+        <v>184</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A9" s="5" t="s">
-        <v>184</v>
-      </c>
-      <c r="B9" s="26" t="n">
-        <v>160</v>
-      </c>
-      <c r="C9" s="33" t="n">
-        <f aca="false">$B9*C$5</f>
-        <v>9840</v>
-      </c>
-      <c r="D9" s="33" t="n">
-        <f aca="false">$B9*D$5</f>
-        <v>11360</v>
-      </c>
-      <c r="E9" s="33" t="n">
-        <f aca="false">$B9*E$5</f>
-        <v>22400</v>
+        <v>185</v>
+      </c>
+      <c r="B9" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C9" s="26" t="n">
+        <v>17900</v>
+      </c>
+      <c r="D9" s="26" t="n">
+        <v>12400</v>
+      </c>
+      <c r="E9" s="26" t="n">
+        <v>49400</v>
       </c>
       <c r="F9" s="24" t="s">
-        <v>185</v>
+        <v>187</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="5" t="s">
-        <v>186</v>
+        <v>188</v>
       </c>
       <c r="B10" s="26" t="n">
         <v>120</v>
       </c>
       <c r="C10" s="33" t="n">
         <f aca="false">$B10*C$5</f>
-        <v>7380</v>
+        <v>11040</v>
       </c>
       <c r="D10" s="33" t="n">
         <f aca="false">$B10*D$5</f>
-        <v>8520</v>
+        <v>15360</v>
       </c>
       <c r="E10" s="33" t="n">
         <f aca="false">$B10*E$5</f>
-        <v>16800</v>
+        <v>20400</v>
       </c>
       <c r="F10" s="24" t="s">
-        <v>187</v>
+        <v>189</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>188</v>
+        <v>190</v>
       </c>
       <c r="B11" s="26" t="n">
         <v>60</v>
       </c>
       <c r="C11" s="33" t="n">
         <f aca="false">$B11*C$5</f>
-        <v>3690</v>
+        <v>5520</v>
       </c>
       <c r="D11" s="33" t="n">
         <f aca="false">$B11*D$5</f>
-        <v>4260</v>
+        <v>7680</v>
       </c>
       <c r="E11" s="33" t="n">
         <f aca="false">$B11*E$5</f>
-        <v>8400</v>
+        <v>10200</v>
       </c>
       <c r="F11" s="24" t="s">
-        <v>189</v>
+        <v>191</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>190</v>
+        <v>192</v>
       </c>
       <c r="B12" s="5" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C12" s="26" t="n">
         <v>6500</v>
@@ -3912,206 +3927,230 @@
         <v>6500</v>
       </c>
       <c r="E12" s="26" t="n">
-        <v>8500</v>
+        <v>9000</v>
       </c>
       <c r="F12" s="24" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="B13" s="5" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C13" s="26" t="n">
         <v>2000</v>
       </c>
       <c r="D13" s="26" t="n">
-        <v>2000</v>
+        <v>3000</v>
       </c>
       <c r="E13" s="26" t="n">
-        <v>3500</v>
+        <v>4500</v>
       </c>
       <c r="F13" s="24" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
       <c r="B14" s="5" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C14" s="26" t="n">
-        <v>9000</v>
+        <v>10000</v>
       </c>
       <c r="D14" s="26" t="n">
-        <v>10000</v>
+        <v>11000</v>
       </c>
       <c r="E14" s="26" t="n">
-        <v>15000</v>
+        <v>18000</v>
       </c>
       <c r="F14" s="24" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="B15" s="5" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C15" s="26" t="n">
-        <v>6000</v>
+        <v>12000</v>
       </c>
       <c r="D15" s="26" t="n">
-        <v>6000</v>
+        <v>18000</v>
       </c>
       <c r="E15" s="26" t="n">
-        <v>12000</v>
+        <v>14000</v>
       </c>
       <c r="F15" s="24" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
     </row>
     <row r="16" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A16" s="5" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="B16" s="5" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C16" s="26" t="n">
-        <v>3500</v>
+        <v>0</v>
       </c>
       <c r="D16" s="26" t="n">
-        <v>3500</v>
+        <v>5000</v>
       </c>
       <c r="E16" s="26" t="n">
-        <v>3500</v>
+        <v>0</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="5" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="B17" s="5" t="s">
-        <v>191</v>
+        <v>186</v>
       </c>
       <c r="C17" s="26" t="n">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="D17" s="26" t="n">
-        <v>6000</v>
+        <v>0</v>
       </c>
       <c r="E17" s="26" t="n">
-        <v>9000</v>
+        <v>63900</v>
       </c>
       <c r="F17" s="24" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A18" s="11" t="s">
-        <v>203</v>
-      </c>
-      <c r="B18" s="2"/>
-      <c r="C18" s="13" t="n">
-        <f aca="false">SUM(C8:C17)</f>
-        <v>158460</v>
-      </c>
-      <c r="D18" s="13" t="n">
-        <f aca="false">SUM(D8:D17)</f>
-        <v>178840</v>
-      </c>
-      <c r="E18" s="13" t="n">
-        <f aca="false">SUM(E8:E17)</f>
-        <v>337100</v>
-      </c>
-      <c r="F18" s="2"/>
+      <c r="A18" s="5" t="s">
+        <v>204</v>
+      </c>
+      <c r="B18" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C18" s="26" t="n">
+        <v>3500</v>
+      </c>
+      <c r="D18" s="26" t="n">
+        <v>3500</v>
+      </c>
+      <c r="E18" s="26" t="n">
+        <v>3500</v>
+      </c>
+      <c r="F18" s="24" t="s">
+        <v>205</v>
+      </c>
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>204</v>
-      </c>
-      <c r="B19" s="27" t="n">
-        <v>0.12</v>
-      </c>
-      <c r="C19" s="33" t="n">
-        <f aca="false">C18*$B19</f>
-        <v>19015.2</v>
-      </c>
-      <c r="D19" s="33" t="n">
-        <f aca="false">D18*$B19</f>
-        <v>21460.8</v>
-      </c>
-      <c r="E19" s="33" t="n">
-        <f aca="false">E18*$B19</f>
-        <v>40452</v>
+        <v>206</v>
+      </c>
+      <c r="B19" s="5" t="s">
+        <v>186</v>
+      </c>
+      <c r="C19" s="26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="D19" s="26" t="n">
+        <v>6000</v>
+      </c>
+      <c r="E19" s="26" t="n">
+        <v>12000</v>
       </c>
       <c r="F19" s="24" t="s">
-        <v>205</v>
+        <v>207</v>
       </c>
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="11" t="s">
-        <v>206</v>
+        <v>208</v>
       </c>
       <c r="B20" s="2"/>
       <c r="C20" s="13" t="n">
-        <f aca="false">C18+C19</f>
-        <v>177475.2</v>
+        <f aca="false">SUM(C8:C19)</f>
+        <v>230860</v>
       </c>
       <c r="D20" s="13" t="n">
-        <f aca="false">D18+D19</f>
-        <v>200300.8</v>
+        <f aca="false">SUM(D8:D19)</f>
+        <v>306040</v>
       </c>
       <c r="E20" s="13" t="n">
-        <f aca="false">E18+E19</f>
-        <v>377552</v>
+        <f aca="false">SUM(E8:E19)</f>
+        <v>493900</v>
       </c>
       <c r="F20" s="2"/>
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A21" s="11" t="s">
-        <v>207</v>
-      </c>
-      <c r="B21" s="2"/>
-      <c r="C21" s="13" t="n">
-        <f aca="false">IF(C5&gt;0,C20/C5,0)</f>
-        <v>2885.7756097561</v>
-      </c>
-      <c r="D21" s="13" t="n">
-        <f aca="false">IF(D5&gt;0,D20/D5,0)</f>
-        <v>2821.13802816901</v>
-      </c>
-      <c r="E21" s="13" t="n">
-        <f aca="false">IF(E5&gt;0,E20/E5,0)</f>
-        <v>2696.8</v>
-      </c>
-      <c r="F21" s="2"/>
+      <c r="A21" s="5" t="s">
+        <v>209</v>
+      </c>
+      <c r="B21" s="27" t="n">
+        <v>0.12</v>
+      </c>
+      <c r="C21" s="33" t="n">
+        <f aca="false">C20*$B21</f>
+        <v>27703.2</v>
+      </c>
+      <c r="D21" s="33" t="n">
+        <f aca="false">D20*$B21</f>
+        <v>36724.8</v>
+      </c>
+      <c r="E21" s="33" t="n">
+        <f aca="false">E20*$B21</f>
+        <v>59268</v>
+      </c>
+      <c r="F21" s="24" t="s">
+        <v>210</v>
+      </c>
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A22" s="2"/>
+      <c r="A22" s="11" t="s">
+        <v>211</v>
+      </c>
       <c r="B22" s="2"/>
-      <c r="C22" s="2"/>
-      <c r="D22" s="2"/>
-      <c r="E22" s="2"/>
+      <c r="C22" s="13" t="n">
+        <f aca="false">C20+C21</f>
+        <v>258563.2</v>
+      </c>
+      <c r="D22" s="13" t="n">
+        <f aca="false">D20+D21</f>
+        <v>342764.8</v>
+      </c>
+      <c r="E22" s="13" t="n">
+        <f aca="false">E20+E21</f>
+        <v>553168</v>
+      </c>
       <c r="F22" s="2"/>
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A23" s="2"/>
+      <c r="A23" s="11" t="s">
+        <v>212</v>
+      </c>
       <c r="B23" s="2"/>
-      <c r="C23" s="2"/>
-      <c r="D23" s="2"/>
-      <c r="E23" s="2"/>
+      <c r="C23" s="13" t="n">
+        <f aca="false">IF(C5&gt;0,C22/C5,0)</f>
+        <v>2810.46956521739</v>
+      </c>
+      <c r="D23" s="13" t="n">
+        <f aca="false">IF(D5&gt;0,D22/D5,0)</f>
+        <v>2677.85</v>
+      </c>
+      <c r="E23" s="13" t="n">
+        <f aca="false">IF(E5&gt;0,E22/E5,0)</f>
+        <v>3253.92941176471</v>
+      </c>
       <c r="F23" s="2"/>
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4140,20 +4179,20 @@
     </row>
     <row r="27" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A27" s="11" t="s">
-        <v>208</v>
+        <v>213</v>
       </c>
       <c r="B27" s="2"/>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
       <c r="E27" s="34" t="n">
-        <f aca="false">SUMPRODUCT(C20:E20,C6:E6)/SUMPRODUCT(C5:E5,C6:E6)</f>
-        <v>2783.18187702265</v>
+        <f aca="false">SUMPRODUCT(C22:E22,C6:E6)/SUMPRODUCT(C5:E5,C6:E6)</f>
+        <v>2848.99698492462</v>
       </c>
       <c r="F27" s="2"/>
     </row>
     <row r="28" customFormat="false" ht="30" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A28" s="20" t="s">
-        <v>209</v>
+        <v>214</v>
       </c>
       <c r="B28" s="20"/>
       <c r="C28" s="20"/>
@@ -4190,7 +4229,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>210</v>
+        <v>215</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -4200,7 +4239,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>211</v>
+        <v>216</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -4221,99 +4260,99 @@
         <v>78</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>86</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="35" t="str">
         <f aca="false">Припущення!$A$5</f>
-        <v>Lake House Compact 61</v>
+        <v>Lake House Standard 92</v>
       </c>
       <c r="B5" s="28" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C5" s="36" t="n">
         <f aca="false">B5*Припущення!$B$5</f>
-        <v>615</v>
+        <v>1380</v>
       </c>
       <c r="D5" s="9" t="n">
         <f aca="false">Припущення!$I$5</f>
-        <v>340000</v>
+        <v>410000</v>
       </c>
       <c r="E5" s="10" t="n">
         <f aca="false">B5*D5</f>
-        <v>3400000</v>
+        <v>6150000</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">B5*Припущення!$J$5</f>
-        <v>3400</v>
+        <v>5250</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="35" t="str">
         <f aca="false">Припущення!$A$6</f>
-        <v>Meadow 71</v>
+        <v>Metropolis 128</v>
       </c>
       <c r="B6" s="28" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" s="36" t="n">
         <f aca="false">B6*Припущення!$B$6</f>
-        <v>568</v>
+        <v>896</v>
       </c>
       <c r="D6" s="9" t="n">
         <f aca="false">Припущення!$I$6</f>
-        <v>390000</v>
+        <v>460000</v>
       </c>
       <c r="E6" s="10" t="n">
         <f aca="false">B6*D6</f>
-        <v>3120000</v>
+        <v>3220000</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">B6*Припущення!$J$6</f>
-        <v>2960</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="35" t="str">
         <f aca="false">Припущення!$A$7</f>
-        <v>Country 140</v>
+        <v>Halcyon Estate 170</v>
       </c>
       <c r="B7" s="28" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C7" s="36" t="n">
         <f aca="false">B7*Припущення!$B$7</f>
-        <v>980</v>
+        <v>510</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">Припущення!$I$7</f>
-        <v>550000</v>
+        <v>700000</v>
       </c>
       <c r="E7" s="10" t="n">
         <f aca="false">B7*D7</f>
-        <v>3850000</v>
+        <v>2100000</v>
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">B7*Припущення!$J$7</f>
-        <v>3920</v>
+        <v>2700</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="B8" s="37" t="n">
         <f aca="false">SUM(B5:B7)</f>
@@ -4321,16 +4360,16 @@
       </c>
       <c r="C8" s="38" t="n">
         <f aca="false">SUM(C5:C7)</f>
-        <v>2163</v>
+        <v>2786</v>
       </c>
       <c r="D8" s="33"/>
       <c r="E8" s="13" t="n">
         <f aca="false">SUM(E5:E7)</f>
-        <v>10370000</v>
+        <v>11470000</v>
       </c>
       <c r="F8" s="37" t="n">
         <f aca="false">SUM(F5:F7)</f>
-        <v>10280</v>
+        <v>10050</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -4343,7 +4382,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -4353,7 +4392,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="B11" s="28" t="n">
         <v>0</v>
@@ -4365,13 +4404,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B12" s="25" t="n">
         <v>0.85</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -4379,13 +4418,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B13" s="28" t="n">
         <v>0</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -4393,13 +4432,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="B14" s="26" t="n">
         <v>100000</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -4407,14 +4446,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B15" s="7" t="n">
         <f aca="false">B8+$B$11*Припущення!$B$50</f>
         <v>25</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
@@ -4430,7 +4469,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="B17" s="22"/>
       <c r="C17" s="22"/>
@@ -4440,11 +4479,11 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B18" s="7" t="n">
         <f aca="false">F8</f>
-        <v>10280</v>
+        <v>10050</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -4453,7 +4492,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="B19" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$13</f>
@@ -4466,7 +4505,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B20" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$14</f>
@@ -4479,7 +4518,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$15</f>
@@ -4492,7 +4531,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">$B$11*Припущення!$B$16</f>
@@ -4505,11 +4544,11 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="B23" s="37" t="n">
         <f aca="false">SUM($B$18:$B$22)</f>
-        <v>14695.95</v>
+        <v>14465.95</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -4518,7 +4557,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B24" s="6" t="n">
         <f aca="false">Припущення!$B$12</f>
@@ -4531,11 +4570,11 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B25" s="37" t="n">
         <f aca="false">$B$24-$B$23</f>
-        <v>-450.950000000001</v>
+        <v>-220.950000000001</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -4544,7 +4583,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B26" s="39" t="str">
         <f aca="false">IF($B$25&gt;=0,"Вміщується","НЕ ВМІЩУЄТЬСЯ")</f>
@@ -4561,7 +4600,7 @@
       </c>
       <c r="B27" s="7" t="n">
         <f aca="false">IF(B8&gt;0,F8/B8,0)</f>
-        <v>411.2</v>
+        <v>402</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -4578,7 +4617,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="B29" s="22"/>
       <c r="C29" s="22"/>
@@ -4588,11 +4627,11 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="B30" s="10" t="n">
         <f aca="false">E8</f>
-        <v>10370000</v>
+        <v>11470000</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -4601,14 +4640,14 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B31" s="7" t="n">
         <f aca="false">ROUNDUP($B$15*Припущення!$B$19,0)</f>
         <v>8</v>
       </c>
       <c r="C31" s="24" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
@@ -4616,7 +4655,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="B32" s="7" t="n">
         <f aca="false">MIN($B$31,INDEX(B5:B7,Припущення!$B$21))</f>
@@ -4629,7 +4668,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B33" s="40" t="str">
         <f aca="false">IF($B$32&lt;$B$31,"Обраного типу замало — потрібні інші типи","OK")</f>
@@ -4642,14 +4681,14 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="B34" s="10" t="n">
         <f aca="false">-$B$31*INDEX(D5:D7,Припущення!$B$21)*(1-Припущення!$B$20)</f>
-        <v>-1088000</v>
+        <v>-1312000</v>
       </c>
       <c r="C34" s="24" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
@@ -4657,7 +4696,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="B35" s="10" t="n">
         <f aca="false">$B$11*Припущення!$B$47*Припущення!$B$48/Припущення!$B$49</f>
@@ -4670,7 +4709,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B36" s="10" t="n">
         <f aca="false">$B$11*Припущення!$B$50*Припущення!$B$51</f>
@@ -4683,11 +4722,11 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="B37" s="13" t="n">
         <f aca="false">SUM($B$30,$B$34,$B$35,$B$36)</f>
-        <v>9282000</v>
+        <v>10158000</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -4704,7 +4743,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="21" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B39" s="22"/>
       <c r="C39" s="22"/>
@@ -4714,11 +4753,11 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="B40" s="10" t="n">
         <f aca="false">C8*Припущення!$B$24</f>
-        <v>6020022.4</v>
+        <v>7937305.6</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -4727,7 +4766,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B41" s="10" t="n">
         <f aca="false">$B$11*Припущення!$B$46*Припущення!$B$25</f>
@@ -4743,21 +4782,23 @@
         <v>125</v>
       </c>
       <c r="B42" s="10" t="n">
-        <f aca="false">($B$40+$B$41)*Припущення!$B$26</f>
-        <v>903003.36</v>
-      </c>
-      <c r="C42" s="2"/>
+        <f aca="false">B8*Припущення!$B$26+$B$11*Припущення!$B$26</f>
+        <v>875000</v>
+      </c>
+      <c r="C42" s="24" t="s">
+        <v>256</v>
+      </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="B43" s="10" t="n">
         <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$27</f>
-        <v>346151.288</v>
+        <v>440615.28</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -4770,7 +4811,7 @@
       </c>
       <c r="B44" s="10" t="n">
         <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$28</f>
-        <v>692302.576</v>
+        <v>881230.56</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
@@ -4779,7 +4820,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="B45" s="10" t="n">
         <f aca="false">$B$15*Припущення!$B$29</f>
@@ -4792,7 +4833,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="B46" s="10" t="n">
         <f aca="false">$B$15*Припущення!$B$30</f>
@@ -4805,7 +4846,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="B47" s="9" t="n">
         <f aca="false">Припущення!$B$31</f>
@@ -4822,7 +4863,7 @@
       </c>
       <c r="B48" s="10" t="n">
         <f aca="false">$B$37*Припущення!$B$34</f>
-        <v>232050</v>
+        <v>253950</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -4831,7 +4872,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="B49" s="10" t="n">
         <f aca="false">$B$15*Припущення!$B$35</f>
@@ -4844,7 +4885,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="B50" s="9" t="n">
         <f aca="false">Припущення!$B$41</f>
@@ -4870,14 +4911,14 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="B52" s="10" t="n">
         <f aca="false">Припущення!$B$36*(Припущення!$B$37*SUM($B$40:$B$49)*Припущення!$B$38/12+($B$50+$B$51)*(Припущення!$B$38+$B$13)/12)</f>
-        <v>1065602.66616</v>
+        <v>1263114.1296</v>
       </c>
       <c r="C52" s="24" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
@@ -4885,11 +4926,11 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="B53" s="13" t="n">
         <f aca="false">SUM($B$40:$B$52)</f>
-        <v>11315632.29016</v>
+        <v>13707715.5696</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
@@ -4906,7 +4947,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="21" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B55" s="22"/>
       <c r="C55" s="22"/>
@@ -4916,11 +4957,11 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B56" s="13" t="n">
         <f aca="false">$B$37-$B$53</f>
-        <v>-2033632.29016</v>
+        <v>-3549715.5696</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
@@ -4933,7 +4974,7 @@
       </c>
       <c r="B57" s="15" t="n">
         <f aca="false">IF($B$37&lt;&gt;0,$B$56/$B$37,0)</f>
-        <v>-0.219094192001724</v>
+        <v>-0.349450243118724</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
@@ -4942,11 +4983,11 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="B58" s="17" t="n">
         <f aca="false">IF($B$53&lt;&gt;0,$B$56/$B$53,0)</f>
-        <v>-0.179718838330266</v>
+        <v>-0.258957486502879</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
@@ -4955,7 +4996,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="B59" s="39" t="str">
         <f aca="false">IF($B$57&gt;=Припущення!$B$43,"Досягає цілі","НИЖЧЕ ЦІЛІ")</f>
@@ -4968,14 +5009,14 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="B60" s="10" t="n">
         <f aca="false">($B$37*(1-Припущення!$B$43)-($B$53-$B$50-$B$51-Припущення!$B$36*($B$50+$B$51)*(Припущення!$B$38+$B$13)/12))/(1+Припущення!$B$42+Припущення!$B$36*(1+Припущення!$B$42)*(Припущення!$B$38+$B$13)/12)</f>
-        <v>-1610035.40946594</v>
+        <v>-2962196.64982411</v>
       </c>
       <c r="C60" s="24" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
@@ -4983,11 +5024,11 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B61" s="13" t="n">
         <f aca="false">$B$12*$B$56-(1-$B$12)*$B$14</f>
-        <v>-1743587.446636</v>
+        <v>-3032258.23416</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
@@ -5004,7 +5045,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="21" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="B63" s="22"/>
       <c r="C63" s="22"/>
@@ -5014,11 +5055,11 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="B64" s="10" t="n">
         <f aca="false">SUM($B$40:$B$44)</f>
-        <v>7961479.624</v>
+        <v>10134151.44</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
@@ -5027,11 +5068,11 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="B65" s="10" t="n">
         <f aca="false">$B$53-$B$64-$B$48</f>
-        <v>3122102.66616</v>
+        <v>3319614.1296</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
@@ -5040,14 +5081,14 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="B66" s="17" t="n">
         <f aca="false">($B$64+$B$65)/($B$37*(1-Припущення!$B$34-Припущення!$B$43))-1</f>
-        <v>0.540766699357063</v>
+        <v>0.708968055637063</v>
       </c>
       <c r="C66" s="24" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>
@@ -5081,7 +5122,7 @@
   <sheetData>
     <row r="1" customFormat="false" ht="17.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A1" s="1" t="s">
-        <v>272</v>
+        <v>278</v>
       </c>
       <c r="B1" s="2"/>
       <c r="C1" s="2"/>
@@ -5091,7 +5132,7 @@
     </row>
     <row r="2" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A2" s="3" t="s">
-        <v>273</v>
+        <v>279</v>
       </c>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
@@ -5112,99 +5153,99 @@
         <v>78</v>
       </c>
       <c r="B4" s="4" t="s">
-        <v>212</v>
+        <v>217</v>
       </c>
       <c r="C4" s="4" t="s">
-        <v>213</v>
+        <v>218</v>
       </c>
       <c r="D4" s="4" t="s">
         <v>86</v>
       </c>
       <c r="E4" s="4" t="s">
-        <v>214</v>
+        <v>219</v>
       </c>
       <c r="F4" s="4" t="s">
-        <v>215</v>
+        <v>220</v>
       </c>
     </row>
     <row r="5" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A5" s="35" t="str">
         <f aca="false">Припущення!$A$5</f>
-        <v>Lake House Compact 61</v>
+        <v>Lake House Standard 92</v>
       </c>
       <c r="B5" s="28" t="n">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="C5" s="36" t="n">
         <f aca="false">B5*Припущення!$B$5</f>
-        <v>615</v>
+        <v>1380</v>
       </c>
       <c r="D5" s="9" t="n">
         <f aca="false">Припущення!$I$5</f>
-        <v>340000</v>
+        <v>410000</v>
       </c>
       <c r="E5" s="10" t="n">
         <f aca="false">B5*D5</f>
-        <v>3400000</v>
+        <v>6150000</v>
       </c>
       <c r="F5" s="7" t="n">
         <f aca="false">B5*Припущення!$J$5</f>
-        <v>3400</v>
+        <v>5250</v>
       </c>
     </row>
     <row r="6" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A6" s="35" t="str">
         <f aca="false">Припущення!$A$6</f>
-        <v>Meadow 71</v>
+        <v>Metropolis 128</v>
       </c>
       <c r="B6" s="28" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="C6" s="36" t="n">
         <f aca="false">B6*Припущення!$B$6</f>
-        <v>568</v>
+        <v>896</v>
       </c>
       <c r="D6" s="9" t="n">
         <f aca="false">Припущення!$I$6</f>
-        <v>390000</v>
+        <v>460000</v>
       </c>
       <c r="E6" s="10" t="n">
         <f aca="false">B6*D6</f>
-        <v>3120000</v>
+        <v>3220000</v>
       </c>
       <c r="F6" s="7" t="n">
         <f aca="false">B6*Припущення!$J$6</f>
-        <v>2960</v>
+        <v>2100</v>
       </c>
     </row>
     <row r="7" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A7" s="35" t="str">
         <f aca="false">Припущення!$A$7</f>
-        <v>Country 140</v>
+        <v>Halcyon Estate 170</v>
       </c>
       <c r="B7" s="28" t="n">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="C7" s="36" t="n">
         <f aca="false">B7*Припущення!$B$7</f>
-        <v>980</v>
+        <v>510</v>
       </c>
       <c r="D7" s="9" t="n">
         <f aca="false">Припущення!$I$7</f>
-        <v>550000</v>
+        <v>700000</v>
       </c>
       <c r="E7" s="10" t="n">
         <f aca="false">B7*D7</f>
-        <v>3850000</v>
+        <v>2100000</v>
       </c>
       <c r="F7" s="7" t="n">
         <f aca="false">B7*Припущення!$J$7</f>
-        <v>3920</v>
+        <v>2700</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A8" s="11" t="s">
-        <v>216</v>
+        <v>221</v>
       </c>
       <c r="B8" s="37" t="n">
         <f aca="false">SUM(B5:B7)</f>
@@ -5212,16 +5253,16 @@
       </c>
       <c r="C8" s="38" t="n">
         <f aca="false">SUM(C5:C7)</f>
-        <v>2163</v>
+        <v>2786</v>
       </c>
       <c r="D8" s="33"/>
       <c r="E8" s="13" t="n">
         <f aca="false">SUM(E5:E7)</f>
-        <v>10370000</v>
+        <v>11470000</v>
       </c>
       <c r="F8" s="37" t="n">
         <f aca="false">SUM(F5:F7)</f>
-        <v>10280</v>
+        <v>10050</v>
       </c>
     </row>
     <row r="9" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
@@ -5234,7 +5275,7 @@
     </row>
     <row r="10" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A10" s="21" t="s">
-        <v>217</v>
+        <v>222</v>
       </c>
       <c r="B10" s="22"/>
       <c r="C10" s="22"/>
@@ -5244,7 +5285,7 @@
     </row>
     <row r="11" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A11" s="5" t="s">
-        <v>218</v>
+        <v>223</v>
       </c>
       <c r="B11" s="28" t="n">
         <v>1</v>
@@ -5256,13 +5297,13 @@
     </row>
     <row r="12" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A12" s="5" t="s">
-        <v>219</v>
+        <v>224</v>
       </c>
       <c r="B12" s="25" t="n">
         <v>0.45</v>
       </c>
       <c r="C12" s="24" t="s">
-        <v>220</v>
+        <v>225</v>
       </c>
       <c r="D12" s="2"/>
       <c r="E12" s="2"/>
@@ -5270,13 +5311,13 @@
     </row>
     <row r="13" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A13" s="5" t="s">
-        <v>221</v>
+        <v>226</v>
       </c>
       <c r="B13" s="28" t="n">
         <v>12</v>
       </c>
       <c r="C13" s="24" t="s">
-        <v>222</v>
+        <v>227</v>
       </c>
       <c r="D13" s="2"/>
       <c r="E13" s="2"/>
@@ -5284,13 +5325,13 @@
     </row>
     <row r="14" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A14" s="5" t="s">
-        <v>223</v>
+        <v>228</v>
       </c>
       <c r="B14" s="26" t="n">
         <v>250000</v>
       </c>
       <c r="C14" s="24" t="s">
-        <v>224</v>
+        <v>229</v>
       </c>
       <c r="D14" s="2"/>
       <c r="E14" s="2"/>
@@ -5298,14 +5339,14 @@
     </row>
     <row r="15" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A15" s="5" t="s">
-        <v>225</v>
+        <v>230</v>
       </c>
       <c r="B15" s="7" t="n">
         <f aca="false">B8+$B$11*Припущення!$B$50</f>
         <v>29</v>
       </c>
       <c r="C15" s="24" t="s">
-        <v>226</v>
+        <v>231</v>
       </c>
       <c r="D15" s="2"/>
       <c r="E15" s="2"/>
@@ -5321,7 +5362,7 @@
     </row>
     <row r="17" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A17" s="21" t="s">
-        <v>227</v>
+        <v>232</v>
       </c>
       <c r="B17" s="22"/>
       <c r="C17" s="22"/>
@@ -5331,11 +5372,11 @@
     </row>
     <row r="18" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A18" s="5" t="s">
-        <v>228</v>
+        <v>233</v>
       </c>
       <c r="B18" s="7" t="n">
         <f aca="false">F8</f>
-        <v>10280</v>
+        <v>10050</v>
       </c>
       <c r="C18" s="2"/>
       <c r="D18" s="2"/>
@@ -5344,7 +5385,7 @@
     </row>
     <row r="19" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A19" s="5" t="s">
-        <v>229</v>
+        <v>234</v>
       </c>
       <c r="B19" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$13</f>
@@ -5357,7 +5398,7 @@
     </row>
     <row r="20" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A20" s="5" t="s">
-        <v>230</v>
+        <v>235</v>
       </c>
       <c r="B20" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$14</f>
@@ -5370,7 +5411,7 @@
     </row>
     <row r="21" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A21" s="5" t="s">
-        <v>231</v>
+        <v>236</v>
       </c>
       <c r="B21" s="6" t="n">
         <f aca="false">Припущення!$B$12*Припущення!$B$15</f>
@@ -5383,7 +5424,7 @@
     </row>
     <row r="22" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A22" s="5" t="s">
-        <v>232</v>
+        <v>237</v>
       </c>
       <c r="B22" s="7" t="n">
         <f aca="false">$B$11*Припущення!$B$16</f>
@@ -5396,11 +5437,11 @@
     </row>
     <row r="23" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A23" s="11" t="s">
-        <v>233</v>
+        <v>238</v>
       </c>
       <c r="B23" s="37" t="n">
         <f aca="false">SUM($B$18:$B$22)</f>
-        <v>15595.95</v>
+        <v>15365.95</v>
       </c>
       <c r="C23" s="2"/>
       <c r="D23" s="2"/>
@@ -5409,7 +5450,7 @@
     </row>
     <row r="24" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A24" s="5" t="s">
-        <v>234</v>
+        <v>239</v>
       </c>
       <c r="B24" s="6" t="n">
         <f aca="false">Припущення!$B$12</f>
@@ -5422,11 +5463,11 @@
     </row>
     <row r="25" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A25" s="11" t="s">
-        <v>235</v>
+        <v>240</v>
       </c>
       <c r="B25" s="37" t="n">
         <f aca="false">$B$24-$B$23</f>
-        <v>-1350.95</v>
+        <v>-1120.95</v>
       </c>
       <c r="C25" s="2"/>
       <c r="D25" s="2"/>
@@ -5435,7 +5476,7 @@
     </row>
     <row r="26" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A26" s="11" t="s">
-        <v>236</v>
+        <v>241</v>
       </c>
       <c r="B26" s="39" t="str">
         <f aca="false">IF($B$25&gt;=0,"Вміщується","НЕ ВМІЩУЄТЬСЯ")</f>
@@ -5452,7 +5493,7 @@
       </c>
       <c r="B27" s="7" t="n">
         <f aca="false">IF(B8&gt;0,F8/B8,0)</f>
-        <v>411.2</v>
+        <v>402</v>
       </c>
       <c r="C27" s="2"/>
       <c r="D27" s="2"/>
@@ -5469,7 +5510,7 @@
     </row>
     <row r="29" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A29" s="21" t="s">
-        <v>237</v>
+        <v>242</v>
       </c>
       <c r="B29" s="22"/>
       <c r="C29" s="22"/>
@@ -5479,11 +5520,11 @@
     </row>
     <row r="30" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A30" s="5" t="s">
-        <v>238</v>
+        <v>243</v>
       </c>
       <c r="B30" s="10" t="n">
         <f aca="false">E8</f>
-        <v>10370000</v>
+        <v>11470000</v>
       </c>
       <c r="C30" s="2"/>
       <c r="D30" s="2"/>
@@ -5492,14 +5533,14 @@
     </row>
     <row r="31" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A31" s="5" t="s">
-        <v>239</v>
+        <v>244</v>
       </c>
       <c r="B31" s="7" t="n">
         <f aca="false">ROUNDUP($B$15*Припущення!$B$19,0)</f>
         <v>9</v>
       </c>
       <c r="C31" s="24" t="s">
-        <v>240</v>
+        <v>245</v>
       </c>
       <c r="D31" s="2"/>
       <c r="E31" s="2"/>
@@ -5507,7 +5548,7 @@
     </row>
     <row r="32" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A32" s="5" t="s">
-        <v>241</v>
+        <v>246</v>
       </c>
       <c r="B32" s="7" t="n">
         <f aca="false">MIN($B$31,INDEX(B5:B7,Припущення!$B$21))</f>
@@ -5520,7 +5561,7 @@
     </row>
     <row r="33" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A33" s="5" t="s">
-        <v>242</v>
+        <v>247</v>
       </c>
       <c r="B33" s="40" t="str">
         <f aca="false">IF($B$32&lt;$B$31,"Обраного типу замало — потрібні інші типи","OK")</f>
@@ -5533,14 +5574,14 @@
     </row>
     <row r="34" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A34" s="5" t="s">
-        <v>243</v>
+        <v>248</v>
       </c>
       <c r="B34" s="10" t="n">
         <f aca="false">-$B$31*INDEX(D5:D7,Припущення!$B$21)*(1-Припущення!$B$20)</f>
-        <v>-1224000</v>
+        <v>-1476000</v>
       </c>
       <c r="C34" s="24" t="s">
-        <v>244</v>
+        <v>249</v>
       </c>
       <c r="D34" s="2"/>
       <c r="E34" s="2"/>
@@ -5548,7 +5589,7 @@
     </row>
     <row r="35" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A35" s="5" t="s">
-        <v>245</v>
+        <v>250</v>
       </c>
       <c r="B35" s="10" t="n">
         <f aca="false">$B$11*Припущення!$B$47*Припущення!$B$48/Припущення!$B$49</f>
@@ -5561,7 +5602,7 @@
     </row>
     <row r="36" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A36" s="5" t="s">
-        <v>246</v>
+        <v>251</v>
       </c>
       <c r="B36" s="10" t="n">
         <f aca="false">$B$11*Припущення!$B$50*Припущення!$B$51</f>
@@ -5574,11 +5615,11 @@
     </row>
     <row r="37" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A37" s="11" t="s">
-        <v>247</v>
+        <v>252</v>
       </c>
       <c r="B37" s="13" t="n">
         <f aca="false">SUM($B$30,$B$34,$B$35,$B$36)</f>
-        <v>10376000</v>
+        <v>11224000</v>
       </c>
       <c r="C37" s="2"/>
       <c r="D37" s="2"/>
@@ -5595,7 +5636,7 @@
     </row>
     <row r="39" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A39" s="21" t="s">
-        <v>248</v>
+        <v>253</v>
       </c>
       <c r="B39" s="22"/>
       <c r="C39" s="22"/>
@@ -5605,11 +5646,11 @@
     </row>
     <row r="40" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A40" s="5" t="s">
-        <v>249</v>
+        <v>254</v>
       </c>
       <c r="B40" s="10" t="n">
         <f aca="false">C8*Припущення!$B$24</f>
-        <v>6020022.4</v>
+        <v>7937305.6</v>
       </c>
       <c r="C40" s="2"/>
       <c r="D40" s="2"/>
@@ -5618,7 +5659,7 @@
     </row>
     <row r="41" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A41" s="5" t="s">
-        <v>250</v>
+        <v>255</v>
       </c>
       <c r="B41" s="10" t="n">
         <f aca="false">$B$11*Припущення!$B$46*Припущення!$B$25</f>
@@ -5634,21 +5675,23 @@
         <v>125</v>
       </c>
       <c r="B42" s="10" t="n">
-        <f aca="false">($B$40+$B$41)*Припущення!$B$26</f>
-        <v>1050003.36</v>
-      </c>
-      <c r="C42" s="2"/>
+        <f aca="false">B8*Припущення!$B$26+$B$11*Припущення!$B$26</f>
+        <v>910000</v>
+      </c>
+      <c r="C42" s="24" t="s">
+        <v>256</v>
+      </c>
       <c r="D42" s="2"/>
       <c r="E42" s="2"/>
       <c r="F42" s="2"/>
     </row>
     <row r="43" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A43" s="5" t="s">
-        <v>251</v>
+        <v>257</v>
       </c>
       <c r="B43" s="10" t="n">
         <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$27</f>
-        <v>402501.288</v>
+        <v>491365.28</v>
       </c>
       <c r="C43" s="2"/>
       <c r="D43" s="2"/>
@@ -5661,7 +5704,7 @@
       </c>
       <c r="B44" s="10" t="n">
         <f aca="false">($B$40+$B$41+$B$42)*Припущення!$B$28</f>
-        <v>805002.576</v>
+        <v>982730.56</v>
       </c>
       <c r="C44" s="2"/>
       <c r="D44" s="2"/>
@@ -5670,7 +5713,7 @@
     </row>
     <row r="45" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A45" s="5" t="s">
-        <v>252</v>
+        <v>258</v>
       </c>
       <c r="B45" s="10" t="n">
         <f aca="false">$B$15*Припущення!$B$29</f>
@@ -5683,7 +5726,7 @@
     </row>
     <row r="46" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A46" s="5" t="s">
-        <v>253</v>
+        <v>259</v>
       </c>
       <c r="B46" s="10" t="n">
         <f aca="false">$B$15*Припущення!$B$30</f>
@@ -5696,7 +5739,7 @@
     </row>
     <row r="47" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A47" s="5" t="s">
-        <v>254</v>
+        <v>260</v>
       </c>
       <c r="B47" s="9" t="n">
         <f aca="false">Припущення!$B$31</f>
@@ -5713,7 +5756,7 @@
       </c>
       <c r="B48" s="10" t="n">
         <f aca="false">$B$37*Припущення!$B$34</f>
-        <v>259400</v>
+        <v>280600</v>
       </c>
       <c r="C48" s="2"/>
       <c r="D48" s="2"/>
@@ -5722,7 +5765,7 @@
     </row>
     <row r="49" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A49" s="5" t="s">
-        <v>255</v>
+        <v>261</v>
       </c>
       <c r="B49" s="10" t="n">
         <f aca="false">$B$15*Припущення!$B$35</f>
@@ -5735,7 +5778,7 @@
     </row>
     <row r="50" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A50" s="5" t="s">
-        <v>256</v>
+        <v>262</v>
       </c>
       <c r="B50" s="9" t="n">
         <f aca="false">Припущення!$B$41</f>
@@ -5761,14 +5804,14 @@
     </row>
     <row r="52" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A52" s="5" t="s">
-        <v>257</v>
+        <v>263</v>
       </c>
       <c r="B52" s="10" t="n">
         <f aca="false">Припущення!$B$36*(Припущення!$B$37*SUM($B$40:$B$49)*Припущення!$B$38/12+($B$50+$B$51)*(Припущення!$B$38+$B$13)/12)</f>
-        <v>1333806.26616</v>
+        <v>1519662.7296</v>
       </c>
       <c r="C52" s="24" t="s">
-        <v>258</v>
+        <v>264</v>
       </c>
       <c r="D52" s="2"/>
       <c r="E52" s="2"/>
@@ -5776,11 +5819,11 @@
     </row>
     <row r="53" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A53" s="11" t="s">
-        <v>259</v>
+        <v>265</v>
       </c>
       <c r="B53" s="13" t="n">
         <f aca="false">SUM($B$40:$B$52)</f>
-        <v>12973875.89016</v>
+        <v>15224804.1696</v>
       </c>
       <c r="C53" s="2"/>
       <c r="D53" s="2"/>
@@ -5797,7 +5840,7 @@
     </row>
     <row r="55" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A55" s="21" t="s">
-        <v>260</v>
+        <v>266</v>
       </c>
       <c r="B55" s="22"/>
       <c r="C55" s="22"/>
@@ -5807,11 +5850,11 @@
     </row>
     <row r="56" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A56" s="11" t="s">
-        <v>261</v>
+        <v>267</v>
       </c>
       <c r="B56" s="13" t="n">
         <f aca="false">$B$37-$B$53</f>
-        <v>-2597875.89016</v>
+        <v>-4000804.1696</v>
       </c>
       <c r="C56" s="2"/>
       <c r="D56" s="2"/>
@@ -5824,7 +5867,7 @@
       </c>
       <c r="B57" s="15" t="n">
         <f aca="false">IF($B$37&lt;&gt;0,$B$56/$B$37,0)</f>
-        <v>-0.250373543770239</v>
+        <v>-0.356450834782609</v>
       </c>
       <c r="C57" s="2"/>
       <c r="D57" s="2"/>
@@ -5833,11 +5876,11 @@
     </row>
     <row r="58" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A58" s="5" t="s">
-        <v>262</v>
+        <v>268</v>
       </c>
       <c r="B58" s="17" t="n">
         <f aca="false">IF($B$53&lt;&gt;0,$B$56/$B$53,0)</f>
-        <v>-0.200238996592402</v>
+        <v>-0.262781979001646</v>
       </c>
       <c r="C58" s="2"/>
       <c r="D58" s="2"/>
@@ -5846,7 +5889,7 @@
     </row>
     <row r="59" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A59" s="11" t="s">
-        <v>263</v>
+        <v>269</v>
       </c>
       <c r="B59" s="39" t="str">
         <f aca="false">IF($B$57&gt;=Припущення!$B$43,"Досягає цілі","НИЖЧЕ ЦІЛІ")</f>
@@ -5859,14 +5902,14 @@
     </row>
     <row r="60" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A60" s="5" t="s">
-        <v>264</v>
+        <v>270</v>
       </c>
       <c r="B60" s="10" t="n">
         <f aca="false">($B$37*(1-Припущення!$B$43)-($B$53-$B$50-$B$51-Припущення!$B$36*($B$50+$B$51)*(Припущення!$B$38+$B$13)/12))/(1+Припущення!$B$42+Припущення!$B$36*(1+Припущення!$B$42)*(Припущення!$B$38+$B$13)/12)</f>
-        <v>-1971308.78781756</v>
+        <v>-3139432.60258505</v>
       </c>
       <c r="C60" s="24" t="s">
-        <v>265</v>
+        <v>271</v>
       </c>
       <c r="D60" s="2"/>
       <c r="E60" s="2"/>
@@ -5874,11 +5917,11 @@
     </row>
     <row r="61" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A61" s="11" t="s">
-        <v>266</v>
+        <v>272</v>
       </c>
       <c r="B61" s="13" t="n">
         <f aca="false">$B$12*$B$56-(1-$B$12)*$B$14</f>
-        <v>-1306544.150572</v>
+        <v>-1937861.87632</v>
       </c>
       <c r="C61" s="2"/>
       <c r="D61" s="2"/>
@@ -5895,7 +5938,7 @@
     </row>
     <row r="63" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A63" s="21" t="s">
-        <v>267</v>
+        <v>273</v>
       </c>
       <c r="B63" s="22"/>
       <c r="C63" s="22"/>
@@ -5905,11 +5948,11 @@
     </row>
     <row r="64" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A64" s="5" t="s">
-        <v>268</v>
+        <v>274</v>
       </c>
       <c r="B64" s="10" t="n">
         <f aca="false">SUM($B$40:$B$44)</f>
-        <v>9257529.624</v>
+        <v>11301401.44</v>
       </c>
       <c r="C64" s="2"/>
       <c r="D64" s="2"/>
@@ -5918,11 +5961,11 @@
     </row>
     <row r="65" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A65" s="5" t="s">
-        <v>269</v>
+        <v>275</v>
       </c>
       <c r="B65" s="10" t="n">
         <f aca="false">$B$53-$B$64-$B$48</f>
-        <v>3456946.26616</v>
+        <v>3642802.7296</v>
       </c>
       <c r="C65" s="2"/>
       <c r="D65" s="2"/>
@@ -5931,14 +5974,14 @@
     </row>
     <row r="66" customFormat="false" ht="15" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
       <c r="A66" s="5" t="s">
-        <v>270</v>
+        <v>276</v>
       </c>
       <c r="B66" s="17" t="n">
         <f aca="false">($B$64+$B$65)/($B$37*(1-Припущення!$B$34-Припущення!$B$43))-1</f>
-        <v>0.581127153251922</v>
+        <v>0.71800107713885</v>
       </c>
       <c r="C66" s="24" t="s">
-        <v>271</v>
+        <v>277</v>
       </c>
       <c r="D66" s="2"/>
       <c r="E66" s="2"/>

</xml_diff>